<commit_message>
Actualización de formatos GFPI-F023
</commit_message>
<xml_diff>
--- a/Formatos/Visita 1 GFPI-F023.xlsx
+++ b/Formatos/Visita 1 GFPI-F023.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SEANT\OneDrive\Documents\Seto 2026\sena\Manual SENA Etapa Productiva\manual-aprendiz-sena\Formatos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/834af06e427efe68/Documents/Seto 2026/sena/Manual SENA Etapa Productiva/manual-aprendiz-sena/Formatos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD5881F2-7753-446A-8E5F-805A07B66FFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="13_ncr:1_{DD5881F2-7753-446A-8E5F-805A07B66FFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AABE3BCB-E6DC-438F-AF45-0DB4F9E7EE49}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BC3553EE-4E49-4F2A-B03E-CFAC4EB3009B}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="Análisis_y_Desarrollo_de_Software">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Formato Visita 1'!$A$1:$M$75</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Formato Visita 1'!$A$8:$M$82</definedName>
     <definedName name="LISTA_38362">#REF!</definedName>
     <definedName name="LISTA_38376">#REF!</definedName>
     <definedName name="LISTA_38392">#REF!</definedName>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="123">
   <si>
     <t>Información general</t>
   </si>
@@ -548,12 +548,36 @@
       <t>Se realiza por una única vez)</t>
     </r>
   </si>
+  <si>
+    <t>PROCESO</t>
+  </si>
+  <si>
+    <t>NOMBRE DEL FORMATO</t>
+  </si>
+  <si>
+    <t>CLASIFICACIÓN DE LA INFORMACIÓN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pública  </t>
+  </si>
+  <si>
+    <t>Pública Clasificada</t>
+  </si>
+  <si>
+    <t>Pública Reservada</t>
+  </si>
+  <si>
+    <t>Formato de Planeación, Seguimiento y Evaluación de Etapa Productiva</t>
+  </si>
+  <si>
+    <t>GESTIÓN DE FORMACIÓN PROFESIONAL INTEGRAL</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -656,8 +680,15 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -670,8 +701,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="45">
+  <borders count="50">
     <border>
       <left/>
       <right/>
@@ -1191,11 +1228,74 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="156">
+  <cellXfs count="178">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
@@ -1260,9 +1360,56 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1417,6 +1564,48 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1465,6 +1654,18 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="15" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1552,9 +1753,6 @@
       <alignment horizontal="justify" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1564,34 +1762,19 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -1921,6 +2104,27 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2255,7 +2459,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:XFC76"/>
+  <dimension ref="A1:XFC83"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="15" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.5703125" customWidth="1"/>
@@ -2269,1468 +2473,1571 @@
     <col min="16384" max="16384" width="7" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="72" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B1" s="24" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="26"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B2" s="33" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
+      <c r="K2" s="35"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B3" s="27" t="s">
+        <v>116</v>
+      </c>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="29"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B4" s="33" t="s">
+        <v>121</v>
+      </c>
+      <c r="C4" s="34"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="34"/>
+      <c r="G4" s="34"/>
+      <c r="H4" s="34"/>
+      <c r="I4" s="34"/>
+      <c r="J4" s="34"/>
+      <c r="K4" s="35"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B5" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="28"/>
+      <c r="K5" s="29"/>
+    </row>
+    <row r="6" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="30" t="s">
+        <v>118</v>
+      </c>
+      <c r="C6" s="31"/>
+      <c r="D6" s="22" t="b">
         <v>0</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-    </row>
-    <row r="2" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="121" t="s">
+      <c r="E6" s="32" t="s">
+        <v>119</v>
+      </c>
+      <c r="F6" s="31"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="22" t="b">
+        <v>0</v>
+      </c>
+      <c r="I6" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="J6" s="31"/>
+      <c r="K6" s="23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="98"/>
+      <c r="C8" s="98"/>
+      <c r="D8" s="98"/>
+      <c r="E8" s="98"/>
+      <c r="F8" s="98"/>
+      <c r="G8" s="98"/>
+      <c r="H8" s="98"/>
+      <c r="I8" s="98"/>
+      <c r="J8" s="98"/>
+      <c r="K8" s="98"/>
+      <c r="L8" s="98"/>
+      <c r="M8" s="98"/>
+    </row>
+    <row r="9" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="143" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="123"/>
-      <c r="C2" s="69" t="s">
+      <c r="B9" s="145"/>
+      <c r="C9" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="71"/>
-    </row>
-    <row r="3" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="121" t="s">
+      <c r="D9" s="95"/>
+      <c r="E9" s="95"/>
+      <c r="F9" s="95"/>
+      <c r="G9" s="95"/>
+      <c r="H9" s="95"/>
+      <c r="I9" s="95"/>
+      <c r="J9" s="95"/>
+      <c r="K9" s="95"/>
+      <c r="L9" s="95"/>
+      <c r="M9" s="96"/>
+    </row>
+    <row r="10" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="143" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="123"/>
-      <c r="C3" s="139" t="s">
+      <c r="B10" s="145"/>
+      <c r="C10" s="161" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="140"/>
-      <c r="E3" s="140"/>
-      <c r="F3" s="140"/>
-      <c r="G3" s="141"/>
-      <c r="H3" s="1" t="s">
+      <c r="D10" s="162"/>
+      <c r="E10" s="162"/>
+      <c r="F10" s="162"/>
+      <c r="G10" s="163"/>
+      <c r="H10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="32"/>
-      <c r="J3" s="33"/>
-      <c r="K3" s="33"/>
-      <c r="L3" s="33"/>
-      <c r="M3" s="34"/>
-    </row>
-    <row r="4" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="121" t="s">
+      <c r="I10" s="45"/>
+      <c r="J10" s="46"/>
+      <c r="K10" s="46"/>
+      <c r="L10" s="46"/>
+      <c r="M10" s="47"/>
+    </row>
+    <row r="11" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="143" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="123"/>
-      <c r="C4" s="151"/>
-      <c r="D4" s="152"/>
-      <c r="E4" s="152"/>
-      <c r="F4" s="152"/>
-      <c r="G4" s="152"/>
-      <c r="H4" s="153"/>
-      <c r="I4" s="29" t="s">
+      <c r="B11" s="145"/>
+      <c r="C11" s="173"/>
+      <c r="D11" s="174"/>
+      <c r="E11" s="174"/>
+      <c r="F11" s="174"/>
+      <c r="G11" s="174"/>
+      <c r="H11" s="175"/>
+      <c r="I11" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="30"/>
-      <c r="K4" s="77"/>
-      <c r="L4" s="78"/>
-      <c r="M4" s="79"/>
-    </row>
-    <row r="5" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="121" t="s">
+      <c r="J11" s="43"/>
+      <c r="K11" s="102"/>
+      <c r="L11" s="103"/>
+      <c r="M11" s="104"/>
+    </row>
+    <row r="12" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="143" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="123"/>
-      <c r="C5" s="2" t="s">
+      <c r="B12" s="145"/>
+      <c r="C12" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="69" t="s">
+      <c r="D12" s="94" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="71"/>
-      <c r="F5" s="154" t="s">
+      <c r="E12" s="96"/>
+      <c r="F12" s="176" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="155"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="154" t="s">
+      <c r="G12" s="177"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="176" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="155"/>
-      <c r="K5" s="80"/>
-      <c r="L5" s="81"/>
-      <c r="M5" s="82"/>
-    </row>
-    <row r="6" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="121" t="s">
+      <c r="J12" s="177"/>
+      <c r="K12" s="105"/>
+      <c r="L12" s="106"/>
+      <c r="M12" s="107"/>
+    </row>
+    <row r="13" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="143" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="123"/>
-      <c r="C6" s="144"/>
-      <c r="D6" s="145"/>
-      <c r="E6" s="145"/>
-      <c r="F6" s="146"/>
-      <c r="G6" s="144" t="s">
+      <c r="B13" s="145"/>
+      <c r="C13" s="166"/>
+      <c r="D13" s="167"/>
+      <c r="E13" s="167"/>
+      <c r="F13" s="168"/>
+      <c r="G13" s="166" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="145"/>
-      <c r="I6" s="146"/>
-      <c r="J6" s="77"/>
-      <c r="K6" s="78"/>
-      <c r="L6" s="78"/>
-      <c r="M6" s="79"/>
-    </row>
-    <row r="7" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="147" t="s">
+      <c r="H13" s="167"/>
+      <c r="I13" s="168"/>
+      <c r="J13" s="108"/>
+      <c r="K13" s="109"/>
+      <c r="L13" s="109"/>
+      <c r="M13" s="110"/>
+    </row>
+    <row r="14" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="169" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="121" t="s">
+      <c r="B14" s="143" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="122"/>
-      <c r="D7" s="123"/>
-      <c r="E7" s="74"/>
-      <c r="F7" s="75"/>
-      <c r="G7" s="75"/>
-      <c r="H7" s="75"/>
-      <c r="I7" s="75"/>
-      <c r="J7" s="75"/>
-      <c r="K7" s="75"/>
-      <c r="L7" s="75"/>
-      <c r="M7" s="76"/>
-    </row>
-    <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="131"/>
-      <c r="B8" s="148" t="s">
+      <c r="C14" s="144"/>
+      <c r="D14" s="145"/>
+      <c r="E14" s="99"/>
+      <c r="F14" s="100"/>
+      <c r="G14" s="100"/>
+      <c r="H14" s="100"/>
+      <c r="I14" s="100"/>
+      <c r="J14" s="100"/>
+      <c r="K14" s="100"/>
+      <c r="L14" s="100"/>
+      <c r="M14" s="101"/>
+    </row>
+    <row r="15" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="153"/>
+      <c r="B15" s="170" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="149"/>
-      <c r="D8" s="150"/>
-      <c r="E8" s="83"/>
-      <c r="F8" s="84"/>
-      <c r="G8" s="84"/>
-      <c r="H8" s="84"/>
-      <c r="I8" s="84"/>
-      <c r="J8" s="84"/>
-      <c r="K8" s="84"/>
-      <c r="L8" s="84"/>
-      <c r="M8" s="85"/>
-    </row>
-    <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="131"/>
-      <c r="B9" s="121" t="s">
+      <c r="C15" s="171"/>
+      <c r="D15" s="172"/>
+      <c r="E15" s="111"/>
+      <c r="F15" s="112"/>
+      <c r="G15" s="112"/>
+      <c r="H15" s="112"/>
+      <c r="I15" s="112"/>
+      <c r="J15" s="112"/>
+      <c r="K15" s="112"/>
+      <c r="L15" s="112"/>
+      <c r="M15" s="113"/>
+    </row>
+    <row r="16" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="153"/>
+      <c r="B16" s="143" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="122"/>
-      <c r="D9" s="123"/>
-      <c r="E9" s="74"/>
-      <c r="F9" s="75"/>
-      <c r="G9" s="75"/>
-      <c r="H9" s="75"/>
-      <c r="I9" s="75"/>
-      <c r="J9" s="75"/>
-      <c r="K9" s="75"/>
-      <c r="L9" s="75"/>
-      <c r="M9" s="76"/>
-    </row>
-    <row r="10" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="131"/>
-      <c r="B10" s="121" t="s">
+      <c r="C16" s="144"/>
+      <c r="D16" s="145"/>
+      <c r="E16" s="99"/>
+      <c r="F16" s="100"/>
+      <c r="G16" s="100"/>
+      <c r="H16" s="100"/>
+      <c r="I16" s="100"/>
+      <c r="J16" s="100"/>
+      <c r="K16" s="100"/>
+      <c r="L16" s="100"/>
+      <c r="M16" s="101"/>
+    </row>
+    <row r="17" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="153"/>
+      <c r="B17" s="143" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="122"/>
-      <c r="D10" s="123"/>
-      <c r="E10" s="74"/>
-      <c r="F10" s="75"/>
-      <c r="G10" s="75"/>
-      <c r="H10" s="75"/>
-      <c r="I10" s="75"/>
-      <c r="J10" s="75"/>
-      <c r="K10" s="75"/>
-      <c r="L10" s="75"/>
-      <c r="M10" s="76"/>
-    </row>
-    <row r="11" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="131"/>
-      <c r="B11" s="121" t="s">
+      <c r="C17" s="144"/>
+      <c r="D17" s="145"/>
+      <c r="E17" s="99"/>
+      <c r="F17" s="100"/>
+      <c r="G17" s="100"/>
+      <c r="H17" s="100"/>
+      <c r="I17" s="100"/>
+      <c r="J17" s="100"/>
+      <c r="K17" s="100"/>
+      <c r="L17" s="100"/>
+      <c r="M17" s="101"/>
+    </row>
+    <row r="18" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="153"/>
+      <c r="B18" s="143" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="122"/>
-      <c r="D11" s="123"/>
-      <c r="E11" s="74"/>
-      <c r="F11" s="75"/>
-      <c r="G11" s="75"/>
-      <c r="H11" s="75"/>
-      <c r="I11" s="75"/>
-      <c r="J11" s="75"/>
-      <c r="K11" s="75"/>
-      <c r="L11" s="75"/>
-      <c r="M11" s="76"/>
-    </row>
-    <row r="12" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="131"/>
-      <c r="B12" s="121" t="s">
+      <c r="C18" s="144"/>
+      <c r="D18" s="145"/>
+      <c r="E18" s="99"/>
+      <c r="F18" s="100"/>
+      <c r="G18" s="100"/>
+      <c r="H18" s="100"/>
+      <c r="I18" s="100"/>
+      <c r="J18" s="100"/>
+      <c r="K18" s="100"/>
+      <c r="L18" s="100"/>
+      <c r="M18" s="101"/>
+    </row>
+    <row r="19" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="153"/>
+      <c r="B19" s="143" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="122"/>
-      <c r="D12" s="123"/>
-      <c r="E12" s="74"/>
-      <c r="F12" s="75"/>
-      <c r="G12" s="75"/>
-      <c r="H12" s="75"/>
-      <c r="I12" s="75"/>
-      <c r="J12" s="75"/>
-      <c r="K12" s="75"/>
-      <c r="L12" s="75"/>
-      <c r="M12" s="76"/>
-    </row>
-    <row r="13" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="131"/>
-      <c r="B13" s="121" t="s">
+      <c r="C19" s="144"/>
+      <c r="D19" s="145"/>
+      <c r="E19" s="99"/>
+      <c r="F19" s="100"/>
+      <c r="G19" s="100"/>
+      <c r="H19" s="100"/>
+      <c r="I19" s="100"/>
+      <c r="J19" s="100"/>
+      <c r="K19" s="100"/>
+      <c r="L19" s="100"/>
+      <c r="M19" s="101"/>
+    </row>
+    <row r="20" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="153"/>
+      <c r="B20" s="143" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="122"/>
-      <c r="D13" s="123"/>
-      <c r="E13" s="124"/>
-      <c r="F13" s="125"/>
-      <c r="G13" s="125"/>
-      <c r="H13" s="125"/>
-      <c r="I13" s="125"/>
-      <c r="J13" s="125"/>
-      <c r="K13" s="125"/>
-      <c r="L13" s="125"/>
-      <c r="M13" s="126"/>
-    </row>
-    <row r="14" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="131"/>
-      <c r="B14" s="121" t="s">
+      <c r="C20" s="144"/>
+      <c r="D20" s="145"/>
+      <c r="E20" s="146"/>
+      <c r="F20" s="147"/>
+      <c r="G20" s="147"/>
+      <c r="H20" s="147"/>
+      <c r="I20" s="147"/>
+      <c r="J20" s="147"/>
+      <c r="K20" s="147"/>
+      <c r="L20" s="147"/>
+      <c r="M20" s="148"/>
+    </row>
+    <row r="21" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="153"/>
+      <c r="B21" s="143" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="122"/>
-      <c r="D14" s="123"/>
-      <c r="E14" s="124"/>
-      <c r="F14" s="125"/>
-      <c r="G14" s="125"/>
-      <c r="H14" s="125"/>
-      <c r="I14" s="125"/>
-      <c r="J14" s="125"/>
-      <c r="K14" s="125"/>
-      <c r="L14" s="125"/>
-      <c r="M14" s="126"/>
-    </row>
-    <row r="15" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="132"/>
-      <c r="B15" s="121" t="s">
+      <c r="C21" s="144"/>
+      <c r="D21" s="145"/>
+      <c r="E21" s="146"/>
+      <c r="F21" s="147"/>
+      <c r="G21" s="147"/>
+      <c r="H21" s="147"/>
+      <c r="I21" s="147"/>
+      <c r="J21" s="147"/>
+      <c r="K21" s="147"/>
+      <c r="L21" s="147"/>
+      <c r="M21" s="148"/>
+    </row>
+    <row r="22" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="154"/>
+      <c r="B22" s="143" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="122"/>
-      <c r="D15" s="123"/>
-      <c r="E15" s="124"/>
-      <c r="F15" s="125"/>
-      <c r="G15" s="125"/>
-      <c r="H15" s="125"/>
-      <c r="I15" s="125"/>
-      <c r="J15" s="125"/>
-      <c r="K15" s="125"/>
-      <c r="L15" s="125"/>
-      <c r="M15" s="126"/>
-    </row>
-    <row r="16" spans="1:13" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="130" t="s">
+      <c r="C22" s="144"/>
+      <c r="D22" s="145"/>
+      <c r="E22" s="146"/>
+      <c r="F22" s="147"/>
+      <c r="G22" s="147"/>
+      <c r="H22" s="147"/>
+      <c r="I22" s="147"/>
+      <c r="J22" s="147"/>
+      <c r="K22" s="147"/>
+      <c r="L22" s="147"/>
+      <c r="M22" s="148"/>
+    </row>
+    <row r="23" spans="1:13" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="152" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="121" t="s">
+      <c r="B23" s="143" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="122"/>
-      <c r="D16" s="123"/>
-      <c r="E16" s="133" t="s">
+      <c r="C23" s="144"/>
+      <c r="D23" s="145"/>
+      <c r="E23" s="155" t="s">
         <v>27</v>
       </c>
-      <c r="F16" s="134"/>
-      <c r="G16" s="134"/>
-      <c r="H16" s="134"/>
-      <c r="I16" s="134"/>
-      <c r="J16" s="134"/>
-      <c r="K16" s="134"/>
-      <c r="L16" s="134"/>
-      <c r="M16" s="135"/>
-    </row>
-    <row r="17" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="131"/>
-      <c r="B17" s="121" t="s">
+      <c r="F23" s="156"/>
+      <c r="G23" s="156"/>
+      <c r="H23" s="156"/>
+      <c r="I23" s="156"/>
+      <c r="J23" s="156"/>
+      <c r="K23" s="156"/>
+      <c r="L23" s="156"/>
+      <c r="M23" s="157"/>
+    </row>
+    <row r="24" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="153"/>
+      <c r="B24" s="143" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="122"/>
-      <c r="D17" s="123"/>
-      <c r="E17" s="136"/>
-      <c r="F17" s="137"/>
-      <c r="G17" s="137"/>
-      <c r="H17" s="137"/>
-      <c r="I17" s="137"/>
-      <c r="J17" s="137"/>
-      <c r="K17" s="137"/>
-      <c r="L17" s="137"/>
-      <c r="M17" s="138"/>
-    </row>
-    <row r="18" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="132"/>
-      <c r="B18" s="121" t="s">
+      <c r="C24" s="144"/>
+      <c r="D24" s="145"/>
+      <c r="E24" s="158"/>
+      <c r="F24" s="159"/>
+      <c r="G24" s="159"/>
+      <c r="H24" s="159"/>
+      <c r="I24" s="159"/>
+      <c r="J24" s="159"/>
+      <c r="K24" s="159"/>
+      <c r="L24" s="159"/>
+      <c r="M24" s="160"/>
+    </row>
+    <row r="25" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="154"/>
+      <c r="B25" s="143" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="122"/>
-      <c r="D18" s="123"/>
-      <c r="E18" s="133" t="s">
+      <c r="C25" s="144"/>
+      <c r="D25" s="145"/>
+      <c r="E25" s="155" t="s">
         <v>28</v>
       </c>
-      <c r="F18" s="134"/>
-      <c r="G18" s="134"/>
-      <c r="H18" s="134"/>
-      <c r="I18" s="134"/>
-      <c r="J18" s="134"/>
-      <c r="K18" s="134"/>
-      <c r="L18" s="134"/>
-      <c r="M18" s="135"/>
-    </row>
-    <row r="19" spans="1:13" ht="25.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
+      <c r="F25" s="156"/>
+      <c r="G25" s="156"/>
+      <c r="H25" s="156"/>
+      <c r="I25" s="156"/>
+      <c r="J25" s="156"/>
+      <c r="K25" s="156"/>
+      <c r="L25" s="156"/>
+      <c r="M25" s="157"/>
+    </row>
+    <row r="26" spans="1:13" ht="25.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="121" t="s">
+      <c r="B26" s="143" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="122"/>
-      <c r="D19" s="123"/>
-      <c r="E19" s="74"/>
-      <c r="F19" s="75"/>
-      <c r="G19" s="75"/>
-      <c r="H19" s="75"/>
-      <c r="I19" s="75"/>
-      <c r="J19" s="75"/>
-      <c r="K19" s="75"/>
-      <c r="L19" s="75"/>
-      <c r="M19" s="76"/>
-    </row>
-    <row r="20" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
+      <c r="C26" s="144"/>
+      <c r="D26" s="145"/>
+      <c r="E26" s="99"/>
+      <c r="F26" s="100"/>
+      <c r="G26" s="100"/>
+      <c r="H26" s="100"/>
+      <c r="I26" s="100"/>
+      <c r="J26" s="100"/>
+      <c r="K26" s="100"/>
+      <c r="L26" s="100"/>
+      <c r="M26" s="101"/>
+    </row>
+    <row r="27" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="121" t="s">
+      <c r="B27" s="143" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="122"/>
-      <c r="D20" s="123"/>
-      <c r="E20" s="74"/>
-      <c r="F20" s="75"/>
-      <c r="G20" s="75"/>
-      <c r="H20" s="75"/>
-      <c r="I20" s="75"/>
-      <c r="J20" s="75"/>
-      <c r="K20" s="75"/>
-      <c r="L20" s="75"/>
-      <c r="M20" s="76"/>
-    </row>
-    <row r="21" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="3"/>
-      <c r="B21" s="121" t="s">
+      <c r="C27" s="144"/>
+      <c r="D27" s="145"/>
+      <c r="E27" s="99"/>
+      <c r="F27" s="100"/>
+      <c r="G27" s="100"/>
+      <c r="H27" s="100"/>
+      <c r="I27" s="100"/>
+      <c r="J27" s="100"/>
+      <c r="K27" s="100"/>
+      <c r="L27" s="100"/>
+      <c r="M27" s="101"/>
+    </row>
+    <row r="28" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="3"/>
+      <c r="B28" s="143" t="s">
         <v>33</v>
       </c>
-      <c r="C21" s="122"/>
-      <c r="D21" s="123"/>
-      <c r="E21" s="74"/>
-      <c r="F21" s="75"/>
-      <c r="G21" s="75"/>
-      <c r="H21" s="75"/>
-      <c r="I21" s="75"/>
-      <c r="J21" s="75"/>
-      <c r="K21" s="75"/>
-      <c r="L21" s="75"/>
-      <c r="M21" s="76"/>
-    </row>
-    <row r="22" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="3"/>
-      <c r="B22" s="121" t="s">
+      <c r="C28" s="144"/>
+      <c r="D28" s="145"/>
+      <c r="E28" s="99"/>
+      <c r="F28" s="100"/>
+      <c r="G28" s="100"/>
+      <c r="H28" s="100"/>
+      <c r="I28" s="100"/>
+      <c r="J28" s="100"/>
+      <c r="K28" s="100"/>
+      <c r="L28" s="100"/>
+      <c r="M28" s="101"/>
+    </row>
+    <row r="29" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="3"/>
+      <c r="B29" s="143" t="s">
         <v>34</v>
       </c>
-      <c r="C22" s="122"/>
-      <c r="D22" s="123"/>
-      <c r="E22" s="74"/>
-      <c r="F22" s="75"/>
-      <c r="G22" s="75"/>
-      <c r="H22" s="75"/>
-      <c r="I22" s="75"/>
-      <c r="J22" s="75"/>
-      <c r="K22" s="75"/>
-      <c r="L22" s="75"/>
-      <c r="M22" s="76"/>
-    </row>
-    <row r="23" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
+      <c r="C29" s="144"/>
+      <c r="D29" s="145"/>
+      <c r="E29" s="99"/>
+      <c r="F29" s="100"/>
+      <c r="G29" s="100"/>
+      <c r="H29" s="100"/>
+      <c r="I29" s="100"/>
+      <c r="J29" s="100"/>
+      <c r="K29" s="100"/>
+      <c r="L29" s="100"/>
+      <c r="M29" s="101"/>
+    </row>
+    <row r="30" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B23" s="121" t="s">
+      <c r="B30" s="143" t="s">
         <v>35</v>
       </c>
-      <c r="C23" s="122"/>
-      <c r="D23" s="123"/>
-      <c r="E23" s="74"/>
-      <c r="F23" s="75"/>
-      <c r="G23" s="75"/>
-      <c r="H23" s="75"/>
-      <c r="I23" s="75"/>
-      <c r="J23" s="75"/>
-      <c r="K23" s="75"/>
-      <c r="L23" s="75"/>
-      <c r="M23" s="76"/>
-    </row>
-    <row r="24" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="6"/>
-      <c r="B24" s="121" t="s">
+      <c r="C30" s="144"/>
+      <c r="D30" s="145"/>
+      <c r="E30" s="99"/>
+      <c r="F30" s="100"/>
+      <c r="G30" s="100"/>
+      <c r="H30" s="100"/>
+      <c r="I30" s="100"/>
+      <c r="J30" s="100"/>
+      <c r="K30" s="100"/>
+      <c r="L30" s="100"/>
+      <c r="M30" s="101"/>
+    </row>
+    <row r="31" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="6"/>
+      <c r="B31" s="143" t="s">
         <v>36</v>
       </c>
-      <c r="C24" s="122"/>
-      <c r="D24" s="123"/>
-      <c r="E24" s="74"/>
-      <c r="F24" s="75"/>
-      <c r="G24" s="75"/>
-      <c r="H24" s="75"/>
-      <c r="I24" s="75"/>
-      <c r="J24" s="75"/>
-      <c r="K24" s="75"/>
-      <c r="L24" s="75"/>
-      <c r="M24" s="76"/>
-    </row>
-    <row r="25" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="6"/>
-      <c r="B25" s="121" t="s">
+      <c r="C31" s="144"/>
+      <c r="D31" s="145"/>
+      <c r="E31" s="99"/>
+      <c r="F31" s="100"/>
+      <c r="G31" s="100"/>
+      <c r="H31" s="100"/>
+      <c r="I31" s="100"/>
+      <c r="J31" s="100"/>
+      <c r="K31" s="100"/>
+      <c r="L31" s="100"/>
+      <c r="M31" s="101"/>
+    </row>
+    <row r="32" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="6"/>
+      <c r="B32" s="143" t="s">
         <v>19</v>
       </c>
-      <c r="C25" s="122"/>
-      <c r="D25" s="123"/>
-      <c r="E25" s="124"/>
-      <c r="F25" s="125"/>
-      <c r="G25" s="125"/>
-      <c r="H25" s="125"/>
-      <c r="I25" s="125"/>
-      <c r="J25" s="125"/>
-      <c r="K25" s="125"/>
-      <c r="L25" s="125"/>
-      <c r="M25" s="126"/>
-    </row>
-    <row r="26" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="6"/>
-      <c r="B26" s="121" t="s">
+      <c r="C32" s="144"/>
+      <c r="D32" s="145"/>
+      <c r="E32" s="146"/>
+      <c r="F32" s="147"/>
+      <c r="G32" s="147"/>
+      <c r="H32" s="147"/>
+      <c r="I32" s="147"/>
+      <c r="J32" s="147"/>
+      <c r="K32" s="147"/>
+      <c r="L32" s="147"/>
+      <c r="M32" s="148"/>
+    </row>
+    <row r="33" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="6"/>
+      <c r="B33" s="143" t="s">
         <v>37</v>
       </c>
-      <c r="C26" s="122"/>
-      <c r="D26" s="123"/>
-      <c r="E26" s="74"/>
-      <c r="F26" s="75"/>
-      <c r="G26" s="75"/>
-      <c r="H26" s="75"/>
-      <c r="I26" s="75"/>
-      <c r="J26" s="75"/>
-      <c r="K26" s="75"/>
-      <c r="L26" s="75"/>
-      <c r="M26" s="76"/>
-    </row>
-    <row r="27" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="7"/>
-      <c r="B27" s="127" t="s">
+      <c r="C33" s="144"/>
+      <c r="D33" s="145"/>
+      <c r="E33" s="99"/>
+      <c r="F33" s="100"/>
+      <c r="G33" s="100"/>
+      <c r="H33" s="100"/>
+      <c r="I33" s="100"/>
+      <c r="J33" s="100"/>
+      <c r="K33" s="100"/>
+      <c r="L33" s="100"/>
+      <c r="M33" s="101"/>
+    </row>
+    <row r="34" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="7"/>
+      <c r="B34" s="149" t="s">
         <v>38</v>
       </c>
-      <c r="C27" s="128"/>
-      <c r="D27" s="129"/>
-      <c r="E27" s="124"/>
-      <c r="F27" s="125"/>
-      <c r="G27" s="125"/>
-      <c r="H27" s="125"/>
-      <c r="I27" s="125"/>
-      <c r="J27" s="125"/>
-      <c r="K27" s="125"/>
-      <c r="L27" s="125"/>
-      <c r="M27" s="126"/>
-    </row>
-    <row r="28" spans="1:13" ht="25.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="8" t="s">
+      <c r="C34" s="150"/>
+      <c r="D34" s="151"/>
+      <c r="E34" s="146"/>
+      <c r="F34" s="147"/>
+      <c r="G34" s="147"/>
+      <c r="H34" s="147"/>
+      <c r="I34" s="147"/>
+      <c r="J34" s="147"/>
+      <c r="K34" s="147"/>
+      <c r="L34" s="147"/>
+      <c r="M34" s="148"/>
+    </row>
+    <row r="35" spans="1:13" ht="25.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="118" t="s">
+      <c r="B35" s="140" t="s">
         <v>41</v>
       </c>
-      <c r="C28" s="119"/>
-      <c r="D28" s="120"/>
-      <c r="E28" s="124"/>
-      <c r="F28" s="125"/>
-      <c r="G28" s="125"/>
-      <c r="H28" s="125"/>
-      <c r="I28" s="125"/>
-      <c r="J28" s="125"/>
-      <c r="K28" s="125"/>
-      <c r="L28" s="125"/>
-      <c r="M28" s="126"/>
-    </row>
-    <row r="29" spans="1:13" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="9" t="s">
+      <c r="C35" s="141"/>
+      <c r="D35" s="142"/>
+      <c r="E35" s="146"/>
+      <c r="F35" s="147"/>
+      <c r="G35" s="147"/>
+      <c r="H35" s="147"/>
+      <c r="I35" s="147"/>
+      <c r="J35" s="147"/>
+      <c r="K35" s="147"/>
+      <c r="L35" s="147"/>
+      <c r="M35" s="148"/>
+    </row>
+    <row r="36" spans="1:13" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B29" s="121" t="s">
+      <c r="B36" s="143" t="s">
         <v>42</v>
       </c>
-      <c r="C29" s="122"/>
-      <c r="D29" s="123"/>
-      <c r="E29" s="124"/>
-      <c r="F29" s="125"/>
-      <c r="G29" s="125"/>
-      <c r="H29" s="125"/>
-      <c r="I29" s="125"/>
-      <c r="J29" s="125"/>
-      <c r="K29" s="125"/>
-      <c r="L29" s="125"/>
-      <c r="M29" s="126"/>
-    </row>
-    <row r="30" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="10"/>
-      <c r="B30" s="121" t="s">
+      <c r="C36" s="144"/>
+      <c r="D36" s="145"/>
+      <c r="E36" s="146"/>
+      <c r="F36" s="147"/>
+      <c r="G36" s="147"/>
+      <c r="H36" s="147"/>
+      <c r="I36" s="147"/>
+      <c r="J36" s="147"/>
+      <c r="K36" s="147"/>
+      <c r="L36" s="147"/>
+      <c r="M36" s="148"/>
+    </row>
+    <row r="37" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="10"/>
+      <c r="B37" s="143" t="s">
         <v>19</v>
       </c>
-      <c r="C30" s="122"/>
-      <c r="D30" s="123"/>
-      <c r="E30" s="124"/>
-      <c r="F30" s="125"/>
-      <c r="G30" s="125"/>
-      <c r="H30" s="125"/>
-      <c r="I30" s="125"/>
-      <c r="J30" s="125"/>
-      <c r="K30" s="125"/>
-      <c r="L30" s="125"/>
-      <c r="M30" s="126"/>
-    </row>
-    <row r="31" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="23" t="s">
+      <c r="C37" s="144"/>
+      <c r="D37" s="145"/>
+      <c r="E37" s="146"/>
+      <c r="F37" s="147"/>
+      <c r="G37" s="147"/>
+      <c r="H37" s="147"/>
+      <c r="I37" s="147"/>
+      <c r="J37" s="147"/>
+      <c r="K37" s="147"/>
+      <c r="L37" s="147"/>
+      <c r="M37" s="148"/>
+    </row>
+    <row r="38" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="B31" s="23"/>
-      <c r="C31" s="23"/>
-      <c r="D31" s="23"/>
-      <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
-      <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
-      <c r="I31" s="23"/>
-      <c r="J31" s="23"/>
-      <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
-    </row>
-    <row r="32" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="23"/>
-      <c r="B32" s="23"/>
-      <c r="C32" s="23"/>
-      <c r="D32" s="23"/>
-      <c r="E32" s="23"/>
-      <c r="F32" s="23"/>
-      <c r="G32" s="23"/>
-      <c r="H32" s="23"/>
-      <c r="I32" s="23"/>
-      <c r="J32" s="23"/>
-      <c r="K32" s="23"/>
-      <c r="L32" s="23"/>
-      <c r="M32" s="23"/>
-    </row>
-    <row r="33" spans="1:13" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="23"/>
-      <c r="B33" s="23"/>
-      <c r="C33" s="23"/>
-      <c r="D33" s="23"/>
-      <c r="E33" s="23"/>
-      <c r="F33" s="23"/>
-      <c r="G33" s="23"/>
-      <c r="H33" s="23"/>
-      <c r="I33" s="23"/>
-      <c r="J33" s="23"/>
-      <c r="K33" s="23"/>
-      <c r="L33" s="23"/>
-      <c r="M33" s="23"/>
-    </row>
-    <row r="34" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="24"/>
-      <c r="B34" s="24"/>
-      <c r="C34" s="24"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="24"/>
-      <c r="G34" s="24"/>
-      <c r="H34" s="24"/>
-      <c r="I34" s="24"/>
-      <c r="J34" s="24"/>
-      <c r="K34" s="24"/>
-      <c r="L34" s="24"/>
-      <c r="M34" s="24"/>
-    </row>
-    <row r="35" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="64" t="s">
+      <c r="B38" s="36"/>
+      <c r="C38" s="36"/>
+      <c r="D38" s="36"/>
+      <c r="E38" s="36"/>
+      <c r="F38" s="36"/>
+      <c r="G38" s="36"/>
+      <c r="H38" s="36"/>
+      <c r="I38" s="36"/>
+      <c r="J38" s="36"/>
+      <c r="K38" s="36"/>
+      <c r="L38" s="36"/>
+      <c r="M38" s="36"/>
+    </row>
+    <row r="39" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="36"/>
+      <c r="B39" s="36"/>
+      <c r="C39" s="36"/>
+      <c r="D39" s="36"/>
+      <c r="E39" s="36"/>
+      <c r="F39" s="36"/>
+      <c r="G39" s="36"/>
+      <c r="H39" s="36"/>
+      <c r="I39" s="36"/>
+      <c r="J39" s="36"/>
+      <c r="K39" s="36"/>
+      <c r="L39" s="36"/>
+      <c r="M39" s="36"/>
+    </row>
+    <row r="40" spans="1:13" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="36"/>
+      <c r="B40" s="36"/>
+      <c r="C40" s="36"/>
+      <c r="D40" s="36"/>
+      <c r="E40" s="36"/>
+      <c r="F40" s="36"/>
+      <c r="G40" s="36"/>
+      <c r="H40" s="36"/>
+      <c r="I40" s="36"/>
+      <c r="J40" s="36"/>
+      <c r="K40" s="36"/>
+      <c r="L40" s="36"/>
+      <c r="M40" s="36"/>
+    </row>
+    <row r="41" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="37"/>
+      <c r="B41" s="37"/>
+      <c r="C41" s="37"/>
+      <c r="D41" s="37"/>
+      <c r="E41" s="37"/>
+      <c r="F41" s="37"/>
+      <c r="G41" s="37"/>
+      <c r="H41" s="37"/>
+      <c r="I41" s="37"/>
+      <c r="J41" s="37"/>
+      <c r="K41" s="37"/>
+      <c r="L41" s="37"/>
+      <c r="M41" s="37"/>
+    </row>
+    <row r="42" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="77" t="s">
         <v>114</v>
       </c>
-      <c r="B35" s="65"/>
-      <c r="C35" s="65"/>
-      <c r="D35" s="65"/>
-      <c r="E35" s="65"/>
-      <c r="F35" s="65"/>
-      <c r="G35" s="65"/>
-      <c r="H35" s="65"/>
-      <c r="I35" s="65"/>
-      <c r="J35" s="65"/>
-      <c r="K35" s="65"/>
-      <c r="L35" s="65"/>
-      <c r="M35" s="66"/>
-    </row>
-    <row r="36" spans="1:13" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="67" t="s">
+      <c r="B42" s="78"/>
+      <c r="C42" s="78"/>
+      <c r="D42" s="78"/>
+      <c r="E42" s="78"/>
+      <c r="F42" s="78"/>
+      <c r="G42" s="78"/>
+      <c r="H42" s="78"/>
+      <c r="I42" s="78"/>
+      <c r="J42" s="78"/>
+      <c r="K42" s="78"/>
+      <c r="L42" s="78"/>
+      <c r="M42" s="79"/>
+    </row>
+    <row r="43" spans="1:13" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="80" t="s">
         <v>44</v>
       </c>
-      <c r="B36" s="52"/>
-      <c r="C36" s="53"/>
-      <c r="D36" s="53"/>
-      <c r="E36" s="54"/>
-      <c r="F36" s="105" t="s">
+      <c r="B43" s="82"/>
+      <c r="C43" s="83"/>
+      <c r="D43" s="83"/>
+      <c r="E43" s="84"/>
+      <c r="F43" s="88" t="s">
         <v>45</v>
       </c>
-      <c r="G36" s="106"/>
-      <c r="H36" s="109"/>
-      <c r="I36" s="54"/>
-      <c r="J36" s="105" t="s">
+      <c r="G43" s="133"/>
+      <c r="H43" s="136"/>
+      <c r="I43" s="84"/>
+      <c r="J43" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="K36" s="111"/>
-      <c r="L36" s="112"/>
-      <c r="M36" s="116"/>
-    </row>
-    <row r="37" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="68"/>
-      <c r="B37" s="58"/>
-      <c r="C37" s="59"/>
-      <c r="D37" s="59"/>
-      <c r="E37" s="60"/>
-      <c r="F37" s="107"/>
-      <c r="G37" s="108"/>
-      <c r="H37" s="110"/>
-      <c r="I37" s="60"/>
-      <c r="J37" s="113" t="s">
+      <c r="K43" s="89"/>
+      <c r="L43" s="90"/>
+      <c r="M43" s="138"/>
+    </row>
+    <row r="44" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="81"/>
+      <c r="B44" s="85"/>
+      <c r="C44" s="86"/>
+      <c r="D44" s="86"/>
+      <c r="E44" s="87"/>
+      <c r="F44" s="134"/>
+      <c r="G44" s="135"/>
+      <c r="H44" s="137"/>
+      <c r="I44" s="87"/>
+      <c r="J44" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="K37" s="114"/>
-      <c r="L37" s="115"/>
-      <c r="M37" s="117"/>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A38" s="25" t="s">
+      <c r="K44" s="92"/>
+      <c r="L44" s="93"/>
+      <c r="M44" s="139"/>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A45" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="B38" s="45"/>
-      <c r="C38" s="26"/>
-      <c r="D38" s="52"/>
-      <c r="E38" s="53"/>
-      <c r="F38" s="53"/>
-      <c r="G38" s="54"/>
-      <c r="H38" s="25" t="s">
+      <c r="B45" s="58"/>
+      <c r="C45" s="39"/>
+      <c r="D45" s="65"/>
+      <c r="E45" s="66"/>
+      <c r="F45" s="66"/>
+      <c r="G45" s="67"/>
+      <c r="H45" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="I38" s="45"/>
-      <c r="J38" s="45"/>
-      <c r="K38" s="61"/>
-      <c r="L38" s="99"/>
-      <c r="M38" s="100"/>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A39" s="46" t="s">
+      <c r="I45" s="58"/>
+      <c r="J45" s="58"/>
+      <c r="K45" s="74"/>
+      <c r="L45" s="127"/>
+      <c r="M45" s="128"/>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A46" s="59" t="s">
         <v>40</v>
       </c>
-      <c r="B39" s="47"/>
-      <c r="C39" s="48"/>
-      <c r="D39" s="55"/>
-      <c r="E39" s="56"/>
-      <c r="F39" s="56"/>
-      <c r="G39" s="57"/>
-      <c r="H39" s="46" t="s">
+      <c r="B46" s="60"/>
+      <c r="C46" s="61"/>
+      <c r="D46" s="68"/>
+      <c r="E46" s="69"/>
+      <c r="F46" s="69"/>
+      <c r="G46" s="70"/>
+      <c r="H46" s="59" t="s">
         <v>50</v>
       </c>
-      <c r="I39" s="47"/>
-      <c r="J39" s="47"/>
-      <c r="K39" s="62"/>
-      <c r="L39" s="101"/>
-      <c r="M39" s="102"/>
-    </row>
-    <row r="40" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="49"/>
-      <c r="B40" s="50"/>
-      <c r="C40" s="51"/>
-      <c r="D40" s="58"/>
-      <c r="E40" s="59"/>
-      <c r="F40" s="59"/>
-      <c r="G40" s="60"/>
-      <c r="H40" s="49"/>
-      <c r="I40" s="50"/>
-      <c r="J40" s="50"/>
-      <c r="K40" s="63"/>
-      <c r="L40" s="103"/>
-      <c r="M40" s="104"/>
-    </row>
-    <row r="41" spans="1:13" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="35" t="s">
+      <c r="I46" s="60"/>
+      <c r="J46" s="60"/>
+      <c r="K46" s="75"/>
+      <c r="L46" s="129"/>
+      <c r="M46" s="130"/>
+    </row>
+    <row r="47" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="62"/>
+      <c r="B47" s="63"/>
+      <c r="C47" s="64"/>
+      <c r="D47" s="71"/>
+      <c r="E47" s="72"/>
+      <c r="F47" s="72"/>
+      <c r="G47" s="73"/>
+      <c r="H47" s="62"/>
+      <c r="I47" s="63"/>
+      <c r="J47" s="63"/>
+      <c r="K47" s="76"/>
+      <c r="L47" s="131"/>
+      <c r="M47" s="132"/>
+    </row>
+    <row r="48" spans="1:13" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="48" t="s">
         <v>51</v>
       </c>
-      <c r="B41" s="36"/>
-      <c r="C41" s="37"/>
-      <c r="D41" s="38"/>
-      <c r="E41" s="39"/>
-      <c r="F41" s="39"/>
-      <c r="G41" s="39"/>
-      <c r="H41" s="39"/>
-      <c r="I41" s="39"/>
-      <c r="J41" s="39"/>
-      <c r="K41" s="39"/>
-      <c r="L41" s="39"/>
-      <c r="M41" s="40"/>
-    </row>
-    <row r="42" spans="1:13" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="41" t="s">
+      <c r="B48" s="49"/>
+      <c r="C48" s="50"/>
+      <c r="D48" s="51"/>
+      <c r="E48" s="52"/>
+      <c r="F48" s="52"/>
+      <c r="G48" s="52"/>
+      <c r="H48" s="52"/>
+      <c r="I48" s="52"/>
+      <c r="J48" s="52"/>
+      <c r="K48" s="52"/>
+      <c r="L48" s="52"/>
+      <c r="M48" s="53"/>
+    </row>
+    <row r="49" spans="1:13" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="54" t="s">
         <v>52</v>
       </c>
-      <c r="B42" s="42"/>
-      <c r="C42" s="43"/>
-      <c r="D42" s="43"/>
-      <c r="E42" s="43"/>
-      <c r="F42" s="43"/>
-      <c r="G42" s="43"/>
-      <c r="H42" s="43"/>
-      <c r="I42" s="43"/>
-      <c r="J42" s="43"/>
-      <c r="K42" s="43"/>
-      <c r="L42" s="43"/>
-      <c r="M42" s="44"/>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A43" s="25" t="s">
+      <c r="B49" s="55"/>
+      <c r="C49" s="56"/>
+      <c r="D49" s="56"/>
+      <c r="E49" s="56"/>
+      <c r="F49" s="56"/>
+      <c r="G49" s="56"/>
+      <c r="H49" s="56"/>
+      <c r="I49" s="56"/>
+      <c r="J49" s="56"/>
+      <c r="K49" s="56"/>
+      <c r="L49" s="56"/>
+      <c r="M49" s="57"/>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A50" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="26"/>
-      <c r="C43" s="142"/>
-      <c r="D43" s="143"/>
-      <c r="E43" s="143"/>
-      <c r="F43" s="143"/>
-      <c r="G43" s="143"/>
-      <c r="H43" s="143"/>
-      <c r="I43" s="143"/>
-      <c r="J43" s="143"/>
-      <c r="K43" s="143"/>
-      <c r="L43" s="143"/>
-      <c r="M43" s="143"/>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A44" s="27"/>
-      <c r="B44" s="28"/>
-      <c r="C44" s="142"/>
-      <c r="D44" s="143"/>
-      <c r="E44" s="143"/>
-      <c r="F44" s="143"/>
-      <c r="G44" s="143"/>
-      <c r="H44" s="143"/>
-      <c r="I44" s="143"/>
-      <c r="J44" s="143"/>
-      <c r="K44" s="143"/>
-      <c r="L44" s="143"/>
-      <c r="M44" s="143"/>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A45" s="27"/>
-      <c r="B45" s="28"/>
-      <c r="C45" s="142"/>
-      <c r="D45" s="143"/>
-      <c r="E45" s="143"/>
-      <c r="F45" s="143"/>
-      <c r="G45" s="143"/>
-      <c r="H45" s="143"/>
-      <c r="I45" s="143"/>
-      <c r="J45" s="143"/>
-      <c r="K45" s="143"/>
-      <c r="L45" s="143"/>
-      <c r="M45" s="143"/>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A46" s="27"/>
-      <c r="B46" s="28"/>
-      <c r="C46" s="142"/>
-      <c r="D46" s="143"/>
-      <c r="E46" s="143"/>
-      <c r="F46" s="143"/>
-      <c r="G46" s="143"/>
-      <c r="H46" s="143"/>
-      <c r="I46" s="143"/>
-      <c r="J46" s="143"/>
-      <c r="K46" s="143"/>
-      <c r="L46" s="143"/>
-      <c r="M46" s="143"/>
-    </row>
-    <row r="47" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="29"/>
-      <c r="B47" s="30"/>
-      <c r="C47" s="142"/>
-      <c r="D47" s="143"/>
-      <c r="E47" s="143"/>
-      <c r="F47" s="143"/>
-      <c r="G47" s="143"/>
-      <c r="H47" s="143"/>
-      <c r="I47" s="143"/>
-      <c r="J47" s="143"/>
-      <c r="K47" s="143"/>
-      <c r="L47" s="143"/>
-      <c r="M47" s="143"/>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A48" s="25" t="s">
+      <c r="B50" s="39"/>
+      <c r="C50" s="164"/>
+      <c r="D50" s="165"/>
+      <c r="E50" s="165"/>
+      <c r="F50" s="165"/>
+      <c r="G50" s="165"/>
+      <c r="H50" s="165"/>
+      <c r="I50" s="165"/>
+      <c r="J50" s="165"/>
+      <c r="K50" s="165"/>
+      <c r="L50" s="165"/>
+      <c r="M50" s="165"/>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A51" s="40"/>
+      <c r="B51" s="41"/>
+      <c r="C51" s="164"/>
+      <c r="D51" s="165"/>
+      <c r="E51" s="165"/>
+      <c r="F51" s="165"/>
+      <c r="G51" s="165"/>
+      <c r="H51" s="165"/>
+      <c r="I51" s="165"/>
+      <c r="J51" s="165"/>
+      <c r="K51" s="165"/>
+      <c r="L51" s="165"/>
+      <c r="M51" s="165"/>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A52" s="40"/>
+      <c r="B52" s="41"/>
+      <c r="C52" s="164"/>
+      <c r="D52" s="165"/>
+      <c r="E52" s="165"/>
+      <c r="F52" s="165"/>
+      <c r="G52" s="165"/>
+      <c r="H52" s="165"/>
+      <c r="I52" s="165"/>
+      <c r="J52" s="165"/>
+      <c r="K52" s="165"/>
+      <c r="L52" s="165"/>
+      <c r="M52" s="165"/>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A53" s="40"/>
+      <c r="B53" s="41"/>
+      <c r="C53" s="164"/>
+      <c r="D53" s="165"/>
+      <c r="E53" s="165"/>
+      <c r="F53" s="165"/>
+      <c r="G53" s="165"/>
+      <c r="H53" s="165"/>
+      <c r="I53" s="165"/>
+      <c r="J53" s="165"/>
+      <c r="K53" s="165"/>
+      <c r="L53" s="165"/>
+      <c r="M53" s="165"/>
+    </row>
+    <row r="54" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="42"/>
+      <c r="B54" s="43"/>
+      <c r="C54" s="164"/>
+      <c r="D54" s="165"/>
+      <c r="E54" s="165"/>
+      <c r="F54" s="165"/>
+      <c r="G54" s="165"/>
+      <c r="H54" s="165"/>
+      <c r="I54" s="165"/>
+      <c r="J54" s="165"/>
+      <c r="K54" s="165"/>
+      <c r="L54" s="165"/>
+      <c r="M54" s="165"/>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A55" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="B48" s="26"/>
-      <c r="C48" s="142"/>
-      <c r="D48" s="143"/>
-      <c r="E48" s="143"/>
-      <c r="F48" s="143"/>
-      <c r="G48" s="143"/>
-      <c r="H48" s="143"/>
-      <c r="I48" s="143"/>
-      <c r="J48" s="143"/>
-      <c r="K48" s="143"/>
-      <c r="L48" s="143"/>
-      <c r="M48" s="143"/>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A49" s="27"/>
-      <c r="B49" s="28"/>
-      <c r="C49" s="142"/>
-      <c r="D49" s="143"/>
-      <c r="E49" s="143"/>
-      <c r="F49" s="143"/>
-      <c r="G49" s="143"/>
-      <c r="H49" s="143"/>
-      <c r="I49" s="143"/>
-      <c r="J49" s="143"/>
-      <c r="K49" s="143"/>
-      <c r="L49" s="143"/>
-      <c r="M49" s="143"/>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A50" s="27"/>
-      <c r="B50" s="28"/>
-      <c r="C50" s="142"/>
-      <c r="D50" s="143"/>
-      <c r="E50" s="143"/>
-      <c r="F50" s="143"/>
-      <c r="G50" s="143"/>
-      <c r="H50" s="143"/>
-      <c r="I50" s="143"/>
-      <c r="J50" s="143"/>
-      <c r="K50" s="143"/>
-      <c r="L50" s="143"/>
-      <c r="M50" s="143"/>
-    </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A51" s="27"/>
-      <c r="B51" s="28"/>
-      <c r="C51" s="142"/>
-      <c r="D51" s="143"/>
-      <c r="E51" s="143"/>
-      <c r="F51" s="143"/>
-      <c r="G51" s="143"/>
-      <c r="H51" s="143"/>
-      <c r="I51" s="143"/>
-      <c r="J51" s="143"/>
-      <c r="K51" s="143"/>
-      <c r="L51" s="143"/>
-      <c r="M51" s="143"/>
-    </row>
-    <row r="52" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="29"/>
-      <c r="B52" s="30"/>
-      <c r="C52" s="142"/>
-      <c r="D52" s="143"/>
-      <c r="E52" s="143"/>
-      <c r="F52" s="143"/>
-      <c r="G52" s="143"/>
-      <c r="H52" s="143"/>
-      <c r="I52" s="143"/>
-      <c r="J52" s="143"/>
-      <c r="K52" s="143"/>
-      <c r="L52" s="143"/>
-      <c r="M52" s="143"/>
-    </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A53" s="25" t="s">
+      <c r="B55" s="39"/>
+      <c r="C55" s="164"/>
+      <c r="D55" s="165"/>
+      <c r="E55" s="165"/>
+      <c r="F55" s="165"/>
+      <c r="G55" s="165"/>
+      <c r="H55" s="165"/>
+      <c r="I55" s="165"/>
+      <c r="J55" s="165"/>
+      <c r="K55" s="165"/>
+      <c r="L55" s="165"/>
+      <c r="M55" s="165"/>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A56" s="40"/>
+      <c r="B56" s="41"/>
+      <c r="C56" s="164"/>
+      <c r="D56" s="165"/>
+      <c r="E56" s="165"/>
+      <c r="F56" s="165"/>
+      <c r="G56" s="165"/>
+      <c r="H56" s="165"/>
+      <c r="I56" s="165"/>
+      <c r="J56" s="165"/>
+      <c r="K56" s="165"/>
+      <c r="L56" s="165"/>
+      <c r="M56" s="165"/>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A57" s="40"/>
+      <c r="B57" s="41"/>
+      <c r="C57" s="164"/>
+      <c r="D57" s="165"/>
+      <c r="E57" s="165"/>
+      <c r="F57" s="165"/>
+      <c r="G57" s="165"/>
+      <c r="H57" s="165"/>
+      <c r="I57" s="165"/>
+      <c r="J57" s="165"/>
+      <c r="K57" s="165"/>
+      <c r="L57" s="165"/>
+      <c r="M57" s="165"/>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A58" s="40"/>
+      <c r="B58" s="41"/>
+      <c r="C58" s="164"/>
+      <c r="D58" s="165"/>
+      <c r="E58" s="165"/>
+      <c r="F58" s="165"/>
+      <c r="G58" s="165"/>
+      <c r="H58" s="165"/>
+      <c r="I58" s="165"/>
+      <c r="J58" s="165"/>
+      <c r="K58" s="165"/>
+      <c r="L58" s="165"/>
+      <c r="M58" s="165"/>
+    </row>
+    <row r="59" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="42"/>
+      <c r="B59" s="43"/>
+      <c r="C59" s="164"/>
+      <c r="D59" s="165"/>
+      <c r="E59" s="165"/>
+      <c r="F59" s="165"/>
+      <c r="G59" s="165"/>
+      <c r="H59" s="165"/>
+      <c r="I59" s="165"/>
+      <c r="J59" s="165"/>
+      <c r="K59" s="165"/>
+      <c r="L59" s="165"/>
+      <c r="M59" s="165"/>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A60" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="B53" s="26"/>
-      <c r="C53" s="142"/>
-      <c r="D53" s="143"/>
-      <c r="E53" s="143"/>
-      <c r="F53" s="143"/>
-      <c r="G53" s="143"/>
-      <c r="H53" s="143"/>
-      <c r="I53" s="143"/>
-      <c r="J53" s="143"/>
-      <c r="K53" s="143"/>
-      <c r="L53" s="143"/>
-      <c r="M53" s="143"/>
-    </row>
-    <row r="54" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="27"/>
-      <c r="B54" s="28"/>
-      <c r="C54" s="142"/>
-      <c r="D54" s="143"/>
-      <c r="E54" s="143"/>
-      <c r="F54" s="143"/>
-      <c r="G54" s="143"/>
-      <c r="H54" s="143"/>
-      <c r="I54" s="143"/>
-      <c r="J54" s="143"/>
-      <c r="K54" s="143"/>
-      <c r="L54" s="143"/>
-      <c r="M54" s="143"/>
-    </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A55" s="27"/>
-      <c r="B55" s="28"/>
-      <c r="C55" s="142"/>
-      <c r="D55" s="143"/>
-      <c r="E55" s="143"/>
-      <c r="F55" s="143"/>
-      <c r="G55" s="143"/>
-      <c r="H55" s="143"/>
-      <c r="I55" s="143"/>
-      <c r="J55" s="143"/>
-      <c r="K55" s="143"/>
-      <c r="L55" s="143"/>
-      <c r="M55" s="143"/>
-    </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A56" s="27"/>
-      <c r="B56" s="28"/>
-      <c r="C56" s="142"/>
-      <c r="D56" s="143"/>
-      <c r="E56" s="143"/>
-      <c r="F56" s="143"/>
-      <c r="G56" s="143"/>
-      <c r="H56" s="143"/>
-      <c r="I56" s="143"/>
-      <c r="J56" s="143"/>
-      <c r="K56" s="143"/>
-      <c r="L56" s="143"/>
-      <c r="M56" s="143"/>
-    </row>
-    <row r="57" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="29"/>
-      <c r="B57" s="30"/>
-      <c r="C57" s="142"/>
-      <c r="D57" s="143"/>
-      <c r="E57" s="143"/>
-      <c r="F57" s="143"/>
-      <c r="G57" s="143"/>
-      <c r="H57" s="143"/>
-      <c r="I57" s="143"/>
-      <c r="J57" s="143"/>
-      <c r="K57" s="143"/>
-      <c r="L57" s="143"/>
-      <c r="M57" s="143"/>
-    </row>
-    <row r="58" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="25" t="s">
+      <c r="B60" s="39"/>
+      <c r="C60" s="164"/>
+      <c r="D60" s="165"/>
+      <c r="E60" s="165"/>
+      <c r="F60" s="165"/>
+      <c r="G60" s="165"/>
+      <c r="H60" s="165"/>
+      <c r="I60" s="165"/>
+      <c r="J60" s="165"/>
+      <c r="K60" s="165"/>
+      <c r="L60" s="165"/>
+      <c r="M60" s="165"/>
+    </row>
+    <row r="61" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="40"/>
+      <c r="B61" s="41"/>
+      <c r="C61" s="164"/>
+      <c r="D61" s="165"/>
+      <c r="E61" s="165"/>
+      <c r="F61" s="165"/>
+      <c r="G61" s="165"/>
+      <c r="H61" s="165"/>
+      <c r="I61" s="165"/>
+      <c r="J61" s="165"/>
+      <c r="K61" s="165"/>
+      <c r="L61" s="165"/>
+      <c r="M61" s="165"/>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A62" s="40"/>
+      <c r="B62" s="41"/>
+      <c r="C62" s="164"/>
+      <c r="D62" s="165"/>
+      <c r="E62" s="165"/>
+      <c r="F62" s="165"/>
+      <c r="G62" s="165"/>
+      <c r="H62" s="165"/>
+      <c r="I62" s="165"/>
+      <c r="J62" s="165"/>
+      <c r="K62" s="165"/>
+      <c r="L62" s="165"/>
+      <c r="M62" s="165"/>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A63" s="40"/>
+      <c r="B63" s="41"/>
+      <c r="C63" s="164"/>
+      <c r="D63" s="165"/>
+      <c r="E63" s="165"/>
+      <c r="F63" s="165"/>
+      <c r="G63" s="165"/>
+      <c r="H63" s="165"/>
+      <c r="I63" s="165"/>
+      <c r="J63" s="165"/>
+      <c r="K63" s="165"/>
+      <c r="L63" s="165"/>
+      <c r="M63" s="165"/>
+    </row>
+    <row r="64" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="42"/>
+      <c r="B64" s="43"/>
+      <c r="C64" s="164"/>
+      <c r="D64" s="165"/>
+      <c r="E64" s="165"/>
+      <c r="F64" s="165"/>
+      <c r="G64" s="165"/>
+      <c r="H64" s="165"/>
+      <c r="I64" s="165"/>
+      <c r="J64" s="165"/>
+      <c r="K64" s="165"/>
+      <c r="L64" s="165"/>
+      <c r="M64" s="165"/>
+    </row>
+    <row r="65" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="B58" s="26"/>
-      <c r="C58" s="91"/>
-      <c r="D58" s="92"/>
-      <c r="E58" s="92"/>
-      <c r="F58" s="92"/>
-      <c r="G58" s="92"/>
-      <c r="H58" s="92"/>
-      <c r="I58" s="92"/>
-      <c r="J58" s="92"/>
-      <c r="K58" s="92"/>
-      <c r="L58" s="92"/>
-      <c r="M58" s="93"/>
-    </row>
-    <row r="59" spans="1:13" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="29"/>
-      <c r="B59" s="30"/>
-      <c r="C59" s="94"/>
-      <c r="D59" s="95"/>
-      <c r="E59" s="95"/>
-      <c r="F59" s="95"/>
-      <c r="G59" s="95"/>
-      <c r="H59" s="95"/>
-      <c r="I59" s="95"/>
-      <c r="J59" s="95"/>
-      <c r="K59" s="95"/>
-      <c r="L59" s="95"/>
-      <c r="M59" s="96"/>
-    </row>
-    <row r="60" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="25" t="s">
+      <c r="B65" s="39"/>
+      <c r="C65" s="119"/>
+      <c r="D65" s="120"/>
+      <c r="E65" s="120"/>
+      <c r="F65" s="120"/>
+      <c r="G65" s="120"/>
+      <c r="H65" s="120"/>
+      <c r="I65" s="120"/>
+      <c r="J65" s="120"/>
+      <c r="K65" s="120"/>
+      <c r="L65" s="120"/>
+      <c r="M65" s="121"/>
+    </row>
+    <row r="66" spans="1:13" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="42"/>
+      <c r="B66" s="43"/>
+      <c r="C66" s="122"/>
+      <c r="D66" s="123"/>
+      <c r="E66" s="123"/>
+      <c r="F66" s="123"/>
+      <c r="G66" s="123"/>
+      <c r="H66" s="123"/>
+      <c r="I66" s="123"/>
+      <c r="J66" s="123"/>
+      <c r="K66" s="123"/>
+      <c r="L66" s="123"/>
+      <c r="M66" s="124"/>
+    </row>
+    <row r="67" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="B60" s="26"/>
-      <c r="C60" s="88"/>
-      <c r="D60" s="89"/>
-      <c r="E60" s="89"/>
-      <c r="F60" s="89"/>
-      <c r="G60" s="89"/>
-      <c r="H60" s="89"/>
-      <c r="I60" s="89"/>
-      <c r="J60" s="89"/>
-      <c r="K60" s="89"/>
-      <c r="L60" s="89"/>
-      <c r="M60" s="90"/>
-    </row>
-    <row r="61" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="27"/>
-      <c r="B61" s="28"/>
-      <c r="C61" s="91"/>
-      <c r="D61" s="92"/>
-      <c r="E61" s="92"/>
-      <c r="F61" s="92"/>
-      <c r="G61" s="92"/>
-      <c r="H61" s="92"/>
-      <c r="I61" s="92"/>
-      <c r="J61" s="92"/>
-      <c r="K61" s="92"/>
-      <c r="L61" s="92"/>
-      <c r="M61" s="93"/>
-    </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A62" s="27"/>
-      <c r="B62" s="28"/>
-      <c r="C62" s="91"/>
-      <c r="D62" s="92"/>
-      <c r="E62" s="92"/>
-      <c r="F62" s="92"/>
-      <c r="G62" s="92"/>
-      <c r="H62" s="92"/>
-      <c r="I62" s="92"/>
-      <c r="J62" s="92"/>
-      <c r="K62" s="92"/>
-      <c r="L62" s="92"/>
-      <c r="M62" s="93"/>
-    </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A63" s="27"/>
-      <c r="B63" s="28"/>
-      <c r="C63" s="91"/>
-      <c r="D63" s="92"/>
-      <c r="E63" s="92"/>
-      <c r="F63" s="92"/>
-      <c r="G63" s="92"/>
-      <c r="H63" s="92"/>
-      <c r="I63" s="92"/>
-      <c r="J63" s="92"/>
-      <c r="K63" s="92"/>
-      <c r="L63" s="92"/>
-      <c r="M63" s="93"/>
-    </row>
-    <row r="64" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="29"/>
-      <c r="B64" s="30"/>
-      <c r="C64" s="94"/>
-      <c r="D64" s="95"/>
-      <c r="E64" s="95"/>
-      <c r="F64" s="95"/>
-      <c r="G64" s="95"/>
-      <c r="H64" s="95"/>
-      <c r="I64" s="95"/>
-      <c r="J64" s="95"/>
-      <c r="K64" s="95"/>
-      <c r="L64" s="95"/>
-      <c r="M64" s="96"/>
-    </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A65" s="97"/>
-      <c r="B65" s="97"/>
-      <c r="C65" s="97"/>
-      <c r="D65" s="97"/>
-      <c r="E65" s="47"/>
-      <c r="F65" s="47"/>
-      <c r="G65" s="97"/>
-      <c r="H65" s="97"/>
-      <c r="I65" s="47"/>
-      <c r="J65" s="47"/>
-      <c r="K65" s="97"/>
-      <c r="L65" s="97"/>
-      <c r="M65" s="97"/>
-    </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A66" s="97"/>
-      <c r="B66" s="97"/>
-      <c r="C66" s="97"/>
-      <c r="D66" s="97"/>
-      <c r="E66" s="47"/>
-      <c r="F66" s="47"/>
-      <c r="G66" s="97"/>
-      <c r="H66" s="97"/>
-      <c r="I66" s="47"/>
-      <c r="J66" s="47"/>
-      <c r="K66" s="97"/>
-      <c r="L66" s="97"/>
-      <c r="M66" s="97"/>
-    </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A67" s="97"/>
-      <c r="B67" s="97"/>
-      <c r="C67" s="97"/>
-      <c r="D67" s="97"/>
-      <c r="E67" s="47"/>
-      <c r="F67" s="47"/>
-      <c r="G67" s="97"/>
-      <c r="H67" s="97"/>
-      <c r="I67" s="47"/>
-      <c r="J67" s="47"/>
-      <c r="K67" s="97"/>
-      <c r="L67" s="97"/>
-      <c r="M67" s="97"/>
-    </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A68" s="97"/>
-      <c r="B68" s="97"/>
-      <c r="C68" s="97"/>
-      <c r="D68" s="97"/>
-      <c r="E68" s="47"/>
-      <c r="F68" s="47"/>
-      <c r="G68" s="97"/>
-      <c r="H68" s="97"/>
-      <c r="I68" s="47"/>
-      <c r="J68" s="47"/>
-      <c r="K68" s="97"/>
-      <c r="L68" s="97"/>
-      <c r="M68" s="97"/>
+      <c r="B67" s="39"/>
+      <c r="C67" s="116"/>
+      <c r="D67" s="117"/>
+      <c r="E67" s="117"/>
+      <c r="F67" s="117"/>
+      <c r="G67" s="117"/>
+      <c r="H67" s="117"/>
+      <c r="I67" s="117"/>
+      <c r="J67" s="117"/>
+      <c r="K67" s="117"/>
+      <c r="L67" s="117"/>
+      <c r="M67" s="118"/>
+    </row>
+    <row r="68" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="40"/>
+      <c r="B68" s="41"/>
+      <c r="C68" s="119"/>
+      <c r="D68" s="120"/>
+      <c r="E68" s="120"/>
+      <c r="F68" s="120"/>
+      <c r="G68" s="120"/>
+      <c r="H68" s="120"/>
+      <c r="I68" s="120"/>
+      <c r="J68" s="120"/>
+      <c r="K68" s="120"/>
+      <c r="L68" s="120"/>
+      <c r="M68" s="121"/>
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A69" s="97"/>
-      <c r="B69" s="97"/>
-      <c r="C69" s="97"/>
-      <c r="D69" s="97"/>
-      <c r="E69" s="47"/>
-      <c r="F69" s="47"/>
-      <c r="G69" s="97"/>
-      <c r="H69" s="97"/>
-      <c r="I69" s="47"/>
-      <c r="J69" s="47"/>
-      <c r="K69" s="97"/>
-      <c r="L69" s="97"/>
-      <c r="M69" s="97"/>
-    </row>
-    <row r="70" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="98"/>
-      <c r="B70" s="98"/>
-      <c r="C70" s="98"/>
-      <c r="D70" s="98"/>
-      <c r="E70" s="47"/>
-      <c r="F70" s="47"/>
-      <c r="G70" s="98"/>
-      <c r="H70" s="98"/>
-      <c r="I70" s="47"/>
-      <c r="J70" s="47"/>
-      <c r="K70" s="98"/>
-      <c r="L70" s="98"/>
-      <c r="M70" s="98"/>
-    </row>
-    <row r="71" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="86"/>
-      <c r="B71" s="86"/>
-      <c r="C71" s="86"/>
-      <c r="D71" s="86"/>
-      <c r="E71" s="47"/>
-      <c r="F71" s="47"/>
-      <c r="G71" s="87" t="s">
+      <c r="A69" s="40"/>
+      <c r="B69" s="41"/>
+      <c r="C69" s="119"/>
+      <c r="D69" s="120"/>
+      <c r="E69" s="120"/>
+      <c r="F69" s="120"/>
+      <c r="G69" s="120"/>
+      <c r="H69" s="120"/>
+      <c r="I69" s="120"/>
+      <c r="J69" s="120"/>
+      <c r="K69" s="120"/>
+      <c r="L69" s="120"/>
+      <c r="M69" s="121"/>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A70" s="40"/>
+      <c r="B70" s="41"/>
+      <c r="C70" s="119"/>
+      <c r="D70" s="120"/>
+      <c r="E70" s="120"/>
+      <c r="F70" s="120"/>
+      <c r="G70" s="120"/>
+      <c r="H70" s="120"/>
+      <c r="I70" s="120"/>
+      <c r="J70" s="120"/>
+      <c r="K70" s="120"/>
+      <c r="L70" s="120"/>
+      <c r="M70" s="121"/>
+    </row>
+    <row r="71" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="42"/>
+      <c r="B71" s="43"/>
+      <c r="C71" s="122"/>
+      <c r="D71" s="123"/>
+      <c r="E71" s="123"/>
+      <c r="F71" s="123"/>
+      <c r="G71" s="123"/>
+      <c r="H71" s="123"/>
+      <c r="I71" s="123"/>
+      <c r="J71" s="123"/>
+      <c r="K71" s="123"/>
+      <c r="L71" s="123"/>
+      <c r="M71" s="124"/>
+    </row>
+    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A72" s="125"/>
+      <c r="B72" s="125"/>
+      <c r="C72" s="125"/>
+      <c r="D72" s="125"/>
+      <c r="E72" s="60"/>
+      <c r="F72" s="60"/>
+      <c r="G72" s="125"/>
+      <c r="H72" s="125"/>
+      <c r="I72" s="60"/>
+      <c r="J72" s="60"/>
+      <c r="K72" s="125"/>
+      <c r="L72" s="125"/>
+      <c r="M72" s="125"/>
+    </row>
+    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A73" s="125"/>
+      <c r="B73" s="125"/>
+      <c r="C73" s="125"/>
+      <c r="D73" s="125"/>
+      <c r="E73" s="60"/>
+      <c r="F73" s="60"/>
+      <c r="G73" s="125"/>
+      <c r="H73" s="125"/>
+      <c r="I73" s="60"/>
+      <c r="J73" s="60"/>
+      <c r="K73" s="125"/>
+      <c r="L73" s="125"/>
+      <c r="M73" s="125"/>
+    </row>
+    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A74" s="125"/>
+      <c r="B74" s="125"/>
+      <c r="C74" s="125"/>
+      <c r="D74" s="125"/>
+      <c r="E74" s="60"/>
+      <c r="F74" s="60"/>
+      <c r="G74" s="125"/>
+      <c r="H74" s="125"/>
+      <c r="I74" s="60"/>
+      <c r="J74" s="60"/>
+      <c r="K74" s="125"/>
+      <c r="L74" s="125"/>
+      <c r="M74" s="125"/>
+    </row>
+    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A75" s="125"/>
+      <c r="B75" s="125"/>
+      <c r="C75" s="125"/>
+      <c r="D75" s="125"/>
+      <c r="E75" s="60"/>
+      <c r="F75" s="60"/>
+      <c r="G75" s="125"/>
+      <c r="H75" s="125"/>
+      <c r="I75" s="60"/>
+      <c r="J75" s="60"/>
+      <c r="K75" s="125"/>
+      <c r="L75" s="125"/>
+      <c r="M75" s="125"/>
+    </row>
+    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A76" s="125"/>
+      <c r="B76" s="125"/>
+      <c r="C76" s="125"/>
+      <c r="D76" s="125"/>
+      <c r="E76" s="60"/>
+      <c r="F76" s="60"/>
+      <c r="G76" s="125"/>
+      <c r="H76" s="125"/>
+      <c r="I76" s="60"/>
+      <c r="J76" s="60"/>
+      <c r="K76" s="125"/>
+      <c r="L76" s="125"/>
+      <c r="M76" s="125"/>
+    </row>
+    <row r="77" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="126"/>
+      <c r="B77" s="126"/>
+      <c r="C77" s="126"/>
+      <c r="D77" s="126"/>
+      <c r="E77" s="60"/>
+      <c r="F77" s="60"/>
+      <c r="G77" s="126"/>
+      <c r="H77" s="126"/>
+      <c r="I77" s="60"/>
+      <c r="J77" s="60"/>
+      <c r="K77" s="126"/>
+      <c r="L77" s="126"/>
+      <c r="M77" s="126"/>
+    </row>
+    <row r="78" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="114"/>
+      <c r="B78" s="114"/>
+      <c r="C78" s="114"/>
+      <c r="D78" s="114"/>
+      <c r="E78" s="60"/>
+      <c r="F78" s="60"/>
+      <c r="G78" s="115" t="s">
         <v>27</v>
       </c>
-      <c r="H71" s="87"/>
-      <c r="I71" s="47"/>
-      <c r="J71" s="47"/>
-      <c r="K71" s="86"/>
-      <c r="L71" s="86"/>
-      <c r="M71" s="86"/>
-    </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A72" s="11"/>
-      <c r="B72" s="11"/>
-      <c r="C72" s="11"/>
-      <c r="D72" s="11"/>
-      <c r="E72" s="11"/>
-      <c r="F72" s="11"/>
-      <c r="G72" s="11"/>
-      <c r="H72" s="11"/>
-      <c r="I72" s="11"/>
-      <c r="J72" s="11"/>
-      <c r="K72" s="11"/>
-      <c r="L72" s="11"/>
-      <c r="M72" s="11"/>
-    </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A73" s="12"/>
-      <c r="C73" s="31"/>
-      <c r="D73" s="31"/>
-      <c r="E73" s="31"/>
-      <c r="F73" s="31"/>
-      <c r="G73" s="31"/>
-      <c r="H73" s="31"/>
-      <c r="I73" s="31"/>
-      <c r="J73" s="31"/>
-    </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="F74" s="22" t="s">
+      <c r="H78" s="115"/>
+      <c r="I78" s="60"/>
+      <c r="J78" s="60"/>
+      <c r="K78" s="114"/>
+      <c r="L78" s="114"/>
+      <c r="M78" s="114"/>
+    </row>
+    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A79" s="11"/>
+      <c r="B79" s="11"/>
+      <c r="C79" s="11"/>
+      <c r="D79" s="11"/>
+      <c r="E79" s="11"/>
+      <c r="F79" s="11"/>
+      <c r="G79" s="11"/>
+      <c r="H79" s="11"/>
+      <c r="I79" s="11"/>
+      <c r="J79" s="11"/>
+      <c r="K79" s="11"/>
+      <c r="L79" s="11"/>
+      <c r="M79" s="11"/>
+    </row>
+    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A80" s="12"/>
+      <c r="C80" s="44"/>
+      <c r="D80" s="44"/>
+      <c r="E80" s="44"/>
+      <c r="F80" s="44"/>
+      <c r="G80" s="44"/>
+      <c r="H80" s="44"/>
+      <c r="I80" s="44"/>
+      <c r="J80" s="44"/>
+    </row>
+    <row r="81" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F81" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="G74" s="22"/>
-    </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.25"/>
+      <c r="G81" s="34"/>
+    </row>
+    <row r="82" spans="6:7" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="6:7" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="124">
-    <mergeCell ref="C49:M49"/>
+  <mergeCells count="132">
+    <mergeCell ref="C56:M56"/>
+    <mergeCell ref="C57:M57"/>
+    <mergeCell ref="C58:M58"/>
+    <mergeCell ref="C59:M59"/>
+    <mergeCell ref="C60:M60"/>
+    <mergeCell ref="C61:M61"/>
+    <mergeCell ref="C62:M62"/>
+    <mergeCell ref="C63:M63"/>
+    <mergeCell ref="C64:M64"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:G10"/>
     <mergeCell ref="C50:M50"/>
     <mergeCell ref="C51:M51"/>
     <mergeCell ref="C52:M52"/>
     <mergeCell ref="C53:M53"/>
     <mergeCell ref="C54:M54"/>
     <mergeCell ref="C55:M55"/>
-    <mergeCell ref="C56:M56"/>
-    <mergeCell ref="C57:M57"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="C43:M43"/>
-    <mergeCell ref="C44:M44"/>
-    <mergeCell ref="C45:M45"/>
-    <mergeCell ref="C46:M46"/>
-    <mergeCell ref="C47:M47"/>
-    <mergeCell ref="C48:M48"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="A7:A15"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:H4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="E13:M13"/>
-    <mergeCell ref="E14:M14"/>
-    <mergeCell ref="E15:M15"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="E10:M10"/>
-    <mergeCell ref="E11:M11"/>
-    <mergeCell ref="E12:M12"/>
-    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="C13:F13"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="A14:A22"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
     <mergeCell ref="B16:D16"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:H11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="E20:M20"/>
+    <mergeCell ref="E21:M21"/>
+    <mergeCell ref="E22:M22"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B18:D18"/>
-    <mergeCell ref="E16:M16"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="E17:M17"/>
     <mergeCell ref="E18:M18"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E19:M19"/>
+    <mergeCell ref="A23:A25"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="B24:D24"/>
-    <mergeCell ref="E22:M22"/>
+    <mergeCell ref="B25:D25"/>
     <mergeCell ref="E23:M23"/>
     <mergeCell ref="E24:M24"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="E25:M25"/>
     <mergeCell ref="B21:D21"/>
-    <mergeCell ref="E19:M19"/>
-    <mergeCell ref="E20:M20"/>
-    <mergeCell ref="E21:M21"/>
-    <mergeCell ref="M36:M37"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E29:M29"/>
+    <mergeCell ref="E30:M30"/>
+    <mergeCell ref="E31:M31"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B27:D27"/>
     <mergeCell ref="B28:D28"/>
+    <mergeCell ref="E26:M26"/>
+    <mergeCell ref="E27:M27"/>
+    <mergeCell ref="E28:M28"/>
+    <mergeCell ref="A8:M8"/>
+    <mergeCell ref="E14:M14"/>
+    <mergeCell ref="K11:M11"/>
+    <mergeCell ref="K12:M12"/>
+    <mergeCell ref="J13:M13"/>
+    <mergeCell ref="E15:M15"/>
+    <mergeCell ref="E16:M16"/>
+    <mergeCell ref="A78:D78"/>
+    <mergeCell ref="E78:F78"/>
+    <mergeCell ref="G78:H78"/>
+    <mergeCell ref="I78:J78"/>
+    <mergeCell ref="K78:M78"/>
+    <mergeCell ref="C67:M71"/>
+    <mergeCell ref="A72:D77"/>
+    <mergeCell ref="E72:F77"/>
+    <mergeCell ref="G72:H77"/>
+    <mergeCell ref="I72:J77"/>
+    <mergeCell ref="K72:M77"/>
+    <mergeCell ref="C65:M66"/>
+    <mergeCell ref="A55:B59"/>
+    <mergeCell ref="L45:M47"/>
+    <mergeCell ref="F43:G44"/>
+    <mergeCell ref="H43:I44"/>
+    <mergeCell ref="M43:M44"/>
+    <mergeCell ref="H45:K45"/>
+    <mergeCell ref="H46:K46"/>
+    <mergeCell ref="H47:K47"/>
+    <mergeCell ref="A42:M42"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="B43:E44"/>
+    <mergeCell ref="J43:L43"/>
+    <mergeCell ref="J44:L44"/>
+    <mergeCell ref="C9:M9"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="E35:M35"/>
+    <mergeCell ref="E36:M36"/>
+    <mergeCell ref="E37:M37"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="E32:M32"/>
+    <mergeCell ref="E33:M33"/>
+    <mergeCell ref="E34:M34"/>
     <mergeCell ref="B29:D29"/>
     <mergeCell ref="B30:D30"/>
-    <mergeCell ref="E28:M28"/>
-    <mergeCell ref="E29:M29"/>
-    <mergeCell ref="E30:M30"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="E25:M25"/>
-    <mergeCell ref="E26:M26"/>
-    <mergeCell ref="E27:M27"/>
-    <mergeCell ref="C2:M2"/>
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="E7:M7"/>
-    <mergeCell ref="K4:M4"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="J6:M6"/>
-    <mergeCell ref="E8:M8"/>
-    <mergeCell ref="E9:M9"/>
-    <mergeCell ref="A71:D71"/>
-    <mergeCell ref="E71:F71"/>
-    <mergeCell ref="G71:H71"/>
-    <mergeCell ref="I71:J71"/>
-    <mergeCell ref="K71:M71"/>
-    <mergeCell ref="C60:M64"/>
-    <mergeCell ref="A65:D70"/>
-    <mergeCell ref="E65:F70"/>
-    <mergeCell ref="G65:H70"/>
-    <mergeCell ref="I65:J70"/>
-    <mergeCell ref="K65:M70"/>
-    <mergeCell ref="C58:M59"/>
-    <mergeCell ref="A48:B52"/>
-    <mergeCell ref="L38:M40"/>
-    <mergeCell ref="F36:G37"/>
-    <mergeCell ref="H36:I37"/>
-    <mergeCell ref="F74:G74"/>
-    <mergeCell ref="A31:M33"/>
-    <mergeCell ref="A34:M34"/>
-    <mergeCell ref="A53:B57"/>
-    <mergeCell ref="A58:B59"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B1:K1"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="B5:K5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="B4:K4"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="F81:G81"/>
+    <mergeCell ref="A38:M40"/>
+    <mergeCell ref="A41:M41"/>
     <mergeCell ref="A60:B64"/>
-    <mergeCell ref="C73:J73"/>
-    <mergeCell ref="I3:M3"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="D41:M41"/>
-    <mergeCell ref="A42:M42"/>
-    <mergeCell ref="A43:B47"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="D38:G40"/>
-    <mergeCell ref="H38:K38"/>
-    <mergeCell ref="H39:K39"/>
-    <mergeCell ref="H40:K40"/>
-    <mergeCell ref="A35:M35"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="B36:E37"/>
-    <mergeCell ref="J36:L36"/>
-    <mergeCell ref="J37:L37"/>
+    <mergeCell ref="A65:B66"/>
+    <mergeCell ref="A67:B71"/>
+    <mergeCell ref="C80:J80"/>
+    <mergeCell ref="I10:M10"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="D48:M48"/>
+    <mergeCell ref="A49:M49"/>
+    <mergeCell ref="A50:B54"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="D45:G47"/>
   </mergeCells>
-  <conditionalFormatting sqref="A71:D71">
+  <conditionalFormatting sqref="A78:D78">
     <cfRule type="containsBlanks" dxfId="3" priority="2">
-      <formula>LEN(TRIM(A71))=0</formula>
+      <formula>LEN(TRIM(A78))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C73">
+  <conditionalFormatting sqref="C80">
     <cfRule type="containsBlanks" dxfId="2" priority="3">
-      <formula>LEN(TRIM(C73))=0</formula>
+      <formula>LEN(TRIM(C80))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:M3 C4:H4 K4:M4 J6:M6 E7:M15 E19:M30 B36:E37 H36:I37 M36:M37 D38:G40 L38:M40 D41:M41 C43:C57 C58:M64">
+  <conditionalFormatting sqref="I10:M10 C11:H11 K11:M11 J13:M13 E14:M22 E26:M37 B43:E44 H43:I44 M43:M44 D45:G47 L45:M47 C50:C64 C65:M71">
     <cfRule type="containsBlanks" dxfId="1" priority="4">
-      <formula>LEN(TRIM(B3))=0</formula>
+      <formula>LEN(TRIM(B10))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K71:M71">
+  <conditionalFormatting sqref="K78:M78">
     <cfRule type="containsBlanks" dxfId="0" priority="1">
-      <formula>LEN(TRIM(K71))=0</formula>
+      <formula>LEN(TRIM(K78))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="36">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar el nivel formativo en el cual se encuentra el aprendiz. Técnio o Tecnólogo" sqref="I3:M3" xr:uid="{FDFD4240-B4E4-40FA-8880-3E4E045C5084}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Número Ficha" prompt="Registre el número de ficha en el que se encuentra matriculado según el programa de formación." sqref="K4:M4" xr:uid="{C295E52F-E427-4103-89DB-18FF195E95C6}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Fin Etapa Lectiva" prompt="Registrar la fecha de culminación de la etapa lectiva del aprendiz." sqref="J6:M6" xr:uid="{5EB3E1EF-1E32-4E95-8D18-C01EA7CF4F61}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar nombre del aprendiz como aparece en su documento de identificación." sqref="E7:M7" xr:uid="{9B40B093-9C34-4E63-9F64-4BFF88393B31}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Tipo Documento Identificación" prompt="Este tipo de documento debe coincidir con las opciones de identificación descritas en el aplicativo Sofia Plus (NUIP, TI, CC, CE, PEP). " sqref="E8:M8" xr:uid="{DA947DA3-FB5C-4D1A-942B-8548E48311E3}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el número de identificación del aprendiz SIN puntos, comas o espacios" sqref="E9:M9" xr:uid="{26796309-EF62-4852-B260-C64A329B6E61}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar teléfonos fijo y celular del aprendiz u otro número de contacto." sqref="E10:M10" xr:uid="{227D64D5-7E2E-48B5-834F-26D52CA83B47}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingrese la dirección residencial actual de correspondencia del aprendiz." sqref="E11:M11" xr:uid="{EC33A478-21D0-417A-960A-07B663B862B0}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el correo electrónico personal del aprendiz" sqref="E12:M12" xr:uid="{CEDF05F3-A498-464C-AF78-C83490E95D67}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el correo electrónico institucional del aprendiz @sena.edu.co , @soysena.edu.co" sqref="E13:M13" xr:uid="{8AC0CC91-D06D-4D82-A06B-CEDFF66185FC}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el nombre de la alternativa de etapa productiva, de acuerdo con las alternativas descritas en el reglamento del aprendiz vigente" sqref="E14:M14" xr:uid="{48CA359C-CBBE-4B45-B681-EA4693D12177}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar la fecha en que quedó registrada la alternativa en el aplicativo SofiaPlus.  Gestione con la coordinación académica el reporte del SVP para obtener la información requerida en este apartado" sqref="E15:M15" xr:uid="{A4B53DE5-4CEE-4C8C-A08B-9C6344C18954}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el nombre completo de la empresa o entidad co-formadora (empresa, entidad o institución gubernamental o no gubernamental)." sqref="E19:M19" xr:uid="{35AC5BC6-659F-4E4C-B567-3C3F16C509BD}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar la dirección de la empresa, entidad o institución gubernamental o no gubernamental." sqref="E20:M20" xr:uid="{18FD205E-10DD-4EB5-8E57-F8B0C00BF5BC}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el numero NIT de la empresa, entidad o institución gubernamental o no gubernamental." sqref="E21:M21" xr:uid="{0E9499EA-A21D-4209-94F0-6561C0BEA458}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el correo organizacional o institucional del jefe inmediato." sqref="E22:M22" xr:uid="{F7B09C4A-6282-4561-9C6E-128034419E72}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el nombre del jefe inmediato o quien va a supervisar las actividades del aprendiz en la empresa. En caso de estar participando en una convocatoria de proyecto productivo, aquí se registran los datos del instructor de proyecto productivo." sqref="E23:M23" xr:uid="{3F1EE247-C76F-4BD4-A0A3-6B6F02F83B03}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el cargo del jefe inmediato dentro de la empresa" sqref="E24:M24" xr:uid="{44C4A18A-BD9D-4153-94CA-F617EBC7DCBA}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el número del celular del jefe inmediato o supervisor y el número fijo de la empresa con extensión" sqref="E25:M25" xr:uid="{D17896B5-5299-404D-BF06-0A7409E6BB11}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="En caso de que aplique, registrar el nombre de otro contacto en la empresa. De no tener digitar N/A" sqref="E26:M26" xr:uid="{A6F4976B-257F-4E38-96A4-122163F2BCDA}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el teléfono institucional al cual contactarse en caso que el ente coformador no responda" sqref="E27:M27" xr:uid="{A593241B-15E7-4EA6-B9DE-E0DF01ED6DB9}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="En caso de que el aprendiz sea una persona en situación de discapacidad, diligencie este espacio con el nombre de la persona que le asiste." sqref="E28:M28" xr:uid="{C19946D2-B571-4104-A1EA-FEF5A7253596}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Aquí se especifica el tipo de asistencia brindada al aprendiz para que desempeñe la totalidad de sus tareas asegurando un ambiente laboral inclusivo adecuado a sus necesidades. Puede incluir asistencias como lenguaje de señas, soporte visual etc" sqref="E29:M29" xr:uid="{B635F5F5-108B-409C-BCAD-0AA5A654CF02}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el número del celular de la persona que asiste al aprendiz " sqref="E30:M30" xr:uid="{77AEF51E-4966-4ADA-B94D-7E72C6BE4FFA}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar la fecha Inicial de ejecución de la etapa productiva del aprendiz,  La cual se encuentra registrada en el sistema de gestión académico administrativo" sqref="B36:E37" xr:uid="{ADDD56B1-A1AE-4F35-A152-F9DAB746A3F8}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar la fecha fin de ejecución de la etapa productiva del aprendiz,  La cual se encuentra registrada en el sistema de gestión académico administrativo" sqref="H36:I37" xr:uid="{A2994507-EBC1-4758-8D2D-041DB7D68E81}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar la fecha de afiliación en la ARL realizada por el centro de formación o la empresa, solo aplica para aprendices que se encuentren en Colombia." sqref="M36:M37" xr:uid="{0E74721C-02A8-4123-BB25-E650EFDE799B}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar el número de póliza que se registra en la ARL." sqref="D38:G40" xr:uid="{AEDBE09E-E16B-4102-8DD1-046357FA9976}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el horario en el cual el aprendiz ejecutará su etapa productiva." sqref="L38:M40" xr:uid="{22678B76-AB93-48B7-B0CA-9F11DDE08012}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Adjuntar enlace de grabacion de la sesion, el enlace le llaga al aprendiz por correo de la citacion." sqref="D41:M41" xr:uid="{81EA4BA8-6491-4C84-9D5E-95D4DAC042D4}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Relacione las actividades que el aprendiz va a realizar según lo acordado. (Estas deben corresponder al perfil del egresado establecido en el programa de formación que el aprendiz está desarrollando.) redactar activ. en  verbos en infinitivo" sqref="C53:C57" xr:uid="{765A44AD-7EE4-4C8A-82B9-AEB337B3CBFF}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Describa las evidencias o entregables que se van a generar de acuerdo con las actividades a desarrollar. En este apartado adicionalmente, es importante definir si dichas evidencias serán entregadas de manera digital o física. " sqref="C58:M59" xr:uid="{6D49D6E6-6363-4D06-90B1-78A757068CEE}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registre los comentarios que considere pertinentes en relación a la visita correspondiente. " sqref="C60:M64" xr:uid="{08D354B0-14A2-4554-94A3-2633D73D772A}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el nombre completo del aprendiz y en la parte superior la Firma manuscrita o digital." sqref="A71:D71" xr:uid="{A7FEFB2B-7370-4FA2-8820-7EB89B730FD1}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el nombre completo del co-formador y en la parte superior de esta la Firma manuscrita o digital." sqref="K71:M71" xr:uid="{DAE2A968-2309-42D5-952C-BC599D7BE50F}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Diligenciar fecha de la sesión en este espacio. Ejemplo: Bogotá dia/mes/año Virtual" sqref="C73:J73" xr:uid="{201095D8-80DA-45BB-84F9-D066E44DB3C5}"/>
+  <dataValidations xWindow="828" yWindow="713" count="36">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar el nivel formativo en el cual se encuentra el aprendiz. Técnio o Tecnólogo" sqref="I10:M10" xr:uid="{FDFD4240-B4E4-40FA-8880-3E4E045C5084}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Número Ficha" prompt="Registre el número de ficha en el que se encuentra matriculado según el programa de formación." sqref="K11:M11" xr:uid="{C295E52F-E427-4103-89DB-18FF195E95C6}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Fin Etapa Lectiva" prompt="Registrar la fecha de culminación de la etapa lectiva del aprendiz." sqref="J13:M13" xr:uid="{5EB3E1EF-1E32-4E95-8D18-C01EA7CF4F61}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar nombre del aprendiz como aparece en su documento de identificación." sqref="E14:M14" xr:uid="{9B40B093-9C34-4E63-9F64-4BFF88393B31}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Tipo Documento Identificación" prompt="Este tipo de documento debe coincidir con las opciones de identificación descritas en el aplicativo Sofia Plus (NUIP, TI, CC, CE, PEP). " sqref="E15:M15" xr:uid="{DA947DA3-FB5C-4D1A-942B-8548E48311E3}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el número de identificación del aprendiz SIN puntos, comas o espacios" sqref="E16:M16" xr:uid="{26796309-EF62-4852-B260-C64A329B6E61}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar teléfonos fijo y celular del aprendiz u otro número de contacto." sqref="E17:M17" xr:uid="{227D64D5-7E2E-48B5-834F-26D52CA83B47}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingrese la dirección residencial actual de correspondencia del aprendiz." sqref="E18:M18" xr:uid="{EC33A478-21D0-417A-960A-07B663B862B0}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el correo electrónico personal del aprendiz" sqref="E19:M19" xr:uid="{CEDF05F3-A498-464C-AF78-C83490E95D67}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el correo electrónico institucional del aprendiz @sena.edu.co , @soysena.edu.co" sqref="E20:M20" xr:uid="{8AC0CC91-D06D-4D82-A06B-CEDFF66185FC}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el nombre de la alternativa de etapa productiva, de acuerdo con las alternativas descritas en el reglamento del aprendiz vigente" sqref="E21:M21" xr:uid="{48CA359C-CBBE-4B45-B681-EA4693D12177}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar la fecha en que quedó registrada la alternativa en el aplicativo SofiaPlus.  Gestione con la coordinación académica el reporte del SVP para obtener la información requerida en este apartado" sqref="E22:M22" xr:uid="{A4B53DE5-4CEE-4C8C-A08B-9C6344C18954}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el nombre completo de la empresa o entidad co-formadora (empresa, entidad o institución gubernamental o no gubernamental)." sqref="E26:M26" xr:uid="{35AC5BC6-659F-4E4C-B567-3C3F16C509BD}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar la dirección de la empresa, entidad o institución gubernamental o no gubernamental." sqref="E27:M27" xr:uid="{18FD205E-10DD-4EB5-8E57-F8B0C00BF5BC}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el numero NIT de la empresa, entidad o institución gubernamental o no gubernamental." sqref="E28:M28" xr:uid="{0E9499EA-A21D-4209-94F0-6561C0BEA458}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el correo organizacional o institucional del jefe inmediato." sqref="E29:M29" xr:uid="{F7B09C4A-6282-4561-9C6E-128034419E72}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el nombre del jefe inmediato o quien va a supervisar las actividades del aprendiz en la empresa. En caso de estar participando en una convocatoria de proyecto productivo, aquí se registran los datos del instructor de proyecto productivo." sqref="E30:M30" xr:uid="{3F1EE247-C76F-4BD4-A0A3-6B6F02F83B03}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el cargo del jefe inmediato dentro de la empresa" sqref="E31:M31" xr:uid="{44C4A18A-BD9D-4153-94CA-F617EBC7DCBA}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el número del celular del jefe inmediato o supervisor y el número fijo de la empresa con extensión" sqref="E32:M32" xr:uid="{D17896B5-5299-404D-BF06-0A7409E6BB11}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="En caso de que aplique, registrar el nombre de otro contacto en la empresa. De no tener digitar N/A" sqref="E33:M33" xr:uid="{A6F4976B-257F-4E38-96A4-122163F2BCDA}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el teléfono institucional al cual contactarse en caso que el ente coformador no responda" sqref="E34:M34" xr:uid="{A593241B-15E7-4EA6-B9DE-E0DF01ED6DB9}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="En caso de que el aprendiz sea una persona en situación de discapacidad, diligencie este espacio con el nombre de la persona que le asiste." sqref="E35:M35" xr:uid="{C19946D2-B571-4104-A1EA-FEF5A7253596}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Aquí se especifica el tipo de asistencia brindada al aprendiz para que desempeñe la totalidad de sus tareas asegurando un ambiente laboral inclusivo adecuado a sus necesidades. Puede incluir asistencias como lenguaje de señas, soporte visual etc" sqref="E36:M36" xr:uid="{B635F5F5-108B-409C-BCAD-0AA5A654CF02}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el número del celular de la persona que asiste al aprendiz " sqref="E37:M37" xr:uid="{77AEF51E-4966-4ADA-B94D-7E72C6BE4FFA}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar la fecha Inicial de ejecución de la etapa productiva del aprendiz,  La cual se encuentra registrada en el sistema de gestión académico administrativo" sqref="B43:E44" xr:uid="{ADDD56B1-A1AE-4F35-A152-F9DAB746A3F8}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar la fecha fin de ejecución de la etapa productiva del aprendiz,  La cual se encuentra registrada en el sistema de gestión académico administrativo" sqref="H43:I44" xr:uid="{A2994507-EBC1-4758-8D2D-041DB7D68E81}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar la fecha de afiliación en la ARL realizada por el centro de formación o la empresa, solo aplica para aprendices que se encuentren en Colombia." sqref="M43:M44" xr:uid="{0E74721C-02A8-4123-BB25-E650EFDE799B}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar el número de póliza que se registra en la ARL." sqref="D45:G47" xr:uid="{AEDBE09E-E16B-4102-8DD1-046357FA9976}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el horario en el cual el aprendiz ejecutará su etapa productiva." sqref="L45:M47" xr:uid="{22678B76-AB93-48B7-B0CA-9F11DDE08012}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Adjuntar enlace de grabacion de la sesion, el enlace le llaga al aprendiz por correo de la citacion." sqref="D48:M48" xr:uid="{81EA4BA8-6491-4C84-9D5E-95D4DAC042D4}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Relacione las actividades que el aprendiz va a realizar según lo acordado. (Estas deben corresponder al perfil del egresado establecido en el programa de formación que el aprendiz está desarrollando.) redactar activ. en  verbos en infinitivo" sqref="C60:C64" xr:uid="{765A44AD-7EE4-4C8A-82B9-AEB337B3CBFF}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Describa las evidencias o entregables que se van a generar de acuerdo con las actividades a desarrollar. En este apartado adicionalmente, es importante definir si dichas evidencias serán entregadas de manera digital o física. " sqref="C65:M66" xr:uid="{6D49D6E6-6363-4D06-90B1-78A757068CEE}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registre los comentarios que considere pertinentes en relación a la visita correspondiente. " sqref="C67:M71" xr:uid="{08D354B0-14A2-4554-94A3-2633D73D772A}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el nombre completo del aprendiz y en la parte superior la Firma manuscrita o digital." sqref="A78:D78" xr:uid="{A7FEFB2B-7370-4FA2-8820-7EB89B730FD1}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el nombre completo del co-formador y en la parte superior de esta la Firma manuscrita o digital." sqref="K78:M78" xr:uid="{DAE2A968-2309-42D5-952C-BC599D7BE50F}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Diligenciar fecha de la sesión en este espacio. Ejemplo: Bogotá dia/mes/año Virtual" sqref="C80:J80" xr:uid="{201095D8-80DA-45BB-84F9-D066E44DB3C5}"/>
   </dataValidations>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" scale="68" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="7">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xWindow="828" yWindow="713" count="7">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Seleccionael nombre del programa" prompt="Elige el programa de la lista desplegable" xr:uid="{34EF5BAD-650F-4FA7-AB25-B4A5694BB4C0}">
           <x14:formula1>
             <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$E$2)</xm:f>
           </x14:formula1>
-          <xm:sqref>C4:H4</xm:sqref>
+          <xm:sqref>C11:H11</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Selecciona del listado las competencias tecnicas que se van a desarrollar a lo largo de la etapa productiva. minimo 3" xr:uid="{22B88745-2B8F-40B6-8916-320FA089DFCF}">
           <x14:formula1>
             <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$F$2)</xm:f>
           </x14:formula1>
-          <xm:sqref>C43:M47</xm:sqref>
+          <xm:sqref>C50:M54</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Relacione el o los resultados de aprendizaje de las competencias que van a desarrollarse." xr:uid="{1DCCDD3C-B075-4833-878D-65AC808D9E9F}">
           <x14:formula1>
             <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$G$2)</xm:f>
           </x14:formula1>
-          <xm:sqref>C48:M48</xm:sqref>
+          <xm:sqref>C55:M55</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Relacione el o los resultados de aprendizaje de las competencias que van a desarrollarse." xr:uid="{934278D6-6E18-4E97-BCEF-064F63567755}">
           <x14:formula1>
             <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$H$2)</xm:f>
           </x14:formula1>
-          <xm:sqref>C49:M49</xm:sqref>
+          <xm:sqref>C56:M56</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Relacione el o los resultados de aprendizaje de las competencias que van a desarrollarse." xr:uid="{0CE56376-096C-4566-B3AF-5321973F5724}">
           <x14:formula1>
             <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$I$2)</xm:f>
           </x14:formula1>
-          <xm:sqref>C50:M50</xm:sqref>
+          <xm:sqref>C57:M57</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Relacione el o los resultados de aprendizaje de las competencias que van a desarrollarse." xr:uid="{DD57E66E-4FD0-4B6F-8647-729A07AB846F}">
           <x14:formula1>
             <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$J$2)</xm:f>
           </x14:formula1>
-          <xm:sqref>C51:M51</xm:sqref>
+          <xm:sqref>C58:M58</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Relacione el o los resultados de aprendizaje de las competencias que van a desarrollarse." xr:uid="{8550080C-D284-4509-8ED8-32A50ECC2F74}">
           <x14:formula1>
             <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$K$2)</xm:f>
           </x14:formula1>
-          <xm:sqref>C52:M52</xm:sqref>
+          <xm:sqref>C59:M59</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3777,27 +4084,27 @@
         <v>Análisis y Desarrollo de Software</v>
       </c>
       <c r="F2" t="str" cm="1">
-        <f t="array" ref="F2">_xlfn.UNIQUE(_xlfn._xlws.FILTER(TablaSena[COMPETENCIA], TablaSena[PROGRAMA]='Formato Visita 1'!$C$4, "Seleccione Programa"))</f>
+        <f t="array" ref="F2">_xlfn.UNIQUE(_xlfn._xlws.FILTER(TablaSena[COMPETENCIA], TablaSena[PROGRAMA]='Formato Visita 1'!$C$11, "Seleccione Programa"))</f>
         <v>Seleccione Programa</v>
       </c>
       <c r="G2" t="str" cm="1">
-        <f t="array" ref="G2">_xlfn._xlws.FILTER(TablaSena[RESULTADO DE APRENDIZAJE (RAP)], TablaSena[COMPETENCIA]='Formato Visita 1'!$C$43, "...")</f>
+        <f t="array" ref="G2">_xlfn._xlws.FILTER(TablaSena[RESULTADO DE APRENDIZAJE (RAP)], TablaSena[COMPETENCIA]='Formato Visita 1'!$C$50, "...")</f>
         <v>...</v>
       </c>
       <c r="H2" t="str" cm="1">
-        <f t="array" ref="H2">_xlfn._xlws.FILTER(TablaSena[RESULTADO DE APRENDIZAJE (RAP)], TablaSena[COMPETENCIA]='Formato Visita 1'!$C$44, "...")</f>
+        <f t="array" ref="H2">_xlfn._xlws.FILTER(TablaSena[RESULTADO DE APRENDIZAJE (RAP)], TablaSena[COMPETENCIA]='Formato Visita 1'!$C$51, "...")</f>
         <v>...</v>
       </c>
       <c r="I2" t="str" cm="1">
-        <f t="array" ref="I2">_xlfn._xlws.FILTER(TablaSena[RESULTADO DE APRENDIZAJE (RAP)], TablaSena[COMPETENCIA]='Formato Visita 1'!$C$45, "...")</f>
+        <f t="array" ref="I2">_xlfn._xlws.FILTER(TablaSena[RESULTADO DE APRENDIZAJE (RAP)], TablaSena[COMPETENCIA]='Formato Visita 1'!$C$52, "...")</f>
         <v>...</v>
       </c>
       <c r="J2" t="str" cm="1">
-        <f t="array" ref="J2">_xlfn._xlws.FILTER(TablaSena[RESULTADO DE APRENDIZAJE (RAP)], TablaSena[COMPETENCIA]='Formato Visita 1'!$C$46, "...")</f>
+        <f t="array" ref="J2">_xlfn._xlws.FILTER(TablaSena[RESULTADO DE APRENDIZAJE (RAP)], TablaSena[COMPETENCIA]='Formato Visita 1'!$C$53, "...")</f>
         <v>...</v>
       </c>
       <c r="K2" t="str" cm="1">
-        <f t="array" ref="K2">_xlfn._xlws.FILTER(TablaSena[RESULTADO DE APRENDIZAJE (RAP)], TablaSena[COMPETENCIA]='Formato Visita 1'!$C$47, "...")</f>
+        <f t="array" ref="K2">_xlfn._xlws.FILTER(TablaSena[RESULTADO DE APRENDIZAJE (RAP)], TablaSena[COMPETENCIA]='Formato Visita 1'!$C$54, "...")</f>
         <v>...</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar formatos GFPI-F023 visitas 1 a 3
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Formatos/Visita 1 GFPI-F023.xlsx
+++ b/Formatos/Visita 1 GFPI-F023.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/834af06e427efe68/Documents/Seto 2026/sena/Manual SENA Etapa Productiva/manual-aprendiz-sena/Formatos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SEANT\3D Objects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="13_ncr:1_{DD5881F2-7753-446A-8E5F-805A07B66FFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AABE3BCB-E6DC-438F-AF45-0DB4F9E7EE49}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9057EC18-0F9F-4B95-BC58-7A90354B991C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BC3553EE-4E49-4F2A-B03E-CFAC4EB3009B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BC3553EE-4E49-4F2A-B03E-CFAC4EB3009B}"/>
   </bookViews>
   <sheets>
     <sheet name="Formato Visita 1" sheetId="1" r:id="rId1"/>
@@ -1615,24 +1615,63 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -1777,45 +1816,6 @@
     <xf numFmtId="15" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2121,10 +2121,6 @@
     </a>
   </bag>
 </FeaturePropertyBags>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2569,27 +2565,27 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25"/>
     <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="97" t="s">
+      <c r="A8" s="112" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="98"/>
-      <c r="C8" s="98"/>
-      <c r="D8" s="98"/>
-      <c r="E8" s="98"/>
-      <c r="F8" s="98"/>
-      <c r="G8" s="98"/>
-      <c r="H8" s="98"/>
-      <c r="I8" s="98"/>
-      <c r="J8" s="98"/>
-      <c r="K8" s="98"/>
-      <c r="L8" s="98"/>
-      <c r="M8" s="98"/>
+      <c r="B8" s="113"/>
+      <c r="C8" s="113"/>
+      <c r="D8" s="113"/>
+      <c r="E8" s="113"/>
+      <c r="F8" s="113"/>
+      <c r="G8" s="113"/>
+      <c r="H8" s="113"/>
+      <c r="I8" s="113"/>
+      <c r="J8" s="113"/>
+      <c r="K8" s="113"/>
+      <c r="L8" s="113"/>
+      <c r="M8" s="113"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="143" t="s">
+      <c r="A9" s="100" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="145"/>
+      <c r="B9" s="102"/>
       <c r="C9" s="94" t="s">
         <v>2</v>
       </c>
@@ -2605,10 +2601,10 @@
       <c r="M9" s="96"/>
     </row>
     <row r="10" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="143" t="s">
+      <c r="A10" s="100" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="145"/>
+      <c r="B10" s="102"/>
       <c r="C10" s="161" t="s">
         <v>4</v>
       </c>
@@ -2626,10 +2622,10 @@
       <c r="M10" s="47"/>
     </row>
     <row r="11" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="143" t="s">
+      <c r="A11" s="100" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="145"/>
+      <c r="B11" s="102"/>
       <c r="C11" s="173"/>
       <c r="D11" s="174"/>
       <c r="E11" s="174"/>
@@ -2640,15 +2636,15 @@
         <v>7</v>
       </c>
       <c r="J11" s="43"/>
-      <c r="K11" s="102"/>
-      <c r="L11" s="103"/>
-      <c r="M11" s="104"/>
+      <c r="K11" s="114"/>
+      <c r="L11" s="115"/>
+      <c r="M11" s="116"/>
     </row>
     <row r="12" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="143" t="s">
+      <c r="A12" s="100" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="145"/>
+      <c r="B12" s="102"/>
       <c r="C12" s="2" t="s">
         <v>9</v>
       </c>
@@ -2665,15 +2661,15 @@
         <v>12</v>
       </c>
       <c r="J12" s="177"/>
-      <c r="K12" s="105"/>
-      <c r="L12" s="106"/>
-      <c r="M12" s="107"/>
+      <c r="K12" s="117"/>
+      <c r="L12" s="118"/>
+      <c r="M12" s="119"/>
     </row>
     <row r="13" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="143" t="s">
+      <c r="A13" s="100" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="145"/>
+      <c r="B13" s="102"/>
       <c r="C13" s="166"/>
       <c r="D13" s="167"/>
       <c r="E13" s="167"/>
@@ -2683,29 +2679,29 @@
       </c>
       <c r="H13" s="167"/>
       <c r="I13" s="168"/>
-      <c r="J13" s="108"/>
-      <c r="K13" s="109"/>
-      <c r="L13" s="109"/>
-      <c r="M13" s="110"/>
+      <c r="J13" s="120"/>
+      <c r="K13" s="121"/>
+      <c r="L13" s="121"/>
+      <c r="M13" s="122"/>
     </row>
     <row r="14" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="169" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="143" t="s">
+      <c r="B14" s="100" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="144"/>
-      <c r="D14" s="145"/>
-      <c r="E14" s="99"/>
-      <c r="F14" s="100"/>
-      <c r="G14" s="100"/>
-      <c r="H14" s="100"/>
-      <c r="I14" s="100"/>
-      <c r="J14" s="100"/>
-      <c r="K14" s="100"/>
-      <c r="L14" s="100"/>
-      <c r="M14" s="101"/>
+      <c r="C14" s="101"/>
+      <c r="D14" s="102"/>
+      <c r="E14" s="109"/>
+      <c r="F14" s="110"/>
+      <c r="G14" s="110"/>
+      <c r="H14" s="110"/>
+      <c r="I14" s="110"/>
+      <c r="J14" s="110"/>
+      <c r="K14" s="110"/>
+      <c r="L14" s="110"/>
+      <c r="M14" s="111"/>
     </row>
     <row r="15" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="153"/>
@@ -2714,144 +2710,144 @@
       </c>
       <c r="C15" s="171"/>
       <c r="D15" s="172"/>
-      <c r="E15" s="111"/>
-      <c r="F15" s="112"/>
-      <c r="G15" s="112"/>
-      <c r="H15" s="112"/>
-      <c r="I15" s="112"/>
-      <c r="J15" s="112"/>
-      <c r="K15" s="112"/>
-      <c r="L15" s="112"/>
-      <c r="M15" s="113"/>
+      <c r="E15" s="123"/>
+      <c r="F15" s="124"/>
+      <c r="G15" s="124"/>
+      <c r="H15" s="124"/>
+      <c r="I15" s="124"/>
+      <c r="J15" s="124"/>
+      <c r="K15" s="124"/>
+      <c r="L15" s="124"/>
+      <c r="M15" s="125"/>
     </row>
     <row r="16" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="153"/>
-      <c r="B16" s="143" t="s">
+      <c r="B16" s="100" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="144"/>
-      <c r="D16" s="145"/>
-      <c r="E16" s="99"/>
-      <c r="F16" s="100"/>
-      <c r="G16" s="100"/>
-      <c r="H16" s="100"/>
-      <c r="I16" s="100"/>
-      <c r="J16" s="100"/>
-      <c r="K16" s="100"/>
-      <c r="L16" s="100"/>
-      <c r="M16" s="101"/>
+      <c r="C16" s="101"/>
+      <c r="D16" s="102"/>
+      <c r="E16" s="109"/>
+      <c r="F16" s="110"/>
+      <c r="G16" s="110"/>
+      <c r="H16" s="110"/>
+      <c r="I16" s="110"/>
+      <c r="J16" s="110"/>
+      <c r="K16" s="110"/>
+      <c r="L16" s="110"/>
+      <c r="M16" s="111"/>
     </row>
     <row r="17" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="153"/>
-      <c r="B17" s="143" t="s">
+      <c r="B17" s="100" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="144"/>
-      <c r="D17" s="145"/>
-      <c r="E17" s="99"/>
-      <c r="F17" s="100"/>
-      <c r="G17" s="100"/>
-      <c r="H17" s="100"/>
-      <c r="I17" s="100"/>
-      <c r="J17" s="100"/>
-      <c r="K17" s="100"/>
-      <c r="L17" s="100"/>
-      <c r="M17" s="101"/>
+      <c r="C17" s="101"/>
+      <c r="D17" s="102"/>
+      <c r="E17" s="109"/>
+      <c r="F17" s="110"/>
+      <c r="G17" s="110"/>
+      <c r="H17" s="110"/>
+      <c r="I17" s="110"/>
+      <c r="J17" s="110"/>
+      <c r="K17" s="110"/>
+      <c r="L17" s="110"/>
+      <c r="M17" s="111"/>
     </row>
     <row r="18" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="153"/>
-      <c r="B18" s="143" t="s">
+      <c r="B18" s="100" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="144"/>
-      <c r="D18" s="145"/>
-      <c r="E18" s="99"/>
-      <c r="F18" s="100"/>
-      <c r="G18" s="100"/>
-      <c r="H18" s="100"/>
-      <c r="I18" s="100"/>
-      <c r="J18" s="100"/>
-      <c r="K18" s="100"/>
-      <c r="L18" s="100"/>
-      <c r="M18" s="101"/>
+      <c r="C18" s="101"/>
+      <c r="D18" s="102"/>
+      <c r="E18" s="109"/>
+      <c r="F18" s="110"/>
+      <c r="G18" s="110"/>
+      <c r="H18" s="110"/>
+      <c r="I18" s="110"/>
+      <c r="J18" s="110"/>
+      <c r="K18" s="110"/>
+      <c r="L18" s="110"/>
+      <c r="M18" s="111"/>
     </row>
     <row r="19" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="153"/>
-      <c r="B19" s="143" t="s">
+      <c r="B19" s="100" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="144"/>
-      <c r="D19" s="145"/>
-      <c r="E19" s="99"/>
-      <c r="F19" s="100"/>
-      <c r="G19" s="100"/>
-      <c r="H19" s="100"/>
-      <c r="I19" s="100"/>
-      <c r="J19" s="100"/>
-      <c r="K19" s="100"/>
-      <c r="L19" s="100"/>
-      <c r="M19" s="101"/>
+      <c r="C19" s="101"/>
+      <c r="D19" s="102"/>
+      <c r="E19" s="109"/>
+      <c r="F19" s="110"/>
+      <c r="G19" s="110"/>
+      <c r="H19" s="110"/>
+      <c r="I19" s="110"/>
+      <c r="J19" s="110"/>
+      <c r="K19" s="110"/>
+      <c r="L19" s="110"/>
+      <c r="M19" s="111"/>
     </row>
     <row r="20" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="153"/>
-      <c r="B20" s="143" t="s">
+      <c r="B20" s="100" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="144"/>
-      <c r="D20" s="145"/>
-      <c r="E20" s="146"/>
-      <c r="F20" s="147"/>
-      <c r="G20" s="147"/>
-      <c r="H20" s="147"/>
-      <c r="I20" s="147"/>
-      <c r="J20" s="147"/>
-      <c r="K20" s="147"/>
-      <c r="L20" s="147"/>
-      <c r="M20" s="148"/>
+      <c r="C20" s="101"/>
+      <c r="D20" s="102"/>
+      <c r="E20" s="103"/>
+      <c r="F20" s="104"/>
+      <c r="G20" s="104"/>
+      <c r="H20" s="104"/>
+      <c r="I20" s="104"/>
+      <c r="J20" s="104"/>
+      <c r="K20" s="104"/>
+      <c r="L20" s="104"/>
+      <c r="M20" s="105"/>
     </row>
     <row r="21" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="153"/>
-      <c r="B21" s="143" t="s">
+      <c r="B21" s="100" t="s">
         <v>23</v>
       </c>
-      <c r="C21" s="144"/>
-      <c r="D21" s="145"/>
-      <c r="E21" s="146"/>
-      <c r="F21" s="147"/>
-      <c r="G21" s="147"/>
-      <c r="H21" s="147"/>
-      <c r="I21" s="147"/>
-      <c r="J21" s="147"/>
-      <c r="K21" s="147"/>
-      <c r="L21" s="147"/>
-      <c r="M21" s="148"/>
+      <c r="C21" s="101"/>
+      <c r="D21" s="102"/>
+      <c r="E21" s="103"/>
+      <c r="F21" s="104"/>
+      <c r="G21" s="104"/>
+      <c r="H21" s="104"/>
+      <c r="I21" s="104"/>
+      <c r="J21" s="104"/>
+      <c r="K21" s="104"/>
+      <c r="L21" s="104"/>
+      <c r="M21" s="105"/>
     </row>
     <row r="22" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="154"/>
-      <c r="B22" s="143" t="s">
+      <c r="B22" s="100" t="s">
         <v>24</v>
       </c>
-      <c r="C22" s="144"/>
-      <c r="D22" s="145"/>
-      <c r="E22" s="146"/>
-      <c r="F22" s="147"/>
-      <c r="G22" s="147"/>
-      <c r="H22" s="147"/>
-      <c r="I22" s="147"/>
-      <c r="J22" s="147"/>
-      <c r="K22" s="147"/>
-      <c r="L22" s="147"/>
-      <c r="M22" s="148"/>
+      <c r="C22" s="101"/>
+      <c r="D22" s="102"/>
+      <c r="E22" s="103"/>
+      <c r="F22" s="104"/>
+      <c r="G22" s="104"/>
+      <c r="H22" s="104"/>
+      <c r="I22" s="104"/>
+      <c r="J22" s="104"/>
+      <c r="K22" s="104"/>
+      <c r="L22" s="104"/>
+      <c r="M22" s="105"/>
     </row>
     <row r="23" spans="1:13" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="152" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="143" t="s">
+      <c r="B23" s="100" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="144"/>
-      <c r="D23" s="145"/>
+      <c r="C23" s="101"/>
+      <c r="D23" s="102"/>
       <c r="E23" s="155" t="s">
         <v>27</v>
       </c>
@@ -2866,11 +2862,11 @@
     </row>
     <row r="24" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="153"/>
-      <c r="B24" s="143" t="s">
+      <c r="B24" s="100" t="s">
         <v>19</v>
       </c>
-      <c r="C24" s="144"/>
-      <c r="D24" s="145"/>
+      <c r="C24" s="101"/>
+      <c r="D24" s="102"/>
       <c r="E24" s="158"/>
       <c r="F24" s="159"/>
       <c r="G24" s="159"/>
@@ -2883,11 +2879,11 @@
     </row>
     <row r="25" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="154"/>
-      <c r="B25" s="143" t="s">
+      <c r="B25" s="100" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="144"/>
-      <c r="D25" s="145"/>
+      <c r="C25" s="101"/>
+      <c r="D25" s="102"/>
       <c r="E25" s="155" t="s">
         <v>28</v>
       </c>
@@ -2904,215 +2900,215 @@
       <c r="A26" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B26" s="143" t="s">
+      <c r="B26" s="100" t="s">
         <v>32</v>
       </c>
-      <c r="C26" s="144"/>
-      <c r="D26" s="145"/>
-      <c r="E26" s="99"/>
-      <c r="F26" s="100"/>
-      <c r="G26" s="100"/>
-      <c r="H26" s="100"/>
-      <c r="I26" s="100"/>
-      <c r="J26" s="100"/>
-      <c r="K26" s="100"/>
-      <c r="L26" s="100"/>
-      <c r="M26" s="101"/>
+      <c r="C26" s="101"/>
+      <c r="D26" s="102"/>
+      <c r="E26" s="109"/>
+      <c r="F26" s="110"/>
+      <c r="G26" s="110"/>
+      <c r="H26" s="110"/>
+      <c r="I26" s="110"/>
+      <c r="J26" s="110"/>
+      <c r="K26" s="110"/>
+      <c r="L26" s="110"/>
+      <c r="M26" s="111"/>
     </row>
     <row r="27" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="143" t="s">
+      <c r="B27" s="100" t="s">
         <v>20</v>
       </c>
-      <c r="C27" s="144"/>
-      <c r="D27" s="145"/>
-      <c r="E27" s="99"/>
-      <c r="F27" s="100"/>
-      <c r="G27" s="100"/>
-      <c r="H27" s="100"/>
-      <c r="I27" s="100"/>
-      <c r="J27" s="100"/>
-      <c r="K27" s="100"/>
-      <c r="L27" s="100"/>
-      <c r="M27" s="101"/>
+      <c r="C27" s="101"/>
+      <c r="D27" s="102"/>
+      <c r="E27" s="109"/>
+      <c r="F27" s="110"/>
+      <c r="G27" s="110"/>
+      <c r="H27" s="110"/>
+      <c r="I27" s="110"/>
+      <c r="J27" s="110"/>
+      <c r="K27" s="110"/>
+      <c r="L27" s="110"/>
+      <c r="M27" s="111"/>
     </row>
     <row r="28" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3"/>
-      <c r="B28" s="143" t="s">
+      <c r="B28" s="100" t="s">
         <v>33</v>
       </c>
-      <c r="C28" s="144"/>
-      <c r="D28" s="145"/>
-      <c r="E28" s="99"/>
-      <c r="F28" s="100"/>
-      <c r="G28" s="100"/>
-      <c r="H28" s="100"/>
-      <c r="I28" s="100"/>
-      <c r="J28" s="100"/>
-      <c r="K28" s="100"/>
-      <c r="L28" s="100"/>
-      <c r="M28" s="101"/>
+      <c r="C28" s="101"/>
+      <c r="D28" s="102"/>
+      <c r="E28" s="109"/>
+      <c r="F28" s="110"/>
+      <c r="G28" s="110"/>
+      <c r="H28" s="110"/>
+      <c r="I28" s="110"/>
+      <c r="J28" s="110"/>
+      <c r="K28" s="110"/>
+      <c r="L28" s="110"/>
+      <c r="M28" s="111"/>
     </row>
     <row r="29" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3"/>
-      <c r="B29" s="143" t="s">
+      <c r="B29" s="100" t="s">
         <v>34</v>
       </c>
-      <c r="C29" s="144"/>
-      <c r="D29" s="145"/>
-      <c r="E29" s="99"/>
-      <c r="F29" s="100"/>
-      <c r="G29" s="100"/>
-      <c r="H29" s="100"/>
-      <c r="I29" s="100"/>
-      <c r="J29" s="100"/>
-      <c r="K29" s="100"/>
-      <c r="L29" s="100"/>
-      <c r="M29" s="101"/>
+      <c r="C29" s="101"/>
+      <c r="D29" s="102"/>
+      <c r="E29" s="109"/>
+      <c r="F29" s="110"/>
+      <c r="G29" s="110"/>
+      <c r="H29" s="110"/>
+      <c r="I29" s="110"/>
+      <c r="J29" s="110"/>
+      <c r="K29" s="110"/>
+      <c r="L29" s="110"/>
+      <c r="M29" s="111"/>
     </row>
     <row r="30" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B30" s="143" t="s">
+      <c r="B30" s="100" t="s">
         <v>35</v>
       </c>
-      <c r="C30" s="144"/>
-      <c r="D30" s="145"/>
-      <c r="E30" s="99"/>
-      <c r="F30" s="100"/>
-      <c r="G30" s="100"/>
-      <c r="H30" s="100"/>
-      <c r="I30" s="100"/>
-      <c r="J30" s="100"/>
-      <c r="K30" s="100"/>
-      <c r="L30" s="100"/>
-      <c r="M30" s="101"/>
+      <c r="C30" s="101"/>
+      <c r="D30" s="102"/>
+      <c r="E30" s="109"/>
+      <c r="F30" s="110"/>
+      <c r="G30" s="110"/>
+      <c r="H30" s="110"/>
+      <c r="I30" s="110"/>
+      <c r="J30" s="110"/>
+      <c r="K30" s="110"/>
+      <c r="L30" s="110"/>
+      <c r="M30" s="111"/>
     </row>
     <row r="31" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="6"/>
-      <c r="B31" s="143" t="s">
+      <c r="B31" s="100" t="s">
         <v>36</v>
       </c>
-      <c r="C31" s="144"/>
-      <c r="D31" s="145"/>
-      <c r="E31" s="99"/>
-      <c r="F31" s="100"/>
-      <c r="G31" s="100"/>
-      <c r="H31" s="100"/>
-      <c r="I31" s="100"/>
-      <c r="J31" s="100"/>
-      <c r="K31" s="100"/>
-      <c r="L31" s="100"/>
-      <c r="M31" s="101"/>
+      <c r="C31" s="101"/>
+      <c r="D31" s="102"/>
+      <c r="E31" s="109"/>
+      <c r="F31" s="110"/>
+      <c r="G31" s="110"/>
+      <c r="H31" s="110"/>
+      <c r="I31" s="110"/>
+      <c r="J31" s="110"/>
+      <c r="K31" s="110"/>
+      <c r="L31" s="110"/>
+      <c r="M31" s="111"/>
     </row>
     <row r="32" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="6"/>
-      <c r="B32" s="143" t="s">
+      <c r="B32" s="100" t="s">
         <v>19</v>
       </c>
-      <c r="C32" s="144"/>
-      <c r="D32" s="145"/>
-      <c r="E32" s="146"/>
-      <c r="F32" s="147"/>
-      <c r="G32" s="147"/>
-      <c r="H32" s="147"/>
-      <c r="I32" s="147"/>
-      <c r="J32" s="147"/>
-      <c r="K32" s="147"/>
-      <c r="L32" s="147"/>
-      <c r="M32" s="148"/>
+      <c r="C32" s="101"/>
+      <c r="D32" s="102"/>
+      <c r="E32" s="103"/>
+      <c r="F32" s="104"/>
+      <c r="G32" s="104"/>
+      <c r="H32" s="104"/>
+      <c r="I32" s="104"/>
+      <c r="J32" s="104"/>
+      <c r="K32" s="104"/>
+      <c r="L32" s="104"/>
+      <c r="M32" s="105"/>
     </row>
     <row r="33" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="6"/>
-      <c r="B33" s="143" t="s">
+      <c r="B33" s="100" t="s">
         <v>37</v>
       </c>
-      <c r="C33" s="144"/>
-      <c r="D33" s="145"/>
-      <c r="E33" s="99"/>
-      <c r="F33" s="100"/>
-      <c r="G33" s="100"/>
-      <c r="H33" s="100"/>
-      <c r="I33" s="100"/>
-      <c r="J33" s="100"/>
-      <c r="K33" s="100"/>
-      <c r="L33" s="100"/>
-      <c r="M33" s="101"/>
+      <c r="C33" s="101"/>
+      <c r="D33" s="102"/>
+      <c r="E33" s="109"/>
+      <c r="F33" s="110"/>
+      <c r="G33" s="110"/>
+      <c r="H33" s="110"/>
+      <c r="I33" s="110"/>
+      <c r="J33" s="110"/>
+      <c r="K33" s="110"/>
+      <c r="L33" s="110"/>
+      <c r="M33" s="111"/>
     </row>
     <row r="34" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="7"/>
-      <c r="B34" s="149" t="s">
+      <c r="B34" s="106" t="s">
         <v>38</v>
       </c>
-      <c r="C34" s="150"/>
-      <c r="D34" s="151"/>
-      <c r="E34" s="146"/>
-      <c r="F34" s="147"/>
-      <c r="G34" s="147"/>
-      <c r="H34" s="147"/>
-      <c r="I34" s="147"/>
-      <c r="J34" s="147"/>
-      <c r="K34" s="147"/>
-      <c r="L34" s="147"/>
-      <c r="M34" s="148"/>
+      <c r="C34" s="107"/>
+      <c r="D34" s="108"/>
+      <c r="E34" s="103"/>
+      <c r="F34" s="104"/>
+      <c r="G34" s="104"/>
+      <c r="H34" s="104"/>
+      <c r="I34" s="104"/>
+      <c r="J34" s="104"/>
+      <c r="K34" s="104"/>
+      <c r="L34" s="104"/>
+      <c r="M34" s="105"/>
     </row>
     <row r="35" spans="1:13" ht="25.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B35" s="140" t="s">
+      <c r="B35" s="97" t="s">
         <v>41</v>
       </c>
-      <c r="C35" s="141"/>
-      <c r="D35" s="142"/>
-      <c r="E35" s="146"/>
-      <c r="F35" s="147"/>
-      <c r="G35" s="147"/>
-      <c r="H35" s="147"/>
-      <c r="I35" s="147"/>
-      <c r="J35" s="147"/>
-      <c r="K35" s="147"/>
-      <c r="L35" s="147"/>
-      <c r="M35" s="148"/>
+      <c r="C35" s="98"/>
+      <c r="D35" s="99"/>
+      <c r="E35" s="103"/>
+      <c r="F35" s="104"/>
+      <c r="G35" s="104"/>
+      <c r="H35" s="104"/>
+      <c r="I35" s="104"/>
+      <c r="J35" s="104"/>
+      <c r="K35" s="104"/>
+      <c r="L35" s="104"/>
+      <c r="M35" s="105"/>
     </row>
     <row r="36" spans="1:13" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B36" s="143" t="s">
+      <c r="B36" s="100" t="s">
         <v>42</v>
       </c>
-      <c r="C36" s="144"/>
-      <c r="D36" s="145"/>
-      <c r="E36" s="146"/>
-      <c r="F36" s="147"/>
-      <c r="G36" s="147"/>
-      <c r="H36" s="147"/>
-      <c r="I36" s="147"/>
-      <c r="J36" s="147"/>
-      <c r="K36" s="147"/>
-      <c r="L36" s="147"/>
-      <c r="M36" s="148"/>
+      <c r="C36" s="101"/>
+      <c r="D36" s="102"/>
+      <c r="E36" s="103"/>
+      <c r="F36" s="104"/>
+      <c r="G36" s="104"/>
+      <c r="H36" s="104"/>
+      <c r="I36" s="104"/>
+      <c r="J36" s="104"/>
+      <c r="K36" s="104"/>
+      <c r="L36" s="104"/>
+      <c r="M36" s="105"/>
     </row>
     <row r="37" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="10"/>
-      <c r="B37" s="143" t="s">
+      <c r="B37" s="100" t="s">
         <v>19</v>
       </c>
-      <c r="C37" s="144"/>
-      <c r="D37" s="145"/>
-      <c r="E37" s="146"/>
-      <c r="F37" s="147"/>
-      <c r="G37" s="147"/>
-      <c r="H37" s="147"/>
-      <c r="I37" s="147"/>
-      <c r="J37" s="147"/>
-      <c r="K37" s="147"/>
-      <c r="L37" s="147"/>
-      <c r="M37" s="148"/>
+      <c r="C37" s="101"/>
+      <c r="D37" s="102"/>
+      <c r="E37" s="103"/>
+      <c r="F37" s="104"/>
+      <c r="G37" s="104"/>
+      <c r="H37" s="104"/>
+      <c r="I37" s="104"/>
+      <c r="J37" s="104"/>
+      <c r="K37" s="104"/>
+      <c r="L37" s="104"/>
+      <c r="M37" s="105"/>
     </row>
     <row r="38" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="36" t="s">
@@ -3204,15 +3200,15 @@
       <c r="F43" s="88" t="s">
         <v>45</v>
       </c>
-      <c r="G43" s="133"/>
-      <c r="H43" s="136"/>
+      <c r="G43" s="145"/>
+      <c r="H43" s="148"/>
       <c r="I43" s="84"/>
       <c r="J43" s="88" t="s">
         <v>46</v>
       </c>
       <c r="K43" s="89"/>
       <c r="L43" s="90"/>
-      <c r="M43" s="138"/>
+      <c r="M43" s="150"/>
     </row>
     <row r="44" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="81"/>
@@ -3220,16 +3216,16 @@
       <c r="C44" s="86"/>
       <c r="D44" s="86"/>
       <c r="E44" s="87"/>
-      <c r="F44" s="134"/>
-      <c r="G44" s="135"/>
-      <c r="H44" s="137"/>
+      <c r="F44" s="146"/>
+      <c r="G44" s="147"/>
+      <c r="H44" s="149"/>
       <c r="I44" s="87"/>
       <c r="J44" s="91" t="s">
         <v>47</v>
       </c>
       <c r="K44" s="92"/>
       <c r="L44" s="93"/>
-      <c r="M44" s="139"/>
+      <c r="M44" s="151"/>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="38" t="s">
@@ -3247,8 +3243,8 @@
       <c r="I45" s="58"/>
       <c r="J45" s="58"/>
       <c r="K45" s="74"/>
-      <c r="L45" s="127"/>
-      <c r="M45" s="128"/>
+      <c r="L45" s="139"/>
+      <c r="M45" s="140"/>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="59" t="s">
@@ -3266,8 +3262,8 @@
       <c r="I46" s="60"/>
       <c r="J46" s="60"/>
       <c r="K46" s="75"/>
-      <c r="L46" s="129"/>
-      <c r="M46" s="130"/>
+      <c r="L46" s="141"/>
+      <c r="M46" s="142"/>
     </row>
     <row r="47" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="62"/>
@@ -3281,8 +3277,8 @@
       <c r="I47" s="63"/>
       <c r="J47" s="63"/>
       <c r="K47" s="76"/>
-      <c r="L47" s="131"/>
-      <c r="M47" s="132"/>
+      <c r="L47" s="143"/>
+      <c r="M47" s="144"/>
     </row>
     <row r="48" spans="1:13" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="48" t="s">
@@ -3554,216 +3550,216 @@
         <v>56</v>
       </c>
       <c r="B65" s="39"/>
-      <c r="C65" s="119"/>
-      <c r="D65" s="120"/>
-      <c r="E65" s="120"/>
-      <c r="F65" s="120"/>
-      <c r="G65" s="120"/>
-      <c r="H65" s="120"/>
-      <c r="I65" s="120"/>
-      <c r="J65" s="120"/>
-      <c r="K65" s="120"/>
-      <c r="L65" s="120"/>
-      <c r="M65" s="121"/>
+      <c r="C65" s="131"/>
+      <c r="D65" s="132"/>
+      <c r="E65" s="132"/>
+      <c r="F65" s="132"/>
+      <c r="G65" s="132"/>
+      <c r="H65" s="132"/>
+      <c r="I65" s="132"/>
+      <c r="J65" s="132"/>
+      <c r="K65" s="132"/>
+      <c r="L65" s="132"/>
+      <c r="M65" s="133"/>
     </row>
     <row r="66" spans="1:13" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="42"/>
       <c r="B66" s="43"/>
-      <c r="C66" s="122"/>
-      <c r="D66" s="123"/>
-      <c r="E66" s="123"/>
-      <c r="F66" s="123"/>
-      <c r="G66" s="123"/>
-      <c r="H66" s="123"/>
-      <c r="I66" s="123"/>
-      <c r="J66" s="123"/>
-      <c r="K66" s="123"/>
-      <c r="L66" s="123"/>
-      <c r="M66" s="124"/>
+      <c r="C66" s="134"/>
+      <c r="D66" s="135"/>
+      <c r="E66" s="135"/>
+      <c r="F66" s="135"/>
+      <c r="G66" s="135"/>
+      <c r="H66" s="135"/>
+      <c r="I66" s="135"/>
+      <c r="J66" s="135"/>
+      <c r="K66" s="135"/>
+      <c r="L66" s="135"/>
+      <c r="M66" s="136"/>
     </row>
     <row r="67" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="38" t="s">
         <v>57</v>
       </c>
       <c r="B67" s="39"/>
-      <c r="C67" s="116"/>
-      <c r="D67" s="117"/>
-      <c r="E67" s="117"/>
-      <c r="F67" s="117"/>
-      <c r="G67" s="117"/>
-      <c r="H67" s="117"/>
-      <c r="I67" s="117"/>
-      <c r="J67" s="117"/>
-      <c r="K67" s="117"/>
-      <c r="L67" s="117"/>
-      <c r="M67" s="118"/>
+      <c r="C67" s="128"/>
+      <c r="D67" s="129"/>
+      <c r="E67" s="129"/>
+      <c r="F67" s="129"/>
+      <c r="G67" s="129"/>
+      <c r="H67" s="129"/>
+      <c r="I67" s="129"/>
+      <c r="J67" s="129"/>
+      <c r="K67" s="129"/>
+      <c r="L67" s="129"/>
+      <c r="M67" s="130"/>
     </row>
     <row r="68" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="40"/>
       <c r="B68" s="41"/>
-      <c r="C68" s="119"/>
-      <c r="D68" s="120"/>
-      <c r="E68" s="120"/>
-      <c r="F68" s="120"/>
-      <c r="G68" s="120"/>
-      <c r="H68" s="120"/>
-      <c r="I68" s="120"/>
-      <c r="J68" s="120"/>
-      <c r="K68" s="120"/>
-      <c r="L68" s="120"/>
-      <c r="M68" s="121"/>
+      <c r="C68" s="131"/>
+      <c r="D68" s="132"/>
+      <c r="E68" s="132"/>
+      <c r="F68" s="132"/>
+      <c r="G68" s="132"/>
+      <c r="H68" s="132"/>
+      <c r="I68" s="132"/>
+      <c r="J68" s="132"/>
+      <c r="K68" s="132"/>
+      <c r="L68" s="132"/>
+      <c r="M68" s="133"/>
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A69" s="40"/>
       <c r="B69" s="41"/>
-      <c r="C69" s="119"/>
-      <c r="D69" s="120"/>
-      <c r="E69" s="120"/>
-      <c r="F69" s="120"/>
-      <c r="G69" s="120"/>
-      <c r="H69" s="120"/>
-      <c r="I69" s="120"/>
-      <c r="J69" s="120"/>
-      <c r="K69" s="120"/>
-      <c r="L69" s="120"/>
-      <c r="M69" s="121"/>
+      <c r="C69" s="131"/>
+      <c r="D69" s="132"/>
+      <c r="E69" s="132"/>
+      <c r="F69" s="132"/>
+      <c r="G69" s="132"/>
+      <c r="H69" s="132"/>
+      <c r="I69" s="132"/>
+      <c r="J69" s="132"/>
+      <c r="K69" s="132"/>
+      <c r="L69" s="132"/>
+      <c r="M69" s="133"/>
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" s="40"/>
       <c r="B70" s="41"/>
-      <c r="C70" s="119"/>
-      <c r="D70" s="120"/>
-      <c r="E70" s="120"/>
-      <c r="F70" s="120"/>
-      <c r="G70" s="120"/>
-      <c r="H70" s="120"/>
-      <c r="I70" s="120"/>
-      <c r="J70" s="120"/>
-      <c r="K70" s="120"/>
-      <c r="L70" s="120"/>
-      <c r="M70" s="121"/>
+      <c r="C70" s="131"/>
+      <c r="D70" s="132"/>
+      <c r="E70" s="132"/>
+      <c r="F70" s="132"/>
+      <c r="G70" s="132"/>
+      <c r="H70" s="132"/>
+      <c r="I70" s="132"/>
+      <c r="J70" s="132"/>
+      <c r="K70" s="132"/>
+      <c r="L70" s="132"/>
+      <c r="M70" s="133"/>
     </row>
     <row r="71" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="42"/>
       <c r="B71" s="43"/>
-      <c r="C71" s="122"/>
-      <c r="D71" s="123"/>
-      <c r="E71" s="123"/>
-      <c r="F71" s="123"/>
-      <c r="G71" s="123"/>
-      <c r="H71" s="123"/>
-      <c r="I71" s="123"/>
-      <c r="J71" s="123"/>
-      <c r="K71" s="123"/>
-      <c r="L71" s="123"/>
-      <c r="M71" s="124"/>
+      <c r="C71" s="134"/>
+      <c r="D71" s="135"/>
+      <c r="E71" s="135"/>
+      <c r="F71" s="135"/>
+      <c r="G71" s="135"/>
+      <c r="H71" s="135"/>
+      <c r="I71" s="135"/>
+      <c r="J71" s="135"/>
+      <c r="K71" s="135"/>
+      <c r="L71" s="135"/>
+      <c r="M71" s="136"/>
     </row>
     <row r="72" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A72" s="125"/>
-      <c r="B72" s="125"/>
-      <c r="C72" s="125"/>
-      <c r="D72" s="125"/>
+      <c r="A72" s="137"/>
+      <c r="B72" s="137"/>
+      <c r="C72" s="137"/>
+      <c r="D72" s="137"/>
       <c r="E72" s="60"/>
       <c r="F72" s="60"/>
-      <c r="G72" s="125"/>
-      <c r="H72" s="125"/>
+      <c r="G72" s="137"/>
+      <c r="H72" s="137"/>
       <c r="I72" s="60"/>
       <c r="J72" s="60"/>
-      <c r="K72" s="125"/>
-      <c r="L72" s="125"/>
-      <c r="M72" s="125"/>
+      <c r="K72" s="137"/>
+      <c r="L72" s="137"/>
+      <c r="M72" s="137"/>
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A73" s="125"/>
-      <c r="B73" s="125"/>
-      <c r="C73" s="125"/>
-      <c r="D73" s="125"/>
+      <c r="A73" s="137"/>
+      <c r="B73" s="137"/>
+      <c r="C73" s="137"/>
+      <c r="D73" s="137"/>
       <c r="E73" s="60"/>
       <c r="F73" s="60"/>
-      <c r="G73" s="125"/>
-      <c r="H73" s="125"/>
+      <c r="G73" s="137"/>
+      <c r="H73" s="137"/>
       <c r="I73" s="60"/>
       <c r="J73" s="60"/>
-      <c r="K73" s="125"/>
-      <c r="L73" s="125"/>
-      <c r="M73" s="125"/>
+      <c r="K73" s="137"/>
+      <c r="L73" s="137"/>
+      <c r="M73" s="137"/>
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A74" s="125"/>
-      <c r="B74" s="125"/>
-      <c r="C74" s="125"/>
-      <c r="D74" s="125"/>
+      <c r="A74" s="137"/>
+      <c r="B74" s="137"/>
+      <c r="C74" s="137"/>
+      <c r="D74" s="137"/>
       <c r="E74" s="60"/>
       <c r="F74" s="60"/>
-      <c r="G74" s="125"/>
-      <c r="H74" s="125"/>
+      <c r="G74" s="137"/>
+      <c r="H74" s="137"/>
       <c r="I74" s="60"/>
       <c r="J74" s="60"/>
-      <c r="K74" s="125"/>
-      <c r="L74" s="125"/>
-      <c r="M74" s="125"/>
+      <c r="K74" s="137"/>
+      <c r="L74" s="137"/>
+      <c r="M74" s="137"/>
     </row>
     <row r="75" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A75" s="125"/>
-      <c r="B75" s="125"/>
-      <c r="C75" s="125"/>
-      <c r="D75" s="125"/>
+      <c r="A75" s="137"/>
+      <c r="B75" s="137"/>
+      <c r="C75" s="137"/>
+      <c r="D75" s="137"/>
       <c r="E75" s="60"/>
       <c r="F75" s="60"/>
-      <c r="G75" s="125"/>
-      <c r="H75" s="125"/>
+      <c r="G75" s="137"/>
+      <c r="H75" s="137"/>
       <c r="I75" s="60"/>
       <c r="J75" s="60"/>
-      <c r="K75" s="125"/>
-      <c r="L75" s="125"/>
-      <c r="M75" s="125"/>
+      <c r="K75" s="137"/>
+      <c r="L75" s="137"/>
+      <c r="M75" s="137"/>
     </row>
     <row r="76" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A76" s="125"/>
-      <c r="B76" s="125"/>
-      <c r="C76" s="125"/>
-      <c r="D76" s="125"/>
+      <c r="A76" s="137"/>
+      <c r="B76" s="137"/>
+      <c r="C76" s="137"/>
+      <c r="D76" s="137"/>
       <c r="E76" s="60"/>
       <c r="F76" s="60"/>
-      <c r="G76" s="125"/>
-      <c r="H76" s="125"/>
+      <c r="G76" s="137"/>
+      <c r="H76" s="137"/>
       <c r="I76" s="60"/>
       <c r="J76" s="60"/>
-      <c r="K76" s="125"/>
-      <c r="L76" s="125"/>
-      <c r="M76" s="125"/>
+      <c r="K76" s="137"/>
+      <c r="L76" s="137"/>
+      <c r="M76" s="137"/>
     </row>
     <row r="77" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="126"/>
-      <c r="B77" s="126"/>
-      <c r="C77" s="126"/>
-      <c r="D77" s="126"/>
+      <c r="A77" s="138"/>
+      <c r="B77" s="138"/>
+      <c r="C77" s="138"/>
+      <c r="D77" s="138"/>
       <c r="E77" s="60"/>
       <c r="F77" s="60"/>
-      <c r="G77" s="126"/>
-      <c r="H77" s="126"/>
+      <c r="G77" s="138"/>
+      <c r="H77" s="138"/>
       <c r="I77" s="60"/>
       <c r="J77" s="60"/>
-      <c r="K77" s="126"/>
-      <c r="L77" s="126"/>
-      <c r="M77" s="126"/>
+      <c r="K77" s="138"/>
+      <c r="L77" s="138"/>
+      <c r="M77" s="138"/>
     </row>
     <row r="78" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="114"/>
-      <c r="B78" s="114"/>
-      <c r="C78" s="114"/>
-      <c r="D78" s="114"/>
+      <c r="A78" s="126"/>
+      <c r="B78" s="126"/>
+      <c r="C78" s="126"/>
+      <c r="D78" s="126"/>
       <c r="E78" s="60"/>
       <c r="F78" s="60"/>
-      <c r="G78" s="115" t="s">
+      <c r="G78" s="127" t="s">
         <v>27</v>
       </c>
-      <c r="H78" s="115"/>
+      <c r="H78" s="127"/>
       <c r="I78" s="60"/>
       <c r="J78" s="60"/>
-      <c r="K78" s="114"/>
-      <c r="L78" s="114"/>
-      <c r="M78" s="114"/>
+      <c r="K78" s="126"/>
+      <c r="L78" s="126"/>
+      <c r="M78" s="126"/>
     </row>
     <row r="79" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A79" s="11"/>
@@ -3966,7 +3962,7 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el correo electrónico personal del aprendiz" sqref="E19:M19" xr:uid="{CEDF05F3-A498-464C-AF78-C83490E95D67}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el correo electrónico institucional del aprendiz @sena.edu.co , @soysena.edu.co" sqref="E20:M20" xr:uid="{8AC0CC91-D06D-4D82-A06B-CEDFF66185FC}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el nombre de la alternativa de etapa productiva, de acuerdo con las alternativas descritas en el reglamento del aprendiz vigente" sqref="E21:M21" xr:uid="{48CA359C-CBBE-4B45-B681-EA4693D12177}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar la fecha en que quedó registrada la alternativa en el aplicativo SofiaPlus.  Gestione con la coordinación académica el reporte del SVP para obtener la información requerida en este apartado" sqref="E22:M22" xr:uid="{A4B53DE5-4CEE-4C8C-A08B-9C6344C18954}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="OBLIGATORIO" prompt="Indicar la fecha de registro en el aplicativo SofiaPlus. RUTA: INGRESAR A SOFIAPLUS-APRENDIZ-CONSULTAR INSCRIPCIONES A PROGRAMAS...----DETALLE DE INSCRIPCION // PARTE INFWERIOR INDICA LA FECHA DE INSCRIPCION" sqref="E22:M22" xr:uid="{A4B53DE5-4CEE-4C8C-A08B-9C6344C18954}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el nombre completo de la empresa o entidad co-formadora (empresa, entidad o institución gubernamental o no gubernamental)." sqref="E26:M26" xr:uid="{35AC5BC6-659F-4E4C-B567-3C3F16C509BD}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar la dirección de la empresa, entidad o institución gubernamental o no gubernamental." sqref="E27:M27" xr:uid="{18FD205E-10DD-4EB5-8E57-F8B0C00BF5BC}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el numero NIT de la empresa, entidad o institución gubernamental o no gubernamental." sqref="E28:M28" xr:uid="{0E9499EA-A21D-4209-94F0-6561C0BEA458}"/>
@@ -3976,13 +3972,13 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el número del celular del jefe inmediato o supervisor y el número fijo de la empresa con extensión" sqref="E32:M32" xr:uid="{D17896B5-5299-404D-BF06-0A7409E6BB11}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="En caso de que aplique, registrar el nombre de otro contacto en la empresa. De no tener digitar N/A" sqref="E33:M33" xr:uid="{A6F4976B-257F-4E38-96A4-122163F2BCDA}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el teléfono institucional al cual contactarse en caso que el ente coformador no responda" sqref="E34:M34" xr:uid="{A593241B-15E7-4EA6-B9DE-E0DF01ED6DB9}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="En caso de que el aprendiz sea una persona en situación de discapacidad, diligencie este espacio con el nombre de la persona que le asiste." sqref="E35:M35" xr:uid="{C19946D2-B571-4104-A1EA-FEF5A7253596}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Aquí se especifica el tipo de asistencia brindada al aprendiz para que desempeñe la totalidad de sus tareas asegurando un ambiente laboral inclusivo adecuado a sus necesidades. Puede incluir asistencias como lenguaje de señas, soporte visual etc" sqref="E36:M36" xr:uid="{B635F5F5-108B-409C-BCAD-0AA5A654CF02}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el número del celular de la persona que asiste al aprendiz " sqref="E37:M37" xr:uid="{77AEF51E-4966-4ADA-B94D-7E72C6BE4FFA}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Si no aplica Colocar N/A" prompt="En caso de que el aprendiz sea una persona en situación de discapacidad, diligencie este espacio con el nombre de la persona que le asiste." sqref="E35:M35" xr:uid="{C19946D2-B571-4104-A1EA-FEF5A7253596}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Si no aplica colocar N/A" prompt="Aquí se especifica el tipo de asistencia brindada al aprendiz para que desempeñe la totalidad de sus tareas asegurando un ambiente laboral inclusivo adecuado a sus necesidades. Puede incluir asistencias como lenguaje de señas, soporte visual etc" sqref="E36:M36" xr:uid="{B635F5F5-108B-409C-BCAD-0AA5A654CF02}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Si no aplica colocar N/A" prompt="Registrar el número del celular de la persona que asiste al aprendiz " sqref="E37:M37" xr:uid="{77AEF51E-4966-4ADA-B94D-7E72C6BE4FFA}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar la fecha Inicial de ejecución de la etapa productiva del aprendiz,  La cual se encuentra registrada en el sistema de gestión académico administrativo" sqref="B43:E44" xr:uid="{ADDD56B1-A1AE-4F35-A152-F9DAB746A3F8}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar la fecha fin de ejecución de la etapa productiva del aprendiz,  La cual se encuentra registrada en el sistema de gestión académico administrativo" sqref="H43:I44" xr:uid="{A2994507-EBC1-4758-8D2D-041DB7D68E81}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar la fecha de afiliación en la ARL realizada por el centro de formación o la empresa, solo aplica para aprendices que se encuentren en Colombia." sqref="M43:M44" xr:uid="{0E74721C-02A8-4123-BB25-E650EFDE799B}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar el número de póliza que se registra en la ARL." sqref="D45:G47" xr:uid="{AEDBE09E-E16B-4102-8DD1-046357FA9976}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="OBLIGATORIO" prompt="Indicar la fecha de afiliación en la ARL realizada por el centro de formación o la empresa, solo aplica para aprendices que se encuentren en Colombia." sqref="M43:M44" xr:uid="{0E74721C-02A8-4123-BB25-E650EFDE799B}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="OBLIGATORIO consultar con RR.HH." prompt="Indicar el número de póliza que se registra en la ARL. SI NO LO REGISTRA EL FORMATO SERA DEVUELTO " sqref="D45:G47" xr:uid="{AEDBE09E-E16B-4102-8DD1-046357FA9976}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el horario en el cual el aprendiz ejecutará su etapa productiva." sqref="L45:M47" xr:uid="{22678B76-AB93-48B7-B0CA-9F11DDE08012}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Adjuntar enlace de grabacion de la sesion, el enlace le llaga al aprendiz por correo de la citacion." sqref="D48:M48" xr:uid="{81EA4BA8-6491-4C84-9D5E-95D4DAC042D4}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Relacione las actividades que el aprendiz va a realizar según lo acordado. (Estas deben corresponder al perfil del egresado establecido en el programa de formación que el aprendiz está desarrollando.) redactar activ. en  verbos en infinitivo" sqref="C60:C64" xr:uid="{765A44AD-7EE4-4C8A-82B9-AEB337B3CBFF}"/>
@@ -3990,7 +3986,7 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registre los comentarios que considere pertinentes en relación a la visita correspondiente. " sqref="C67:M71" xr:uid="{08D354B0-14A2-4554-94A3-2633D73D772A}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el nombre completo del aprendiz y en la parte superior la Firma manuscrita o digital." sqref="A78:D78" xr:uid="{A7FEFB2B-7370-4FA2-8820-7EB89B730FD1}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registrar el nombre completo del co-formador y en la parte superior de esta la Firma manuscrita o digital." sqref="K78:M78" xr:uid="{DAE2A968-2309-42D5-952C-BC599D7BE50F}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Diligenciar fecha de la sesión en este espacio. Ejemplo: Bogotá dia/mes/año Virtual" sqref="C80:J80" xr:uid="{201095D8-80DA-45BB-84F9-D066E44DB3C5}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Bogotá dd/mm/aaaa   virtual" prompt="Diligenciar fecha de la sesión en este espacio. Ejemplo: Bogotá dia/mes/año Virtual" sqref="C80:J80" xr:uid="{201095D8-80DA-45BB-84F9-D066E44DB3C5}"/>
   </dataValidations>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" scale="68" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Actualiza formatos: Bitacoras y Visita 1
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Formatos/Visita 1 GFPI-F023.xlsx
+++ b/Formatos/Visita 1 GFPI-F023.xlsx
@@ -5,16 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/834af06e427efe68/Documents/Seto 2026/sena/Manual SENA Etapa Productiva/manual-aprendiz-sena/Formatos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{9057EC18-0F9F-4B95-BC58-7A90354B991C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C9572E7-A1D1-4AC0-BC16-42E3574CC708}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7298B0B-D518-46BF-A6D4-8320B0565BBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BC3553EE-4E49-4F2A-B03E-CFAC4EB3009B}"/>
   </bookViews>
   <sheets>
     <sheet name="Formato Visita 1" sheetId="1" r:id="rId1"/>
-    <sheet name="BD_SENA" sheetId="5" state="hidden" r:id="rId2"/>
+    <sheet name="BD_SENA" sheetId="5" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="Análisis_y_Desarrollo_de_Software">#REF!</definedName>
@@ -1374,6 +1374,399 @@
         </ext>
       </extLst>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1416,24 +1809,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -1483,23 +1858,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1512,10 +1872,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1524,367 +1880,11 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -2458,1296 +2458,1296 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="139" t="s">
         <v>115</v>
       </c>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="26"/>
+      <c r="C1" s="140"/>
+      <c r="D1" s="140"/>
+      <c r="E1" s="140"/>
+      <c r="F1" s="140"/>
+      <c r="G1" s="140"/>
+      <c r="H1" s="140"/>
+      <c r="I1" s="140"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="141"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="148" t="s">
         <v>122</v>
       </c>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="35"/>
+      <c r="C2" s="149"/>
+      <c r="D2" s="149"/>
+      <c r="E2" s="149"/>
+      <c r="F2" s="149"/>
+      <c r="G2" s="149"/>
+      <c r="H2" s="149"/>
+      <c r="I2" s="149"/>
+      <c r="J2" s="149"/>
+      <c r="K2" s="150"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="142" t="s">
         <v>116</v>
       </c>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
-      <c r="I3" s="28"/>
-      <c r="J3" s="28"/>
-      <c r="K3" s="29"/>
+      <c r="C3" s="143"/>
+      <c r="D3" s="143"/>
+      <c r="E3" s="143"/>
+      <c r="F3" s="143"/>
+      <c r="G3" s="143"/>
+      <c r="H3" s="143"/>
+      <c r="I3" s="143"/>
+      <c r="J3" s="143"/>
+      <c r="K3" s="144"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="148" t="s">
         <v>121</v>
       </c>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="35"/>
+      <c r="C4" s="149"/>
+      <c r="D4" s="149"/>
+      <c r="E4" s="149"/>
+      <c r="F4" s="149"/>
+      <c r="G4" s="149"/>
+      <c r="H4" s="149"/>
+      <c r="I4" s="149"/>
+      <c r="J4" s="149"/>
+      <c r="K4" s="150"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="142" t="s">
         <v>117</v>
       </c>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
-      <c r="K5" s="29"/>
+      <c r="C5" s="143"/>
+      <c r="D5" s="143"/>
+      <c r="E5" s="143"/>
+      <c r="F5" s="143"/>
+      <c r="G5" s="143"/>
+      <c r="H5" s="143"/>
+      <c r="I5" s="143"/>
+      <c r="J5" s="143"/>
+      <c r="K5" s="144"/>
     </row>
     <row r="6" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="145" t="s">
         <v>118</v>
       </c>
-      <c r="C6" s="31"/>
+      <c r="C6" s="146"/>
       <c r="D6" s="22" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="32" t="s">
+      <c r="E6" s="147" t="s">
         <v>119</v>
       </c>
-      <c r="F6" s="31"/>
-      <c r="G6" s="31"/>
+      <c r="F6" s="146"/>
+      <c r="G6" s="146"/>
       <c r="H6" s="22" t="b">
         <v>0</v>
       </c>
-      <c r="I6" s="32" t="s">
+      <c r="I6" s="147" t="s">
         <v>120</v>
       </c>
-      <c r="J6" s="31"/>
+      <c r="J6" s="146"/>
       <c r="K6" s="23" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25"/>
     <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="112" t="s">
+      <c r="A8" s="63" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="113"/>
-      <c r="C8" s="113"/>
-      <c r="D8" s="113"/>
-      <c r="E8" s="113"/>
-      <c r="F8" s="113"/>
-      <c r="G8" s="113"/>
-      <c r="H8" s="113"/>
-      <c r="I8" s="113"/>
-      <c r="J8" s="113"/>
-      <c r="K8" s="113"/>
-      <c r="L8" s="113"/>
-      <c r="M8" s="113"/>
+      <c r="B8" s="64"/>
+      <c r="C8" s="64"/>
+      <c r="D8" s="64"/>
+      <c r="E8" s="64"/>
+      <c r="F8" s="64"/>
+      <c r="G8" s="64"/>
+      <c r="H8" s="64"/>
+      <c r="I8" s="64"/>
+      <c r="J8" s="64"/>
+      <c r="K8" s="64"/>
+      <c r="L8" s="64"/>
+      <c r="M8" s="64"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="100" t="s">
+      <c r="A9" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="102"/>
-      <c r="C9" s="94" t="s">
+      <c r="B9" s="27"/>
+      <c r="C9" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="D9" s="95"/>
-      <c r="E9" s="95"/>
-      <c r="F9" s="95"/>
-      <c r="G9" s="95"/>
-      <c r="H9" s="95"/>
-      <c r="I9" s="95"/>
-      <c r="J9" s="95"/>
-      <c r="K9" s="95"/>
-      <c r="L9" s="95"/>
-      <c r="M9" s="96"/>
+      <c r="D9" s="132"/>
+      <c r="E9" s="132"/>
+      <c r="F9" s="132"/>
+      <c r="G9" s="132"/>
+      <c r="H9" s="132"/>
+      <c r="I9" s="132"/>
+      <c r="J9" s="132"/>
+      <c r="K9" s="132"/>
+      <c r="L9" s="132"/>
+      <c r="M9" s="47"/>
     </row>
     <row r="10" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="100" t="s">
+      <c r="A10" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="102"/>
-      <c r="C10" s="155" t="s">
+      <c r="B10" s="27"/>
+      <c r="C10" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="D10" s="156"/>
-      <c r="E10" s="156"/>
-      <c r="F10" s="156"/>
-      <c r="G10" s="157"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="30"/>
       <c r="H10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I10" s="45"/>
-      <c r="J10" s="46"/>
-      <c r="K10" s="46"/>
-      <c r="L10" s="46"/>
-      <c r="M10" s="47"/>
+      <c r="I10" s="154"/>
+      <c r="J10" s="155"/>
+      <c r="K10" s="155"/>
+      <c r="L10" s="155"/>
+      <c r="M10" s="156"/>
     </row>
     <row r="11" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="100" t="s">
+      <c r="A11" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="102"/>
-      <c r="C11" s="167"/>
-      <c r="D11" s="168"/>
-      <c r="E11" s="168"/>
-      <c r="F11" s="168"/>
-      <c r="G11" s="168"/>
-      <c r="H11" s="169"/>
-      <c r="I11" s="42" t="s">
+      <c r="B11" s="27"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="42"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="42"/>
+      <c r="H11" s="43"/>
+      <c r="I11" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="J11" s="43"/>
-      <c r="K11" s="114"/>
-      <c r="L11" s="115"/>
-      <c r="M11" s="116"/>
+      <c r="J11" s="45"/>
+      <c r="K11" s="65"/>
+      <c r="L11" s="66"/>
+      <c r="M11" s="67"/>
     </row>
     <row r="12" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="100" t="s">
+      <c r="A12" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="102"/>
+      <c r="B12" s="27"/>
       <c r="C12" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D12" s="94" t="s">
+      <c r="D12" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="96"/>
-      <c r="F12" s="170" t="s">
+      <c r="E12" s="47"/>
+      <c r="F12" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="G12" s="171"/>
+      <c r="G12" s="49"/>
       <c r="H12" s="1"/>
-      <c r="I12" s="170" t="s">
+      <c r="I12" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="J12" s="171"/>
-      <c r="K12" s="117"/>
-      <c r="L12" s="118"/>
-      <c r="M12" s="119"/>
+      <c r="J12" s="49"/>
+      <c r="K12" s="68"/>
+      <c r="L12" s="69"/>
+      <c r="M12" s="70"/>
     </row>
     <row r="13" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="100" t="s">
+      <c r="A13" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="102"/>
-      <c r="C13" s="160"/>
-      <c r="D13" s="161"/>
-      <c r="E13" s="161"/>
-      <c r="F13" s="162"/>
-      <c r="G13" s="160" t="s">
+      <c r="B13" s="27"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="H13" s="161"/>
-      <c r="I13" s="162"/>
-      <c r="J13" s="120"/>
-      <c r="K13" s="121"/>
-      <c r="L13" s="121"/>
-      <c r="M13" s="122"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="33"/>
+      <c r="J13" s="71"/>
+      <c r="K13" s="72"/>
+      <c r="L13" s="72"/>
+      <c r="M13" s="73"/>
     </row>
     <row r="14" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="163" t="s">
+      <c r="A14" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="100" t="s">
+      <c r="B14" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="101"/>
-      <c r="D14" s="102"/>
-      <c r="E14" s="109"/>
-      <c r="F14" s="110"/>
-      <c r="G14" s="110"/>
-      <c r="H14" s="110"/>
-      <c r="I14" s="110"/>
-      <c r="J14" s="110"/>
-      <c r="K14" s="110"/>
-      <c r="L14" s="110"/>
-      <c r="M14" s="111"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="53"/>
+      <c r="F14" s="54"/>
+      <c r="G14" s="54"/>
+      <c r="H14" s="54"/>
+      <c r="I14" s="54"/>
+      <c r="J14" s="54"/>
+      <c r="K14" s="54"/>
+      <c r="L14" s="54"/>
+      <c r="M14" s="55"/>
     </row>
     <row r="15" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="147"/>
-      <c r="B15" s="164" t="s">
+      <c r="A15" s="35"/>
+      <c r="B15" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="165"/>
-      <c r="D15" s="166"/>
-      <c r="E15" s="123"/>
-      <c r="F15" s="124"/>
-      <c r="G15" s="124"/>
-      <c r="H15" s="124"/>
-      <c r="I15" s="124"/>
-      <c r="J15" s="124"/>
-      <c r="K15" s="124"/>
-      <c r="L15" s="124"/>
-      <c r="M15" s="125"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="74"/>
+      <c r="F15" s="75"/>
+      <c r="G15" s="75"/>
+      <c r="H15" s="75"/>
+      <c r="I15" s="75"/>
+      <c r="J15" s="75"/>
+      <c r="K15" s="75"/>
+      <c r="L15" s="75"/>
+      <c r="M15" s="76"/>
     </row>
     <row r="16" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="147"/>
-      <c r="B16" s="100" t="s">
+      <c r="A16" s="35"/>
+      <c r="B16" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="101"/>
-      <c r="D16" s="102"/>
-      <c r="E16" s="109"/>
-      <c r="F16" s="110"/>
-      <c r="G16" s="110"/>
-      <c r="H16" s="110"/>
-      <c r="I16" s="110"/>
-      <c r="J16" s="110"/>
-      <c r="K16" s="110"/>
-      <c r="L16" s="110"/>
-      <c r="M16" s="111"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="53"/>
+      <c r="F16" s="54"/>
+      <c r="G16" s="54"/>
+      <c r="H16" s="54"/>
+      <c r="I16" s="54"/>
+      <c r="J16" s="54"/>
+      <c r="K16" s="54"/>
+      <c r="L16" s="54"/>
+      <c r="M16" s="55"/>
     </row>
     <row r="17" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="147"/>
-      <c r="B17" s="100" t="s">
+      <c r="A17" s="35"/>
+      <c r="B17" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="101"/>
-      <c r="D17" s="102"/>
-      <c r="E17" s="109"/>
-      <c r="F17" s="110"/>
-      <c r="G17" s="110"/>
-      <c r="H17" s="110"/>
-      <c r="I17" s="110"/>
-      <c r="J17" s="110"/>
-      <c r="K17" s="110"/>
-      <c r="L17" s="110"/>
-      <c r="M17" s="111"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="53"/>
+      <c r="F17" s="54"/>
+      <c r="G17" s="54"/>
+      <c r="H17" s="54"/>
+      <c r="I17" s="54"/>
+      <c r="J17" s="54"/>
+      <c r="K17" s="54"/>
+      <c r="L17" s="54"/>
+      <c r="M17" s="55"/>
     </row>
     <row r="18" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="147"/>
-      <c r="B18" s="100" t="s">
+      <c r="A18" s="35"/>
+      <c r="B18" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="101"/>
-      <c r="D18" s="102"/>
-      <c r="E18" s="109"/>
-      <c r="F18" s="110"/>
-      <c r="G18" s="110"/>
-      <c r="H18" s="110"/>
-      <c r="I18" s="110"/>
-      <c r="J18" s="110"/>
-      <c r="K18" s="110"/>
-      <c r="L18" s="110"/>
-      <c r="M18" s="111"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="53"/>
+      <c r="F18" s="54"/>
+      <c r="G18" s="54"/>
+      <c r="H18" s="54"/>
+      <c r="I18" s="54"/>
+      <c r="J18" s="54"/>
+      <c r="K18" s="54"/>
+      <c r="L18" s="54"/>
+      <c r="M18" s="55"/>
     </row>
     <row r="19" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="147"/>
-      <c r="B19" s="100" t="s">
+      <c r="A19" s="35"/>
+      <c r="B19" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="101"/>
-      <c r="D19" s="102"/>
-      <c r="E19" s="109"/>
-      <c r="F19" s="110"/>
-      <c r="G19" s="110"/>
-      <c r="H19" s="110"/>
-      <c r="I19" s="110"/>
-      <c r="J19" s="110"/>
-      <c r="K19" s="110"/>
-      <c r="L19" s="110"/>
-      <c r="M19" s="111"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="53"/>
+      <c r="F19" s="54"/>
+      <c r="G19" s="54"/>
+      <c r="H19" s="54"/>
+      <c r="I19" s="54"/>
+      <c r="J19" s="54"/>
+      <c r="K19" s="54"/>
+      <c r="L19" s="54"/>
+      <c r="M19" s="55"/>
     </row>
     <row r="20" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="147"/>
-      <c r="B20" s="100" t="s">
+      <c r="A20" s="35"/>
+      <c r="B20" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="101"/>
-      <c r="D20" s="102"/>
-      <c r="E20" s="103"/>
-      <c r="F20" s="104"/>
-      <c r="G20" s="104"/>
-      <c r="H20" s="104"/>
-      <c r="I20" s="104"/>
-      <c r="J20" s="104"/>
-      <c r="K20" s="104"/>
-      <c r="L20" s="104"/>
-      <c r="M20" s="105"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="51"/>
+      <c r="G20" s="51"/>
+      <c r="H20" s="51"/>
+      <c r="I20" s="51"/>
+      <c r="J20" s="51"/>
+      <c r="K20" s="51"/>
+      <c r="L20" s="51"/>
+      <c r="M20" s="52"/>
     </row>
     <row r="21" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="147"/>
-      <c r="B21" s="100" t="s">
+      <c r="A21" s="35"/>
+      <c r="B21" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="C21" s="101"/>
-      <c r="D21" s="102"/>
-      <c r="E21" s="103"/>
-      <c r="F21" s="104"/>
-      <c r="G21" s="104"/>
-      <c r="H21" s="104"/>
-      <c r="I21" s="104"/>
-      <c r="J21" s="104"/>
-      <c r="K21" s="104"/>
-      <c r="L21" s="104"/>
-      <c r="M21" s="105"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="51"/>
+      <c r="H21" s="51"/>
+      <c r="I21" s="51"/>
+      <c r="J21" s="51"/>
+      <c r="K21" s="51"/>
+      <c r="L21" s="51"/>
+      <c r="M21" s="52"/>
     </row>
     <row r="22" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="148"/>
-      <c r="B22" s="100" t="s">
+      <c r="A22" s="36"/>
+      <c r="B22" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="C22" s="101"/>
-      <c r="D22" s="102"/>
-      <c r="E22" s="103"/>
-      <c r="F22" s="104"/>
-      <c r="G22" s="104"/>
-      <c r="H22" s="104"/>
-      <c r="I22" s="104"/>
-      <c r="J22" s="104"/>
-      <c r="K22" s="104"/>
-      <c r="L22" s="104"/>
-      <c r="M22" s="105"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="51"/>
+      <c r="H22" s="51"/>
+      <c r="I22" s="51"/>
+      <c r="J22" s="51"/>
+      <c r="K22" s="51"/>
+      <c r="L22" s="51"/>
+      <c r="M22" s="52"/>
     </row>
     <row r="23" spans="1:13" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="146" t="s">
+      <c r="A23" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="100" t="s">
+      <c r="B23" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="101"/>
-      <c r="D23" s="102"/>
-      <c r="E23" s="149" t="s">
+      <c r="C23" s="37"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="57" t="s">
         <v>27</v>
       </c>
-      <c r="F23" s="150"/>
-      <c r="G23" s="150"/>
-      <c r="H23" s="150"/>
-      <c r="I23" s="150"/>
-      <c r="J23" s="150"/>
-      <c r="K23" s="150"/>
-      <c r="L23" s="150"/>
-      <c r="M23" s="151"/>
+      <c r="F23" s="58"/>
+      <c r="G23" s="58"/>
+      <c r="H23" s="58"/>
+      <c r="I23" s="58"/>
+      <c r="J23" s="58"/>
+      <c r="K23" s="58"/>
+      <c r="L23" s="58"/>
+      <c r="M23" s="59"/>
     </row>
     <row r="24" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="147"/>
-      <c r="B24" s="100" t="s">
+      <c r="A24" s="35"/>
+      <c r="B24" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C24" s="101"/>
-      <c r="D24" s="102"/>
-      <c r="E24" s="152"/>
-      <c r="F24" s="153"/>
-      <c r="G24" s="153"/>
-      <c r="H24" s="153"/>
-      <c r="I24" s="153"/>
-      <c r="J24" s="153"/>
-      <c r="K24" s="153"/>
-      <c r="L24" s="153"/>
-      <c r="M24" s="154"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="60"/>
+      <c r="F24" s="61"/>
+      <c r="G24" s="61"/>
+      <c r="H24" s="61"/>
+      <c r="I24" s="61"/>
+      <c r="J24" s="61"/>
+      <c r="K24" s="61"/>
+      <c r="L24" s="61"/>
+      <c r="M24" s="62"/>
     </row>
     <row r="25" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="148"/>
-      <c r="B25" s="100" t="s">
+      <c r="A25" s="36"/>
+      <c r="B25" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="101"/>
-      <c r="D25" s="102"/>
-      <c r="E25" s="149" t="s">
+      <c r="C25" s="37"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="57" t="s">
         <v>28</v>
       </c>
-      <c r="F25" s="150"/>
-      <c r="G25" s="150"/>
-      <c r="H25" s="150"/>
-      <c r="I25" s="150"/>
-      <c r="J25" s="150"/>
-      <c r="K25" s="150"/>
-      <c r="L25" s="150"/>
-      <c r="M25" s="151"/>
+      <c r="F25" s="58"/>
+      <c r="G25" s="58"/>
+      <c r="H25" s="58"/>
+      <c r="I25" s="58"/>
+      <c r="J25" s="58"/>
+      <c r="K25" s="58"/>
+      <c r="L25" s="58"/>
+      <c r="M25" s="59"/>
     </row>
     <row r="26" spans="1:13" ht="25.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B26" s="100" t="s">
+      <c r="B26" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C26" s="101"/>
-      <c r="D26" s="102"/>
-      <c r="E26" s="109"/>
-      <c r="F26" s="110"/>
-      <c r="G26" s="110"/>
-      <c r="H26" s="110"/>
-      <c r="I26" s="110"/>
-      <c r="J26" s="110"/>
-      <c r="K26" s="110"/>
-      <c r="L26" s="110"/>
-      <c r="M26" s="111"/>
+      <c r="C26" s="37"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="53"/>
+      <c r="F26" s="54"/>
+      <c r="G26" s="54"/>
+      <c r="H26" s="54"/>
+      <c r="I26" s="54"/>
+      <c r="J26" s="54"/>
+      <c r="K26" s="54"/>
+      <c r="L26" s="54"/>
+      <c r="M26" s="55"/>
     </row>
     <row r="27" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="100" t="s">
+      <c r="B27" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="C27" s="101"/>
-      <c r="D27" s="102"/>
-      <c r="E27" s="109"/>
-      <c r="F27" s="110"/>
-      <c r="G27" s="110"/>
-      <c r="H27" s="110"/>
-      <c r="I27" s="110"/>
-      <c r="J27" s="110"/>
-      <c r="K27" s="110"/>
-      <c r="L27" s="110"/>
-      <c r="M27" s="111"/>
+      <c r="C27" s="37"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="53"/>
+      <c r="F27" s="54"/>
+      <c r="G27" s="54"/>
+      <c r="H27" s="54"/>
+      <c r="I27" s="54"/>
+      <c r="J27" s="54"/>
+      <c r="K27" s="54"/>
+      <c r="L27" s="54"/>
+      <c r="M27" s="55"/>
     </row>
     <row r="28" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3"/>
-      <c r="B28" s="100" t="s">
+      <c r="B28" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="C28" s="101"/>
-      <c r="D28" s="102"/>
-      <c r="E28" s="109"/>
-      <c r="F28" s="110"/>
-      <c r="G28" s="110"/>
-      <c r="H28" s="110"/>
-      <c r="I28" s="110"/>
-      <c r="J28" s="110"/>
-      <c r="K28" s="110"/>
-      <c r="L28" s="110"/>
-      <c r="M28" s="111"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="53"/>
+      <c r="F28" s="54"/>
+      <c r="G28" s="54"/>
+      <c r="H28" s="54"/>
+      <c r="I28" s="54"/>
+      <c r="J28" s="54"/>
+      <c r="K28" s="54"/>
+      <c r="L28" s="54"/>
+      <c r="M28" s="55"/>
     </row>
     <row r="29" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3"/>
-      <c r="B29" s="100" t="s">
+      <c r="B29" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="C29" s="101"/>
-      <c r="D29" s="102"/>
-      <c r="E29" s="109"/>
-      <c r="F29" s="110"/>
-      <c r="G29" s="110"/>
-      <c r="H29" s="110"/>
-      <c r="I29" s="110"/>
-      <c r="J29" s="110"/>
-      <c r="K29" s="110"/>
-      <c r="L29" s="110"/>
-      <c r="M29" s="111"/>
+      <c r="C29" s="37"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="53"/>
+      <c r="F29" s="54"/>
+      <c r="G29" s="54"/>
+      <c r="H29" s="54"/>
+      <c r="I29" s="54"/>
+      <c r="J29" s="54"/>
+      <c r="K29" s="54"/>
+      <c r="L29" s="54"/>
+      <c r="M29" s="55"/>
     </row>
     <row r="30" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B30" s="100" t="s">
+      <c r="B30" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="C30" s="101"/>
-      <c r="D30" s="102"/>
-      <c r="E30" s="109"/>
-      <c r="F30" s="110"/>
-      <c r="G30" s="110"/>
-      <c r="H30" s="110"/>
-      <c r="I30" s="110"/>
-      <c r="J30" s="110"/>
-      <c r="K30" s="110"/>
-      <c r="L30" s="110"/>
-      <c r="M30" s="111"/>
+      <c r="C30" s="37"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="53"/>
+      <c r="F30" s="54"/>
+      <c r="G30" s="54"/>
+      <c r="H30" s="54"/>
+      <c r="I30" s="54"/>
+      <c r="J30" s="54"/>
+      <c r="K30" s="54"/>
+      <c r="L30" s="54"/>
+      <c r="M30" s="55"/>
     </row>
     <row r="31" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="6"/>
-      <c r="B31" s="100" t="s">
+      <c r="B31" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="C31" s="101"/>
-      <c r="D31" s="102"/>
-      <c r="E31" s="109"/>
-      <c r="F31" s="110"/>
-      <c r="G31" s="110"/>
-      <c r="H31" s="110"/>
-      <c r="I31" s="110"/>
-      <c r="J31" s="110"/>
-      <c r="K31" s="110"/>
-      <c r="L31" s="110"/>
-      <c r="M31" s="111"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="27"/>
+      <c r="E31" s="53"/>
+      <c r="F31" s="54"/>
+      <c r="G31" s="54"/>
+      <c r="H31" s="54"/>
+      <c r="I31" s="54"/>
+      <c r="J31" s="54"/>
+      <c r="K31" s="54"/>
+      <c r="L31" s="54"/>
+      <c r="M31" s="55"/>
     </row>
     <row r="32" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="6"/>
-      <c r="B32" s="100" t="s">
+      <c r="B32" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C32" s="101"/>
-      <c r="D32" s="102"/>
-      <c r="E32" s="103"/>
-      <c r="F32" s="104"/>
-      <c r="G32" s="104"/>
-      <c r="H32" s="104"/>
-      <c r="I32" s="104"/>
-      <c r="J32" s="104"/>
-      <c r="K32" s="104"/>
-      <c r="L32" s="104"/>
-      <c r="M32" s="105"/>
+      <c r="C32" s="37"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="50"/>
+      <c r="F32" s="51"/>
+      <c r="G32" s="51"/>
+      <c r="H32" s="51"/>
+      <c r="I32" s="51"/>
+      <c r="J32" s="51"/>
+      <c r="K32" s="51"/>
+      <c r="L32" s="51"/>
+      <c r="M32" s="52"/>
     </row>
     <row r="33" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="6"/>
-      <c r="B33" s="100" t="s">
+      <c r="B33" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="C33" s="101"/>
-      <c r="D33" s="102"/>
-      <c r="E33" s="109"/>
-      <c r="F33" s="110"/>
-      <c r="G33" s="110"/>
-      <c r="H33" s="110"/>
-      <c r="I33" s="110"/>
-      <c r="J33" s="110"/>
-      <c r="K33" s="110"/>
-      <c r="L33" s="110"/>
-      <c r="M33" s="111"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="53"/>
+      <c r="F33" s="54"/>
+      <c r="G33" s="54"/>
+      <c r="H33" s="54"/>
+      <c r="I33" s="54"/>
+      <c r="J33" s="54"/>
+      <c r="K33" s="54"/>
+      <c r="L33" s="54"/>
+      <c r="M33" s="55"/>
     </row>
     <row r="34" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="7"/>
-      <c r="B34" s="106" t="s">
+      <c r="B34" s="136" t="s">
         <v>38</v>
       </c>
-      <c r="C34" s="107"/>
-      <c r="D34" s="108"/>
-      <c r="E34" s="103"/>
-      <c r="F34" s="104"/>
-      <c r="G34" s="104"/>
-      <c r="H34" s="104"/>
-      <c r="I34" s="104"/>
-      <c r="J34" s="104"/>
-      <c r="K34" s="104"/>
-      <c r="L34" s="104"/>
-      <c r="M34" s="105"/>
+      <c r="C34" s="137"/>
+      <c r="D34" s="138"/>
+      <c r="E34" s="50"/>
+      <c r="F34" s="51"/>
+      <c r="G34" s="51"/>
+      <c r="H34" s="51"/>
+      <c r="I34" s="51"/>
+      <c r="J34" s="51"/>
+      <c r="K34" s="51"/>
+      <c r="L34" s="51"/>
+      <c r="M34" s="52"/>
     </row>
     <row r="35" spans="1:13" ht="25.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B35" s="97" t="s">
+      <c r="B35" s="133" t="s">
         <v>41</v>
       </c>
-      <c r="C35" s="98"/>
-      <c r="D35" s="99"/>
-      <c r="E35" s="103"/>
-      <c r="F35" s="104"/>
-      <c r="G35" s="104"/>
-      <c r="H35" s="104"/>
-      <c r="I35" s="104"/>
-      <c r="J35" s="104"/>
-      <c r="K35" s="104"/>
-      <c r="L35" s="104"/>
-      <c r="M35" s="105"/>
+      <c r="C35" s="134"/>
+      <c r="D35" s="135"/>
+      <c r="E35" s="50"/>
+      <c r="F35" s="51"/>
+      <c r="G35" s="51"/>
+      <c r="H35" s="51"/>
+      <c r="I35" s="51"/>
+      <c r="J35" s="51"/>
+      <c r="K35" s="51"/>
+      <c r="L35" s="51"/>
+      <c r="M35" s="52"/>
     </row>
     <row r="36" spans="1:13" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B36" s="100" t="s">
+      <c r="B36" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="C36" s="101"/>
-      <c r="D36" s="102"/>
-      <c r="E36" s="103"/>
-      <c r="F36" s="104"/>
-      <c r="G36" s="104"/>
-      <c r="H36" s="104"/>
-      <c r="I36" s="104"/>
-      <c r="J36" s="104"/>
-      <c r="K36" s="104"/>
-      <c r="L36" s="104"/>
-      <c r="M36" s="105"/>
+      <c r="C36" s="37"/>
+      <c r="D36" s="27"/>
+      <c r="E36" s="50"/>
+      <c r="F36" s="51"/>
+      <c r="G36" s="51"/>
+      <c r="H36" s="51"/>
+      <c r="I36" s="51"/>
+      <c r="J36" s="51"/>
+      <c r="K36" s="51"/>
+      <c r="L36" s="51"/>
+      <c r="M36" s="52"/>
     </row>
     <row r="37" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="10"/>
-      <c r="B37" s="100" t="s">
+      <c r="B37" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C37" s="101"/>
-      <c r="D37" s="102"/>
-      <c r="E37" s="103"/>
-      <c r="F37" s="104"/>
-      <c r="G37" s="104"/>
-      <c r="H37" s="104"/>
-      <c r="I37" s="104"/>
-      <c r="J37" s="104"/>
-      <c r="K37" s="104"/>
-      <c r="L37" s="104"/>
-      <c r="M37" s="105"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="27"/>
+      <c r="E37" s="50"/>
+      <c r="F37" s="51"/>
+      <c r="G37" s="51"/>
+      <c r="H37" s="51"/>
+      <c r="I37" s="51"/>
+      <c r="J37" s="51"/>
+      <c r="K37" s="51"/>
+      <c r="L37" s="51"/>
+      <c r="M37" s="52"/>
     </row>
     <row r="38" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="36" t="s">
+      <c r="A38" s="151" t="s">
         <v>43</v>
       </c>
-      <c r="B38" s="36"/>
-      <c r="C38" s="36"/>
-      <c r="D38" s="36"/>
-      <c r="E38" s="36"/>
-      <c r="F38" s="36"/>
-      <c r="G38" s="36"/>
-      <c r="H38" s="36"/>
-      <c r="I38" s="36"/>
-      <c r="J38" s="36"/>
-      <c r="K38" s="36"/>
-      <c r="L38" s="36"/>
-      <c r="M38" s="36"/>
+      <c r="B38" s="151"/>
+      <c r="C38" s="151"/>
+      <c r="D38" s="151"/>
+      <c r="E38" s="151"/>
+      <c r="F38" s="151"/>
+      <c r="G38" s="151"/>
+      <c r="H38" s="151"/>
+      <c r="I38" s="151"/>
+      <c r="J38" s="151"/>
+      <c r="K38" s="151"/>
+      <c r="L38" s="151"/>
+      <c r="M38" s="151"/>
     </row>
     <row r="39" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="36"/>
-      <c r="B39" s="36"/>
-      <c r="C39" s="36"/>
-      <c r="D39" s="36"/>
-      <c r="E39" s="36"/>
-      <c r="F39" s="36"/>
-      <c r="G39" s="36"/>
-      <c r="H39" s="36"/>
-      <c r="I39" s="36"/>
-      <c r="J39" s="36"/>
-      <c r="K39" s="36"/>
-      <c r="L39" s="36"/>
-      <c r="M39" s="36"/>
+      <c r="A39" s="151"/>
+      <c r="B39" s="151"/>
+      <c r="C39" s="151"/>
+      <c r="D39" s="151"/>
+      <c r="E39" s="151"/>
+      <c r="F39" s="151"/>
+      <c r="G39" s="151"/>
+      <c r="H39" s="151"/>
+      <c r="I39" s="151"/>
+      <c r="J39" s="151"/>
+      <c r="K39" s="151"/>
+      <c r="L39" s="151"/>
+      <c r="M39" s="151"/>
     </row>
     <row r="40" spans="1:13" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="36"/>
-      <c r="B40" s="36"/>
-      <c r="C40" s="36"/>
-      <c r="D40" s="36"/>
-      <c r="E40" s="36"/>
-      <c r="F40" s="36"/>
-      <c r="G40" s="36"/>
-      <c r="H40" s="36"/>
-      <c r="I40" s="36"/>
-      <c r="J40" s="36"/>
-      <c r="K40" s="36"/>
-      <c r="L40" s="36"/>
-      <c r="M40" s="36"/>
+      <c r="A40" s="151"/>
+      <c r="B40" s="151"/>
+      <c r="C40" s="151"/>
+      <c r="D40" s="151"/>
+      <c r="E40" s="151"/>
+      <c r="F40" s="151"/>
+      <c r="G40" s="151"/>
+      <c r="H40" s="151"/>
+      <c r="I40" s="151"/>
+      <c r="J40" s="151"/>
+      <c r="K40" s="151"/>
+      <c r="L40" s="151"/>
+      <c r="M40" s="151"/>
     </row>
     <row r="41" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="37"/>
-      <c r="B41" s="37"/>
-      <c r="C41" s="37"/>
-      <c r="D41" s="37"/>
-      <c r="E41" s="37"/>
-      <c r="F41" s="37"/>
-      <c r="G41" s="37"/>
-      <c r="H41" s="37"/>
-      <c r="I41" s="37"/>
-      <c r="J41" s="37"/>
-      <c r="K41" s="37"/>
-      <c r="L41" s="37"/>
-      <c r="M41" s="37"/>
+      <c r="A41" s="152"/>
+      <c r="B41" s="152"/>
+      <c r="C41" s="152"/>
+      <c r="D41" s="152"/>
+      <c r="E41" s="152"/>
+      <c r="F41" s="152"/>
+      <c r="G41" s="152"/>
+      <c r="H41" s="152"/>
+      <c r="I41" s="152"/>
+      <c r="J41" s="152"/>
+      <c r="K41" s="152"/>
+      <c r="L41" s="152"/>
+      <c r="M41" s="152"/>
     </row>
     <row r="42" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="77" t="s">
+      <c r="A42" s="118" t="s">
         <v>114</v>
       </c>
-      <c r="B42" s="78"/>
-      <c r="C42" s="78"/>
-      <c r="D42" s="78"/>
-      <c r="E42" s="78"/>
-      <c r="F42" s="78"/>
-      <c r="G42" s="78"/>
-      <c r="H42" s="78"/>
-      <c r="I42" s="78"/>
-      <c r="J42" s="78"/>
-      <c r="K42" s="78"/>
-      <c r="L42" s="78"/>
-      <c r="M42" s="79"/>
+      <c r="B42" s="119"/>
+      <c r="C42" s="119"/>
+      <c r="D42" s="119"/>
+      <c r="E42" s="119"/>
+      <c r="F42" s="119"/>
+      <c r="G42" s="119"/>
+      <c r="H42" s="119"/>
+      <c r="I42" s="119"/>
+      <c r="J42" s="119"/>
+      <c r="K42" s="119"/>
+      <c r="L42" s="119"/>
+      <c r="M42" s="120"/>
     </row>
     <row r="43" spans="1:13" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="80" t="s">
+      <c r="A43" s="121" t="s">
         <v>44</v>
       </c>
-      <c r="B43" s="82"/>
-      <c r="C43" s="83"/>
-      <c r="D43" s="83"/>
-      <c r="E43" s="84"/>
-      <c r="F43" s="88" t="s">
+      <c r="B43" s="123"/>
+      <c r="C43" s="124"/>
+      <c r="D43" s="124"/>
+      <c r="E43" s="106"/>
+      <c r="F43" s="101" t="s">
         <v>45</v>
       </c>
-      <c r="G43" s="139"/>
-      <c r="H43" s="142"/>
-      <c r="I43" s="84"/>
-      <c r="J43" s="88" t="s">
+      <c r="G43" s="102"/>
+      <c r="H43" s="105"/>
+      <c r="I43" s="106"/>
+      <c r="J43" s="101" t="s">
         <v>46</v>
       </c>
-      <c r="K43" s="89"/>
-      <c r="L43" s="90"/>
-      <c r="M43" s="144"/>
+      <c r="K43" s="127"/>
+      <c r="L43" s="128"/>
+      <c r="M43" s="109"/>
     </row>
     <row r="44" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="81"/>
-      <c r="B44" s="85"/>
-      <c r="C44" s="86"/>
-      <c r="D44" s="86"/>
-      <c r="E44" s="87"/>
-      <c r="F44" s="140"/>
-      <c r="G44" s="141"/>
-      <c r="H44" s="143"/>
-      <c r="I44" s="87"/>
-      <c r="J44" s="91" t="s">
+      <c r="A44" s="122"/>
+      <c r="B44" s="125"/>
+      <c r="C44" s="126"/>
+      <c r="D44" s="126"/>
+      <c r="E44" s="108"/>
+      <c r="F44" s="103"/>
+      <c r="G44" s="104"/>
+      <c r="H44" s="107"/>
+      <c r="I44" s="108"/>
+      <c r="J44" s="129" t="s">
         <v>47</v>
       </c>
-      <c r="K44" s="92"/>
-      <c r="L44" s="93"/>
-      <c r="M44" s="145"/>
+      <c r="K44" s="130"/>
+      <c r="L44" s="131"/>
+      <c r="M44" s="110"/>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A45" s="38" t="s">
+      <c r="A45" s="91" t="s">
         <v>48</v>
       </c>
-      <c r="B45" s="58"/>
-      <c r="C45" s="39"/>
-      <c r="D45" s="65"/>
-      <c r="E45" s="66"/>
-      <c r="F45" s="66"/>
-      <c r="G45" s="67"/>
-      <c r="H45" s="38" t="s">
+      <c r="B45" s="111"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="169"/>
+      <c r="E45" s="170"/>
+      <c r="F45" s="170"/>
+      <c r="G45" s="96"/>
+      <c r="H45" s="91" t="s">
         <v>49</v>
       </c>
-      <c r="I45" s="58"/>
-      <c r="J45" s="58"/>
-      <c r="K45" s="74"/>
-      <c r="L45" s="172"/>
-      <c r="M45" s="67"/>
+      <c r="I45" s="111"/>
+      <c r="J45" s="111"/>
+      <c r="K45" s="112"/>
+      <c r="L45" s="95"/>
+      <c r="M45" s="96"/>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A46" s="59" t="s">
+      <c r="A46" s="113" t="s">
         <v>40</v>
       </c>
-      <c r="B46" s="60"/>
-      <c r="C46" s="61"/>
-      <c r="D46" s="68"/>
-      <c r="E46" s="69"/>
-      <c r="F46" s="69"/>
-      <c r="G46" s="70"/>
-      <c r="H46" s="59" t="s">
+      <c r="B46" s="78"/>
+      <c r="C46" s="167"/>
+      <c r="D46" s="171"/>
+      <c r="E46" s="172"/>
+      <c r="F46" s="172"/>
+      <c r="G46" s="98"/>
+      <c r="H46" s="113" t="s">
         <v>50</v>
       </c>
-      <c r="I46" s="60"/>
-      <c r="J46" s="60"/>
-      <c r="K46" s="75"/>
-      <c r="L46" s="173"/>
-      <c r="M46" s="70"/>
+      <c r="I46" s="78"/>
+      <c r="J46" s="78"/>
+      <c r="K46" s="114"/>
+      <c r="L46" s="97"/>
+      <c r="M46" s="98"/>
     </row>
     <row r="47" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="62"/>
-      <c r="B47" s="63"/>
-      <c r="C47" s="64"/>
-      <c r="D47" s="71"/>
-      <c r="E47" s="72"/>
-      <c r="F47" s="72"/>
-      <c r="G47" s="73"/>
-      <c r="H47" s="62"/>
-      <c r="I47" s="63"/>
-      <c r="J47" s="63"/>
-      <c r="K47" s="76"/>
-      <c r="L47" s="174"/>
-      <c r="M47" s="73"/>
+      <c r="A47" s="115"/>
+      <c r="B47" s="116"/>
+      <c r="C47" s="168"/>
+      <c r="D47" s="173"/>
+      <c r="E47" s="174"/>
+      <c r="F47" s="174"/>
+      <c r="G47" s="100"/>
+      <c r="H47" s="115"/>
+      <c r="I47" s="116"/>
+      <c r="J47" s="116"/>
+      <c r="K47" s="117"/>
+      <c r="L47" s="99"/>
+      <c r="M47" s="100"/>
     </row>
     <row r="48" spans="1:13" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="48" t="s">
+      <c r="A48" s="157" t="s">
         <v>51</v>
       </c>
-      <c r="B48" s="49"/>
-      <c r="C48" s="50"/>
-      <c r="D48" s="51"/>
-      <c r="E48" s="52"/>
-      <c r="F48" s="52"/>
-      <c r="G48" s="52"/>
-      <c r="H48" s="52"/>
-      <c r="I48" s="52"/>
-      <c r="J48" s="52"/>
-      <c r="K48" s="52"/>
-      <c r="L48" s="52"/>
-      <c r="M48" s="53"/>
+      <c r="B48" s="158"/>
+      <c r="C48" s="159"/>
+      <c r="D48" s="160"/>
+      <c r="E48" s="161"/>
+      <c r="F48" s="161"/>
+      <c r="G48" s="161"/>
+      <c r="H48" s="161"/>
+      <c r="I48" s="161"/>
+      <c r="J48" s="161"/>
+      <c r="K48" s="161"/>
+      <c r="L48" s="161"/>
+      <c r="M48" s="162"/>
     </row>
     <row r="49" spans="1:13" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="54" t="s">
+      <c r="A49" s="163" t="s">
         <v>52</v>
       </c>
-      <c r="B49" s="55"/>
-      <c r="C49" s="56"/>
-      <c r="D49" s="56"/>
-      <c r="E49" s="56"/>
-      <c r="F49" s="56"/>
-      <c r="G49" s="56"/>
-      <c r="H49" s="56"/>
-      <c r="I49" s="56"/>
-      <c r="J49" s="56"/>
-      <c r="K49" s="56"/>
-      <c r="L49" s="56"/>
-      <c r="M49" s="57"/>
+      <c r="B49" s="164"/>
+      <c r="C49" s="165"/>
+      <c r="D49" s="165"/>
+      <c r="E49" s="165"/>
+      <c r="F49" s="165"/>
+      <c r="G49" s="165"/>
+      <c r="H49" s="165"/>
+      <c r="I49" s="165"/>
+      <c r="J49" s="165"/>
+      <c r="K49" s="165"/>
+      <c r="L49" s="165"/>
+      <c r="M49" s="166"/>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A50" s="38" t="s">
+      <c r="A50" s="91" t="s">
         <v>53</v>
       </c>
-      <c r="B50" s="39"/>
-      <c r="C50" s="158"/>
-      <c r="D50" s="159"/>
-      <c r="E50" s="159"/>
-      <c r="F50" s="159"/>
-      <c r="G50" s="159"/>
-      <c r="H50" s="159"/>
-      <c r="I50" s="159"/>
-      <c r="J50" s="159"/>
-      <c r="K50" s="159"/>
-      <c r="L50" s="159"/>
-      <c r="M50" s="159"/>
+      <c r="B50" s="92"/>
+      <c r="C50" s="24"/>
+      <c r="D50" s="25"/>
+      <c r="E50" s="25"/>
+      <c r="F50" s="25"/>
+      <c r="G50" s="25"/>
+      <c r="H50" s="25"/>
+      <c r="I50" s="25"/>
+      <c r="J50" s="25"/>
+      <c r="K50" s="25"/>
+      <c r="L50" s="25"/>
+      <c r="M50" s="25"/>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A51" s="40"/>
-      <c r="B51" s="41"/>
-      <c r="C51" s="158"/>
-      <c r="D51" s="159"/>
-      <c r="E51" s="159"/>
-      <c r="F51" s="159"/>
-      <c r="G51" s="159"/>
-      <c r="H51" s="159"/>
-      <c r="I51" s="159"/>
-      <c r="J51" s="159"/>
-      <c r="K51" s="159"/>
-      <c r="L51" s="159"/>
-      <c r="M51" s="159"/>
+      <c r="A51" s="93"/>
+      <c r="B51" s="94"/>
+      <c r="C51" s="24"/>
+      <c r="D51" s="25"/>
+      <c r="E51" s="25"/>
+      <c r="F51" s="25"/>
+      <c r="G51" s="25"/>
+      <c r="H51" s="25"/>
+      <c r="I51" s="25"/>
+      <c r="J51" s="25"/>
+      <c r="K51" s="25"/>
+      <c r="L51" s="25"/>
+      <c r="M51" s="25"/>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A52" s="40"/>
-      <c r="B52" s="41"/>
-      <c r="C52" s="158"/>
-      <c r="D52" s="159"/>
-      <c r="E52" s="159"/>
-      <c r="F52" s="159"/>
-      <c r="G52" s="159"/>
-      <c r="H52" s="159"/>
-      <c r="I52" s="159"/>
-      <c r="J52" s="159"/>
-      <c r="K52" s="159"/>
-      <c r="L52" s="159"/>
-      <c r="M52" s="159"/>
+      <c r="A52" s="93"/>
+      <c r="B52" s="94"/>
+      <c r="C52" s="24"/>
+      <c r="D52" s="25"/>
+      <c r="E52" s="25"/>
+      <c r="F52" s="25"/>
+      <c r="G52" s="25"/>
+      <c r="H52" s="25"/>
+      <c r="I52" s="25"/>
+      <c r="J52" s="25"/>
+      <c r="K52" s="25"/>
+      <c r="L52" s="25"/>
+      <c r="M52" s="25"/>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A53" s="40"/>
-      <c r="B53" s="41"/>
-      <c r="C53" s="158"/>
-      <c r="D53" s="159"/>
-      <c r="E53" s="159"/>
-      <c r="F53" s="159"/>
-      <c r="G53" s="159"/>
-      <c r="H53" s="159"/>
-      <c r="I53" s="159"/>
-      <c r="J53" s="159"/>
-      <c r="K53" s="159"/>
-      <c r="L53" s="159"/>
-      <c r="M53" s="159"/>
+      <c r="A53" s="93"/>
+      <c r="B53" s="94"/>
+      <c r="C53" s="24"/>
+      <c r="D53" s="25"/>
+      <c r="E53" s="25"/>
+      <c r="F53" s="25"/>
+      <c r="G53" s="25"/>
+      <c r="H53" s="25"/>
+      <c r="I53" s="25"/>
+      <c r="J53" s="25"/>
+      <c r="K53" s="25"/>
+      <c r="L53" s="25"/>
+      <c r="M53" s="25"/>
     </row>
     <row r="54" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="42"/>
-      <c r="B54" s="43"/>
-      <c r="C54" s="158"/>
-      <c r="D54" s="159"/>
-      <c r="E54" s="159"/>
-      <c r="F54" s="159"/>
-      <c r="G54" s="159"/>
-      <c r="H54" s="159"/>
-      <c r="I54" s="159"/>
-      <c r="J54" s="159"/>
-      <c r="K54" s="159"/>
-      <c r="L54" s="159"/>
-      <c r="M54" s="159"/>
+      <c r="A54" s="44"/>
+      <c r="B54" s="45"/>
+      <c r="C54" s="24"/>
+      <c r="D54" s="25"/>
+      <c r="E54" s="25"/>
+      <c r="F54" s="25"/>
+      <c r="G54" s="25"/>
+      <c r="H54" s="25"/>
+      <c r="I54" s="25"/>
+      <c r="J54" s="25"/>
+      <c r="K54" s="25"/>
+      <c r="L54" s="25"/>
+      <c r="M54" s="25"/>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A55" s="38" t="s">
+      <c r="A55" s="91" t="s">
         <v>54</v>
       </c>
-      <c r="B55" s="39"/>
-      <c r="C55" s="158"/>
-      <c r="D55" s="159"/>
-      <c r="E55" s="159"/>
-      <c r="F55" s="159"/>
-      <c r="G55" s="159"/>
-      <c r="H55" s="159"/>
-      <c r="I55" s="159"/>
-      <c r="J55" s="159"/>
-      <c r="K55" s="159"/>
-      <c r="L55" s="159"/>
-      <c r="M55" s="159"/>
+      <c r="B55" s="92"/>
+      <c r="C55" s="24"/>
+      <c r="D55" s="25"/>
+      <c r="E55" s="25"/>
+      <c r="F55" s="25"/>
+      <c r="G55" s="25"/>
+      <c r="H55" s="25"/>
+      <c r="I55" s="25"/>
+      <c r="J55" s="25"/>
+      <c r="K55" s="25"/>
+      <c r="L55" s="25"/>
+      <c r="M55" s="25"/>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A56" s="40"/>
-      <c r="B56" s="41"/>
-      <c r="C56" s="158"/>
-      <c r="D56" s="159"/>
-      <c r="E56" s="159"/>
-      <c r="F56" s="159"/>
-      <c r="G56" s="159"/>
-      <c r="H56" s="159"/>
-      <c r="I56" s="159"/>
-      <c r="J56" s="159"/>
-      <c r="K56" s="159"/>
-      <c r="L56" s="159"/>
-      <c r="M56" s="159"/>
+      <c r="A56" s="93"/>
+      <c r="B56" s="94"/>
+      <c r="C56" s="24"/>
+      <c r="D56" s="25"/>
+      <c r="E56" s="25"/>
+      <c r="F56" s="25"/>
+      <c r="G56" s="25"/>
+      <c r="H56" s="25"/>
+      <c r="I56" s="25"/>
+      <c r="J56" s="25"/>
+      <c r="K56" s="25"/>
+      <c r="L56" s="25"/>
+      <c r="M56" s="25"/>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A57" s="40"/>
-      <c r="B57" s="41"/>
-      <c r="C57" s="158"/>
-      <c r="D57" s="159"/>
-      <c r="E57" s="159"/>
-      <c r="F57" s="159"/>
-      <c r="G57" s="159"/>
-      <c r="H57" s="159"/>
-      <c r="I57" s="159"/>
-      <c r="J57" s="159"/>
-      <c r="K57" s="159"/>
-      <c r="L57" s="159"/>
-      <c r="M57" s="159"/>
+      <c r="A57" s="93"/>
+      <c r="B57" s="94"/>
+      <c r="C57" s="24"/>
+      <c r="D57" s="25"/>
+      <c r="E57" s="25"/>
+      <c r="F57" s="25"/>
+      <c r="G57" s="25"/>
+      <c r="H57" s="25"/>
+      <c r="I57" s="25"/>
+      <c r="J57" s="25"/>
+      <c r="K57" s="25"/>
+      <c r="L57" s="25"/>
+      <c r="M57" s="25"/>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A58" s="40"/>
-      <c r="B58" s="41"/>
-      <c r="C58" s="158"/>
-      <c r="D58" s="159"/>
-      <c r="E58" s="159"/>
-      <c r="F58" s="159"/>
-      <c r="G58" s="159"/>
-      <c r="H58" s="159"/>
-      <c r="I58" s="159"/>
-      <c r="J58" s="159"/>
-      <c r="K58" s="159"/>
-      <c r="L58" s="159"/>
-      <c r="M58" s="159"/>
+      <c r="A58" s="93"/>
+      <c r="B58" s="94"/>
+      <c r="C58" s="24"/>
+      <c r="D58" s="25"/>
+      <c r="E58" s="25"/>
+      <c r="F58" s="25"/>
+      <c r="G58" s="25"/>
+      <c r="H58" s="25"/>
+      <c r="I58" s="25"/>
+      <c r="J58" s="25"/>
+      <c r="K58" s="25"/>
+      <c r="L58" s="25"/>
+      <c r="M58" s="25"/>
     </row>
     <row r="59" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="42"/>
-      <c r="B59" s="43"/>
-      <c r="C59" s="158"/>
-      <c r="D59" s="159"/>
-      <c r="E59" s="159"/>
-      <c r="F59" s="159"/>
-      <c r="G59" s="159"/>
-      <c r="H59" s="159"/>
-      <c r="I59" s="159"/>
-      <c r="J59" s="159"/>
-      <c r="K59" s="159"/>
-      <c r="L59" s="159"/>
-      <c r="M59" s="159"/>
+      <c r="A59" s="44"/>
+      <c r="B59" s="45"/>
+      <c r="C59" s="24"/>
+      <c r="D59" s="25"/>
+      <c r="E59" s="25"/>
+      <c r="F59" s="25"/>
+      <c r="G59" s="25"/>
+      <c r="H59" s="25"/>
+      <c r="I59" s="25"/>
+      <c r="J59" s="25"/>
+      <c r="K59" s="25"/>
+      <c r="L59" s="25"/>
+      <c r="M59" s="25"/>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A60" s="38" t="s">
+      <c r="A60" s="91" t="s">
         <v>55</v>
       </c>
-      <c r="B60" s="39"/>
-      <c r="C60" s="158"/>
-      <c r="D60" s="159"/>
-      <c r="E60" s="159"/>
-      <c r="F60" s="159"/>
-      <c r="G60" s="159"/>
-      <c r="H60" s="159"/>
-      <c r="I60" s="159"/>
-      <c r="J60" s="159"/>
-      <c r="K60" s="159"/>
-      <c r="L60" s="159"/>
-      <c r="M60" s="159"/>
+      <c r="B60" s="92"/>
+      <c r="C60" s="24"/>
+      <c r="D60" s="25"/>
+      <c r="E60" s="25"/>
+      <c r="F60" s="25"/>
+      <c r="G60" s="25"/>
+      <c r="H60" s="25"/>
+      <c r="I60" s="25"/>
+      <c r="J60" s="25"/>
+      <c r="K60" s="25"/>
+      <c r="L60" s="25"/>
+      <c r="M60" s="25"/>
     </row>
     <row r="61" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="40"/>
-      <c r="B61" s="41"/>
-      <c r="C61" s="158"/>
-      <c r="D61" s="159"/>
-      <c r="E61" s="159"/>
-      <c r="F61" s="159"/>
-      <c r="G61" s="159"/>
-      <c r="H61" s="159"/>
-      <c r="I61" s="159"/>
-      <c r="J61" s="159"/>
-      <c r="K61" s="159"/>
-      <c r="L61" s="159"/>
-      <c r="M61" s="159"/>
+      <c r="A61" s="93"/>
+      <c r="B61" s="94"/>
+      <c r="C61" s="24"/>
+      <c r="D61" s="25"/>
+      <c r="E61" s="25"/>
+      <c r="F61" s="25"/>
+      <c r="G61" s="25"/>
+      <c r="H61" s="25"/>
+      <c r="I61" s="25"/>
+      <c r="J61" s="25"/>
+      <c r="K61" s="25"/>
+      <c r="L61" s="25"/>
+      <c r="M61" s="25"/>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A62" s="40"/>
-      <c r="B62" s="41"/>
-      <c r="C62" s="158"/>
-      <c r="D62" s="159"/>
-      <c r="E62" s="159"/>
-      <c r="F62" s="159"/>
-      <c r="G62" s="159"/>
-      <c r="H62" s="159"/>
-      <c r="I62" s="159"/>
-      <c r="J62" s="159"/>
-      <c r="K62" s="159"/>
-      <c r="L62" s="159"/>
-      <c r="M62" s="159"/>
+      <c r="A62" s="93"/>
+      <c r="B62" s="94"/>
+      <c r="C62" s="24"/>
+      <c r="D62" s="25"/>
+      <c r="E62" s="25"/>
+      <c r="F62" s="25"/>
+      <c r="G62" s="25"/>
+      <c r="H62" s="25"/>
+      <c r="I62" s="25"/>
+      <c r="J62" s="25"/>
+      <c r="K62" s="25"/>
+      <c r="L62" s="25"/>
+      <c r="M62" s="25"/>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A63" s="40"/>
-      <c r="B63" s="41"/>
-      <c r="C63" s="158"/>
-      <c r="D63" s="159"/>
-      <c r="E63" s="159"/>
-      <c r="F63" s="159"/>
-      <c r="G63" s="159"/>
-      <c r="H63" s="159"/>
-      <c r="I63" s="159"/>
-      <c r="J63" s="159"/>
-      <c r="K63" s="159"/>
-      <c r="L63" s="159"/>
-      <c r="M63" s="159"/>
+      <c r="A63" s="93"/>
+      <c r="B63" s="94"/>
+      <c r="C63" s="24"/>
+      <c r="D63" s="25"/>
+      <c r="E63" s="25"/>
+      <c r="F63" s="25"/>
+      <c r="G63" s="25"/>
+      <c r="H63" s="25"/>
+      <c r="I63" s="25"/>
+      <c r="J63" s="25"/>
+      <c r="K63" s="25"/>
+      <c r="L63" s="25"/>
+      <c r="M63" s="25"/>
     </row>
     <row r="64" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="42"/>
-      <c r="B64" s="43"/>
-      <c r="C64" s="158"/>
-      <c r="D64" s="159"/>
-      <c r="E64" s="159"/>
-      <c r="F64" s="159"/>
-      <c r="G64" s="159"/>
-      <c r="H64" s="159"/>
-      <c r="I64" s="159"/>
-      <c r="J64" s="159"/>
-      <c r="K64" s="159"/>
-      <c r="L64" s="159"/>
-      <c r="M64" s="159"/>
+      <c r="A64" s="44"/>
+      <c r="B64" s="45"/>
+      <c r="C64" s="24"/>
+      <c r="D64" s="25"/>
+      <c r="E64" s="25"/>
+      <c r="F64" s="25"/>
+      <c r="G64" s="25"/>
+      <c r="H64" s="25"/>
+      <c r="I64" s="25"/>
+      <c r="J64" s="25"/>
+      <c r="K64" s="25"/>
+      <c r="L64" s="25"/>
+      <c r="M64" s="25"/>
     </row>
     <row r="65" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="38" t="s">
+      <c r="A65" s="91" t="s">
         <v>56</v>
       </c>
-      <c r="B65" s="39"/>
-      <c r="C65" s="131"/>
-      <c r="D65" s="132"/>
-      <c r="E65" s="132"/>
-      <c r="F65" s="132"/>
-      <c r="G65" s="132"/>
-      <c r="H65" s="132"/>
-      <c r="I65" s="132"/>
-      <c r="J65" s="132"/>
-      <c r="K65" s="132"/>
-      <c r="L65" s="132"/>
-      <c r="M65" s="133"/>
+      <c r="B65" s="92"/>
+      <c r="C65" s="83"/>
+      <c r="D65" s="84"/>
+      <c r="E65" s="84"/>
+      <c r="F65" s="84"/>
+      <c r="G65" s="84"/>
+      <c r="H65" s="84"/>
+      <c r="I65" s="84"/>
+      <c r="J65" s="84"/>
+      <c r="K65" s="84"/>
+      <c r="L65" s="84"/>
+      <c r="M65" s="85"/>
     </row>
     <row r="66" spans="1:13" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="42"/>
-      <c r="B66" s="43"/>
-      <c r="C66" s="134"/>
-      <c r="D66" s="135"/>
-      <c r="E66" s="135"/>
-      <c r="F66" s="135"/>
-      <c r="G66" s="135"/>
-      <c r="H66" s="135"/>
-      <c r="I66" s="135"/>
-      <c r="J66" s="135"/>
-      <c r="K66" s="135"/>
-      <c r="L66" s="135"/>
-      <c r="M66" s="136"/>
+      <c r="A66" s="44"/>
+      <c r="B66" s="45"/>
+      <c r="C66" s="86"/>
+      <c r="D66" s="87"/>
+      <c r="E66" s="87"/>
+      <c r="F66" s="87"/>
+      <c r="G66" s="87"/>
+      <c r="H66" s="87"/>
+      <c r="I66" s="87"/>
+      <c r="J66" s="87"/>
+      <c r="K66" s="87"/>
+      <c r="L66" s="87"/>
+      <c r="M66" s="88"/>
     </row>
     <row r="67" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="38" t="s">
+      <c r="A67" s="91" t="s">
         <v>57</v>
       </c>
-      <c r="B67" s="39"/>
-      <c r="C67" s="128"/>
-      <c r="D67" s="129"/>
-      <c r="E67" s="129"/>
-      <c r="F67" s="129"/>
-      <c r="G67" s="129"/>
-      <c r="H67" s="129"/>
-      <c r="I67" s="129"/>
-      <c r="J67" s="129"/>
-      <c r="K67" s="129"/>
-      <c r="L67" s="129"/>
-      <c r="M67" s="130"/>
+      <c r="B67" s="92"/>
+      <c r="C67" s="80"/>
+      <c r="D67" s="81"/>
+      <c r="E67" s="81"/>
+      <c r="F67" s="81"/>
+      <c r="G67" s="81"/>
+      <c r="H67" s="81"/>
+      <c r="I67" s="81"/>
+      <c r="J67" s="81"/>
+      <c r="K67" s="81"/>
+      <c r="L67" s="81"/>
+      <c r="M67" s="82"/>
     </row>
     <row r="68" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="40"/>
-      <c r="B68" s="41"/>
-      <c r="C68" s="131"/>
-      <c r="D68" s="132"/>
-      <c r="E68" s="132"/>
-      <c r="F68" s="132"/>
-      <c r="G68" s="132"/>
-      <c r="H68" s="132"/>
-      <c r="I68" s="132"/>
-      <c r="J68" s="132"/>
-      <c r="K68" s="132"/>
-      <c r="L68" s="132"/>
-      <c r="M68" s="133"/>
+      <c r="A68" s="93"/>
+      <c r="B68" s="94"/>
+      <c r="C68" s="83"/>
+      <c r="D68" s="84"/>
+      <c r="E68" s="84"/>
+      <c r="F68" s="84"/>
+      <c r="G68" s="84"/>
+      <c r="H68" s="84"/>
+      <c r="I68" s="84"/>
+      <c r="J68" s="84"/>
+      <c r="K68" s="84"/>
+      <c r="L68" s="84"/>
+      <c r="M68" s="85"/>
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A69" s="40"/>
-      <c r="B69" s="41"/>
-      <c r="C69" s="131"/>
-      <c r="D69" s="132"/>
-      <c r="E69" s="132"/>
-      <c r="F69" s="132"/>
-      <c r="G69" s="132"/>
-      <c r="H69" s="132"/>
-      <c r="I69" s="132"/>
-      <c r="J69" s="132"/>
-      <c r="K69" s="132"/>
-      <c r="L69" s="132"/>
-      <c r="M69" s="133"/>
+      <c r="A69" s="93"/>
+      <c r="B69" s="94"/>
+      <c r="C69" s="83"/>
+      <c r="D69" s="84"/>
+      <c r="E69" s="84"/>
+      <c r="F69" s="84"/>
+      <c r="G69" s="84"/>
+      <c r="H69" s="84"/>
+      <c r="I69" s="84"/>
+      <c r="J69" s="84"/>
+      <c r="K69" s="84"/>
+      <c r="L69" s="84"/>
+      <c r="M69" s="85"/>
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A70" s="40"/>
-      <c r="B70" s="41"/>
-      <c r="C70" s="131"/>
-      <c r="D70" s="132"/>
-      <c r="E70" s="132"/>
-      <c r="F70" s="132"/>
-      <c r="G70" s="132"/>
-      <c r="H70" s="132"/>
-      <c r="I70" s="132"/>
-      <c r="J70" s="132"/>
-      <c r="K70" s="132"/>
-      <c r="L70" s="132"/>
-      <c r="M70" s="133"/>
+      <c r="A70" s="93"/>
+      <c r="B70" s="94"/>
+      <c r="C70" s="83"/>
+      <c r="D70" s="84"/>
+      <c r="E70" s="84"/>
+      <c r="F70" s="84"/>
+      <c r="G70" s="84"/>
+      <c r="H70" s="84"/>
+      <c r="I70" s="84"/>
+      <c r="J70" s="84"/>
+      <c r="K70" s="84"/>
+      <c r="L70" s="84"/>
+      <c r="M70" s="85"/>
     </row>
     <row r="71" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="42"/>
-      <c r="B71" s="43"/>
-      <c r="C71" s="134"/>
-      <c r="D71" s="135"/>
-      <c r="E71" s="135"/>
-      <c r="F71" s="135"/>
-      <c r="G71" s="135"/>
-      <c r="H71" s="135"/>
-      <c r="I71" s="135"/>
-      <c r="J71" s="135"/>
-      <c r="K71" s="135"/>
-      <c r="L71" s="135"/>
-      <c r="M71" s="136"/>
+      <c r="A71" s="44"/>
+      <c r="B71" s="45"/>
+      <c r="C71" s="86"/>
+      <c r="D71" s="87"/>
+      <c r="E71" s="87"/>
+      <c r="F71" s="87"/>
+      <c r="G71" s="87"/>
+      <c r="H71" s="87"/>
+      <c r="I71" s="87"/>
+      <c r="J71" s="87"/>
+      <c r="K71" s="87"/>
+      <c r="L71" s="87"/>
+      <c r="M71" s="88"/>
     </row>
     <row r="72" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A72" s="137"/>
-      <c r="B72" s="137"/>
-      <c r="C72" s="137"/>
-      <c r="D72" s="137"/>
-      <c r="E72" s="60"/>
-      <c r="F72" s="60"/>
-      <c r="G72" s="137"/>
-      <c r="H72" s="137"/>
-      <c r="I72" s="60"/>
-      <c r="J72" s="60"/>
-      <c r="K72" s="137"/>
-      <c r="L72" s="137"/>
-      <c r="M72" s="137"/>
+      <c r="A72" s="89"/>
+      <c r="B72" s="89"/>
+      <c r="C72" s="89"/>
+      <c r="D72" s="89"/>
+      <c r="E72" s="78"/>
+      <c r="F72" s="78"/>
+      <c r="G72" s="89"/>
+      <c r="H72" s="89"/>
+      <c r="I72" s="78"/>
+      <c r="J72" s="78"/>
+      <c r="K72" s="89"/>
+      <c r="L72" s="89"/>
+      <c r="M72" s="89"/>
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A73" s="137"/>
-      <c r="B73" s="137"/>
-      <c r="C73" s="137"/>
-      <c r="D73" s="137"/>
-      <c r="E73" s="60"/>
-      <c r="F73" s="60"/>
-      <c r="G73" s="137"/>
-      <c r="H73" s="137"/>
-      <c r="I73" s="60"/>
-      <c r="J73" s="60"/>
-      <c r="K73" s="137"/>
-      <c r="L73" s="137"/>
-      <c r="M73" s="137"/>
+      <c r="A73" s="89"/>
+      <c r="B73" s="89"/>
+      <c r="C73" s="89"/>
+      <c r="D73" s="89"/>
+      <c r="E73" s="78"/>
+      <c r="F73" s="78"/>
+      <c r="G73" s="89"/>
+      <c r="H73" s="89"/>
+      <c r="I73" s="78"/>
+      <c r="J73" s="78"/>
+      <c r="K73" s="89"/>
+      <c r="L73" s="89"/>
+      <c r="M73" s="89"/>
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A74" s="137"/>
-      <c r="B74" s="137"/>
-      <c r="C74" s="137"/>
-      <c r="D74" s="137"/>
-      <c r="E74" s="60"/>
-      <c r="F74" s="60"/>
-      <c r="G74" s="137"/>
-      <c r="H74" s="137"/>
-      <c r="I74" s="60"/>
-      <c r="J74" s="60"/>
-      <c r="K74" s="137"/>
-      <c r="L74" s="137"/>
-      <c r="M74" s="137"/>
+      <c r="A74" s="89"/>
+      <c r="B74" s="89"/>
+      <c r="C74" s="89"/>
+      <c r="D74" s="89"/>
+      <c r="E74" s="78"/>
+      <c r="F74" s="78"/>
+      <c r="G74" s="89"/>
+      <c r="H74" s="89"/>
+      <c r="I74" s="78"/>
+      <c r="J74" s="78"/>
+      <c r="K74" s="89"/>
+      <c r="L74" s="89"/>
+      <c r="M74" s="89"/>
     </row>
     <row r="75" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A75" s="137"/>
-      <c r="B75" s="137"/>
-      <c r="C75" s="137"/>
-      <c r="D75" s="137"/>
-      <c r="E75" s="60"/>
-      <c r="F75" s="60"/>
-      <c r="G75" s="137"/>
-      <c r="H75" s="137"/>
-      <c r="I75" s="60"/>
-      <c r="J75" s="60"/>
-      <c r="K75" s="137"/>
-      <c r="L75" s="137"/>
-      <c r="M75" s="137"/>
+      <c r="A75" s="89"/>
+      <c r="B75" s="89"/>
+      <c r="C75" s="89"/>
+      <c r="D75" s="89"/>
+      <c r="E75" s="78"/>
+      <c r="F75" s="78"/>
+      <c r="G75" s="89"/>
+      <c r="H75" s="89"/>
+      <c r="I75" s="78"/>
+      <c r="J75" s="78"/>
+      <c r="K75" s="89"/>
+      <c r="L75" s="89"/>
+      <c r="M75" s="89"/>
     </row>
     <row r="76" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A76" s="137"/>
-      <c r="B76" s="137"/>
-      <c r="C76" s="137"/>
-      <c r="D76" s="137"/>
-      <c r="E76" s="60"/>
-      <c r="F76" s="60"/>
-      <c r="G76" s="137"/>
-      <c r="H76" s="137"/>
-      <c r="I76" s="60"/>
-      <c r="J76" s="60"/>
-      <c r="K76" s="137"/>
-      <c r="L76" s="137"/>
-      <c r="M76" s="137"/>
+      <c r="A76" s="89"/>
+      <c r="B76" s="89"/>
+      <c r="C76" s="89"/>
+      <c r="D76" s="89"/>
+      <c r="E76" s="78"/>
+      <c r="F76" s="78"/>
+      <c r="G76" s="89"/>
+      <c r="H76" s="89"/>
+      <c r="I76" s="78"/>
+      <c r="J76" s="78"/>
+      <c r="K76" s="89"/>
+      <c r="L76" s="89"/>
+      <c r="M76" s="89"/>
     </row>
     <row r="77" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="138"/>
-      <c r="B77" s="138"/>
-      <c r="C77" s="138"/>
-      <c r="D77" s="138"/>
-      <c r="E77" s="60"/>
-      <c r="F77" s="60"/>
-      <c r="G77" s="138"/>
-      <c r="H77" s="138"/>
-      <c r="I77" s="60"/>
-      <c r="J77" s="60"/>
-      <c r="K77" s="138"/>
-      <c r="L77" s="138"/>
-      <c r="M77" s="138"/>
+      <c r="A77" s="90"/>
+      <c r="B77" s="90"/>
+      <c r="C77" s="90"/>
+      <c r="D77" s="90"/>
+      <c r="E77" s="78"/>
+      <c r="F77" s="78"/>
+      <c r="G77" s="90"/>
+      <c r="H77" s="90"/>
+      <c r="I77" s="78"/>
+      <c r="J77" s="78"/>
+      <c r="K77" s="90"/>
+      <c r="L77" s="90"/>
+      <c r="M77" s="90"/>
     </row>
     <row r="78" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="126"/>
-      <c r="B78" s="126"/>
-      <c r="C78" s="126"/>
-      <c r="D78" s="126"/>
-      <c r="E78" s="60"/>
-      <c r="F78" s="60"/>
-      <c r="G78" s="127" t="s">
+      <c r="A78" s="77"/>
+      <c r="B78" s="77"/>
+      <c r="C78" s="77"/>
+      <c r="D78" s="77"/>
+      <c r="E78" s="78"/>
+      <c r="F78" s="78"/>
+      <c r="G78" s="79" t="s">
         <v>27</v>
       </c>
-      <c r="H78" s="127"/>
-      <c r="I78" s="60"/>
-      <c r="J78" s="60"/>
-      <c r="K78" s="126"/>
-      <c r="L78" s="126"/>
-      <c r="M78" s="126"/>
+      <c r="H78" s="79"/>
+      <c r="I78" s="78"/>
+      <c r="J78" s="78"/>
+      <c r="K78" s="77"/>
+      <c r="L78" s="77"/>
+      <c r="M78" s="77"/>
     </row>
     <row r="79" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A79" s="11"/>
@@ -3766,35 +3766,125 @@
     </row>
     <row r="80" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A80" s="12"/>
-      <c r="C80" s="44"/>
-      <c r="D80" s="44"/>
-      <c r="E80" s="44"/>
-      <c r="F80" s="44"/>
-      <c r="G80" s="44"/>
-      <c r="H80" s="44"/>
-      <c r="I80" s="44"/>
-      <c r="J80" s="44"/>
+      <c r="C80" s="153"/>
+      <c r="D80" s="153"/>
+      <c r="E80" s="153"/>
+      <c r="F80" s="153"/>
+      <c r="G80" s="153"/>
+      <c r="H80" s="153"/>
+      <c r="I80" s="153"/>
+      <c r="J80" s="153"/>
     </row>
     <row r="81" spans="6:7" x14ac:dyDescent="0.25">
-      <c r="F81" s="34" t="s">
+      <c r="F81" s="149" t="s">
         <v>58</v>
       </c>
-      <c r="G81" s="34"/>
+      <c r="G81" s="149"/>
     </row>
     <row r="82" spans="6:7" x14ac:dyDescent="0.25"/>
     <row r="83" spans="6:7" x14ac:dyDescent="0.25"/>
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="132">
-    <mergeCell ref="C56:M56"/>
-    <mergeCell ref="C57:M57"/>
-    <mergeCell ref="C58:M58"/>
-    <mergeCell ref="C59:M59"/>
-    <mergeCell ref="C60:M60"/>
-    <mergeCell ref="C61:M61"/>
-    <mergeCell ref="C62:M62"/>
-    <mergeCell ref="C63:M63"/>
-    <mergeCell ref="C64:M64"/>
+    <mergeCell ref="B1:K1"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="B5:K5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="B4:K4"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="F81:G81"/>
+    <mergeCell ref="A38:M40"/>
+    <mergeCell ref="A41:M41"/>
+    <mergeCell ref="A60:B64"/>
+    <mergeCell ref="A65:B66"/>
+    <mergeCell ref="A67:B71"/>
+    <mergeCell ref="C80:J80"/>
+    <mergeCell ref="I10:M10"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="D48:M48"/>
+    <mergeCell ref="A49:M49"/>
+    <mergeCell ref="A50:B54"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="D45:G47"/>
+    <mergeCell ref="H45:K45"/>
+    <mergeCell ref="H46:K46"/>
+    <mergeCell ref="H47:K47"/>
+    <mergeCell ref="A42:M42"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="B43:E44"/>
+    <mergeCell ref="J43:L43"/>
+    <mergeCell ref="J44:L44"/>
+    <mergeCell ref="C9:M9"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="E35:M35"/>
+    <mergeCell ref="E36:M36"/>
+    <mergeCell ref="E37:M37"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="E32:M32"/>
+    <mergeCell ref="E33:M33"/>
+    <mergeCell ref="E34:M34"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="A8:M8"/>
+    <mergeCell ref="E14:M14"/>
+    <mergeCell ref="K11:M11"/>
+    <mergeCell ref="K12:M12"/>
+    <mergeCell ref="J13:M13"/>
+    <mergeCell ref="E15:M15"/>
+    <mergeCell ref="E16:M16"/>
+    <mergeCell ref="A78:D78"/>
+    <mergeCell ref="E78:F78"/>
+    <mergeCell ref="G78:H78"/>
+    <mergeCell ref="I78:J78"/>
+    <mergeCell ref="K78:M78"/>
+    <mergeCell ref="C67:M71"/>
+    <mergeCell ref="A72:D77"/>
+    <mergeCell ref="E72:F77"/>
+    <mergeCell ref="G72:H77"/>
+    <mergeCell ref="I72:J77"/>
+    <mergeCell ref="K72:M77"/>
+    <mergeCell ref="C65:M66"/>
+    <mergeCell ref="A55:B59"/>
+    <mergeCell ref="L45:M47"/>
+    <mergeCell ref="F43:G44"/>
+    <mergeCell ref="H43:I44"/>
+    <mergeCell ref="M43:M44"/>
+    <mergeCell ref="E29:M29"/>
+    <mergeCell ref="E30:M30"/>
+    <mergeCell ref="E31:M31"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="E26:M26"/>
+    <mergeCell ref="E27:M27"/>
+    <mergeCell ref="E28:M28"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="E23:M23"/>
+    <mergeCell ref="E24:M24"/>
+    <mergeCell ref="E25:M25"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E20:M20"/>
+    <mergeCell ref="E21:M21"/>
+    <mergeCell ref="E22:M22"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="E17:M17"/>
+    <mergeCell ref="E18:M18"/>
+    <mergeCell ref="E19:M19"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="C10:G10"/>
@@ -3819,105 +3909,15 @@
     <mergeCell ref="F12:G12"/>
     <mergeCell ref="I12:J12"/>
     <mergeCell ref="B20:D20"/>
-    <mergeCell ref="E20:M20"/>
-    <mergeCell ref="E21:M21"/>
-    <mergeCell ref="E22:M22"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="E17:M17"/>
-    <mergeCell ref="E18:M18"/>
-    <mergeCell ref="E19:M19"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="E23:M23"/>
-    <mergeCell ref="E24:M24"/>
-    <mergeCell ref="E25:M25"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="E29:M29"/>
-    <mergeCell ref="E30:M30"/>
-    <mergeCell ref="E31:M31"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="E26:M26"/>
-    <mergeCell ref="E27:M27"/>
-    <mergeCell ref="E28:M28"/>
-    <mergeCell ref="A8:M8"/>
-    <mergeCell ref="E14:M14"/>
-    <mergeCell ref="K11:M11"/>
-    <mergeCell ref="K12:M12"/>
-    <mergeCell ref="J13:M13"/>
-    <mergeCell ref="E15:M15"/>
-    <mergeCell ref="E16:M16"/>
-    <mergeCell ref="A78:D78"/>
-    <mergeCell ref="E78:F78"/>
-    <mergeCell ref="G78:H78"/>
-    <mergeCell ref="I78:J78"/>
-    <mergeCell ref="K78:M78"/>
-    <mergeCell ref="C67:M71"/>
-    <mergeCell ref="A72:D77"/>
-    <mergeCell ref="E72:F77"/>
-    <mergeCell ref="G72:H77"/>
-    <mergeCell ref="I72:J77"/>
-    <mergeCell ref="K72:M77"/>
-    <mergeCell ref="C65:M66"/>
-    <mergeCell ref="A55:B59"/>
-    <mergeCell ref="L45:M47"/>
-    <mergeCell ref="F43:G44"/>
-    <mergeCell ref="H43:I44"/>
-    <mergeCell ref="M43:M44"/>
-    <mergeCell ref="H45:K45"/>
-    <mergeCell ref="H46:K46"/>
-    <mergeCell ref="H47:K47"/>
-    <mergeCell ref="A42:M42"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="B43:E44"/>
-    <mergeCell ref="J43:L43"/>
-    <mergeCell ref="J44:L44"/>
-    <mergeCell ref="C9:M9"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="E35:M35"/>
-    <mergeCell ref="E36:M36"/>
-    <mergeCell ref="E37:M37"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="E32:M32"/>
-    <mergeCell ref="E33:M33"/>
-    <mergeCell ref="E34:M34"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="B1:K1"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="B5:K5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="B4:K4"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="F81:G81"/>
-    <mergeCell ref="A38:M40"/>
-    <mergeCell ref="A41:M41"/>
-    <mergeCell ref="A60:B64"/>
-    <mergeCell ref="A65:B66"/>
-    <mergeCell ref="A67:B71"/>
-    <mergeCell ref="C80:J80"/>
-    <mergeCell ref="I10:M10"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="D48:M48"/>
-    <mergeCell ref="A49:M49"/>
-    <mergeCell ref="A50:B54"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="D45:G47"/>
+    <mergeCell ref="C56:M56"/>
+    <mergeCell ref="C57:M57"/>
+    <mergeCell ref="C58:M58"/>
+    <mergeCell ref="C59:M59"/>
+    <mergeCell ref="C60:M60"/>
+    <mergeCell ref="C61:M61"/>
+    <mergeCell ref="C62:M62"/>
+    <mergeCell ref="C63:M63"/>
+    <mergeCell ref="C64:M64"/>
   </mergeCells>
   <conditionalFormatting sqref="A78:D78">
     <cfRule type="containsBlanks" dxfId="3" priority="2">

</xml_diff>

<commit_message>
Actualiza Formatos: visitas GFPI-F023
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Formatos/Visita 1 GFPI-F023.xlsx
+++ b/Formatos/Visita 1 GFPI-F023.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SEANT\OneDrive\Documents\Seto 2026\sena\Manual SENA Etapa Productiva\manual-aprendiz-sena\Formatos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7298B0B-D518-46BF-A6D4-8320B0565BBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83A521C4-0D45-4A49-857A-DD8313A422E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BC3553EE-4E49-4F2A-B03E-CFAC4EB3009B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BC3553EE-4E49-4F2A-B03E-CFAC4EB3009B}"/>
   </bookViews>
   <sheets>
     <sheet name="Formato Visita 1" sheetId="1" r:id="rId1"/>
-    <sheet name="BD_SENA" sheetId="5" r:id="rId2"/>
+    <sheet name="BD_SENA" sheetId="5" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="Análisis_y_Desarrollo_de_Software">#REF!</definedName>
@@ -1295,7 +1295,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="175">
+  <cellXfs count="178">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
@@ -1620,6 +1620,255 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1627,7 +1876,11 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1635,256 +1888,15 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="justify" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="justify" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="justify" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -3224,7 +3236,7 @@
       <c r="D45" s="169"/>
       <c r="E45" s="170"/>
       <c r="F45" s="170"/>
-      <c r="G45" s="96"/>
+      <c r="G45" s="171"/>
       <c r="H45" s="91" t="s">
         <v>49</v>
       </c>
@@ -3240,10 +3252,10 @@
       </c>
       <c r="B46" s="78"/>
       <c r="C46" s="167"/>
-      <c r="D46" s="171"/>
-      <c r="E46" s="172"/>
-      <c r="F46" s="172"/>
-      <c r="G46" s="98"/>
+      <c r="D46" s="172"/>
+      <c r="E46" s="173"/>
+      <c r="F46" s="173"/>
+      <c r="G46" s="174"/>
       <c r="H46" s="113" t="s">
         <v>50</v>
       </c>
@@ -3257,10 +3269,10 @@
       <c r="A47" s="115"/>
       <c r="B47" s="116"/>
       <c r="C47" s="168"/>
-      <c r="D47" s="173"/>
-      <c r="E47" s="174"/>
-      <c r="F47" s="174"/>
-      <c r="G47" s="100"/>
+      <c r="D47" s="175"/>
+      <c r="E47" s="176"/>
+      <c r="F47" s="176"/>
+      <c r="G47" s="177"/>
       <c r="H47" s="115"/>
       <c r="I47" s="116"/>
       <c r="J47" s="116"/>
@@ -3784,7 +3796,6 @@
     <row r="82" spans="6:7" x14ac:dyDescent="0.25"/>
     <row r="83" spans="6:7" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <dataConsolidate/>
   <mergeCells count="132">
     <mergeCell ref="B1:K1"/>
     <mergeCell ref="B3:K3"/>
@@ -3939,7 +3950,7 @@
       <formula>LEN(TRIM(K78))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations xWindow="828" yWindow="713" count="36">
+  <dataValidations xWindow="1033" yWindow="481" count="36">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indicar el nivel formativo en el cual se encuentra el aprendiz. Técnio o Tecnólogo" sqref="I10:M10" xr:uid="{FDFD4240-B4E4-40FA-8880-3E4E045C5084}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Número Ficha" prompt="Registre el número de ficha en el que se encuentra matriculado según el programa de formación." sqref="K11:M11" xr:uid="{C295E52F-E427-4103-89DB-18FF195E95C6}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Fin Etapa Lectiva" prompt="Registrar la fecha de culminación de la etapa lectiva del aprendiz." sqref="J13:M13" xr:uid="{5EB3E1EF-1E32-4E95-8D18-C01EA7CF4F61}"/>
@@ -3973,40 +3984,46 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Relacione las actividades que el aprendiz va a realizar según lo acordado. (Estas deben corresponder al perfil del egresado establecido en el programa de formación que el aprendiz está desarrollando.) redactar activ. en  verbos en infinitivo" sqref="C60:C64" xr:uid="{765A44AD-7EE4-4C8A-82B9-AEB337B3CBFF}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Describa las evidencias o entregables que se van a generar de acuerdo con las actividades a desarrollar. En este apartado adicionalmente, es importante definir si dichas evidencias serán entregadas de manera digital o física. " sqref="C65:M66" xr:uid="{6D49D6E6-6363-4D06-90B1-78A757068CEE}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Registre los comentarios que considere pertinentes en relación a la visita correspondiente. " sqref="C67:M71" xr:uid="{08D354B0-14A2-4554-94A3-2633D73D772A}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Nombre y Firma Aprendiz" prompt="Registrar el nombre completo del aprendiz y en la parte superior la Firma manuscrita o digital." sqref="A78:D78" xr:uid="{A7FEFB2B-7370-4FA2-8820-7EB89B730FD1}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Nombre y Firma Coformador" prompt="Registrar el nombre completo del co-formador y en la parte superior de esta la Firma manuscrita o digital." sqref="K78:M78" xr:uid="{DAE2A968-2309-42D5-952C-BC599D7BE50F}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="OBLIGATORIO NOMBRE Y FIRMA APREN" prompt="Registrar el nombre completo del aprendiz y en la parte superior la Firma manuscrita o digital." sqref="A78:D78" xr:uid="{A7FEFB2B-7370-4FA2-8820-7EB89B730FD1}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="OBLIGATORIO NOMBRE Y FIRMA JEFE" prompt="Registrar el nombre completo del co-formador y en la parte superior de esta la Firma manuscrita o digital." sqref="K78:M78" xr:uid="{DAE2A968-2309-42D5-952C-BC599D7BE50F}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Bogotá dd/mm/aaaa   virtual" prompt="Diligenciar fecha de la sesión en este espacio. Ejemplo: Bogotá dia/mes/año Virtual" sqref="C80:J80" xr:uid="{201095D8-80DA-45BB-84F9-D066E44DB3C5}"/>
   </dataValidations>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" scale="68" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xWindow="828" yWindow="713" count="7">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xWindow="1033" yWindow="481" count="7">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Seleccionael nombre del programa" prompt="Elige el programa de la lista desplegable" xr:uid="{34EF5BAD-650F-4FA7-AB25-B4A5694BB4C0}">
           <x14:formula1>
             <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$E$2)</xm:f>
           </x14:formula1>
           <xm:sqref>C11:H11</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Despliegue listado AQUI" prompt="Relacione el o los resultados de aprendizaje de las competencias que van a desarrollarse." xr:uid="{1DCCDD3C-B075-4833-878D-65AC808D9E9F}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Selecciona del listado las competencias tecnicas que se van a desarrollar a lo largo de la etapa productiva. minimo 3" xr:uid="{22B88745-2B8F-40B6-8916-320FA089DFCF}">
+          <x14:formula1>
+            <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$F$2)</xm:f>
+          </x14:formula1>
+          <xm:sqref>C50:M54</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Relacione el o los resultados de aprendizaje de las competencias que van a desarrollarse." xr:uid="{1DCCDD3C-B075-4833-878D-65AC808D9E9F}">
           <x14:formula1>
             <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$G$2)</xm:f>
           </x14:formula1>
           <xm:sqref>C55:M55</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Despliegue listado AQUI" prompt="Relacione el o los resultados de aprendizaje de las competencias que van a desarrollarse." xr:uid="{934278D6-6E18-4E97-BCEF-064F63567755}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Relacione el o los resultados de aprendizaje de las competencias que van a desarrollarse." xr:uid="{934278D6-6E18-4E97-BCEF-064F63567755}">
           <x14:formula1>
             <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$H$2)</xm:f>
           </x14:formula1>
           <xm:sqref>C56:M56</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Despliegue Listado AQUI" prompt="Relacione el o los resultados de aprendizaje de las competencias que van a desarrollarse." xr:uid="{0CE56376-096C-4566-B3AF-5321973F5724}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Relacione el o los resultados de aprendizaje de las competencias que van a desarrollarse." xr:uid="{0CE56376-096C-4566-B3AF-5321973F5724}">
           <x14:formula1>
             <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$I$2)</xm:f>
           </x14:formula1>
           <xm:sqref>C57:M57</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Despliegue Listado AQUI" prompt="Relacione el o los resultados de aprendizaje de las competencias que van a desarrollarse." xr:uid="{DD57E66E-4FD0-4B6F-8647-729A07AB846F}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Relacione el o los resultados de aprendizaje de las competencias que van a desarrollarse." xr:uid="{DD57E66E-4FD0-4B6F-8647-729A07AB846F}">
           <x14:formula1>
             <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$J$2)</xm:f>
           </x14:formula1>
@@ -4017,12 +4034,6 @@
             <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$K$2)</xm:f>
           </x14:formula1>
           <xm:sqref>C59:M59</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Despliegue la lista AQUI" prompt="Selecciona del listado las competencias tecnicas que se van a desarrollar a lo largo de la etapa productiva. minimo 3" xr:uid="{84F550D0-FC4B-4536-96E8-182B89C2F815}">
-          <x14:formula1>
-            <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$F$2)</xm:f>
-          </x14:formula1>
-          <xm:sqref>C50:M54</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4505,9 +4516,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>